<commit_message>
Add new platform to spreadsheet template example and tests
</commit_message>
<xml_diff>
--- a/eva_sub_cli/etc/EVA_Submission_template.xlsx
+++ b/eva_sub_cli/etc/EVA_Submission_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcezard/PycharmProjects/eva-sub-cli/eva_sub_cli/etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC871D1-7D13-104A-A2B6-89FCABA63623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A9AA12-83B5-5F4E-A99B-DAAE6E8CF182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,12 +35,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="556">
   <si>
     <t>PLEASE READ FIRST</t>
-  </si>
-  <si>
-    <t>V3.0.0 Sep 2025</t>
   </si>
   <si>
     <t>This Spreadsheet is meant to be used with the EVA submissions command line tools eva-sub-cli.</t>
@@ -1897,6 +1894,24 @@
   </si>
   <si>
     <t>Date to publicly release (if in the future). In the format: yyyy-mm-dd. The hold date should not be later than 2 years from now.</t>
+  </si>
+  <si>
+    <t>PacBio Revio</t>
+  </si>
+  <si>
+    <t>PacBio Sequel</t>
+  </si>
+  <si>
+    <t>PacBio Sequel IIe</t>
+  </si>
+  <si>
+    <t>PacBio Onso</t>
+  </si>
+  <si>
+    <t>PacBio Vega</t>
+  </si>
+  <si>
+    <t>V3.0.1 Jun 2026</t>
   </si>
 </sst>
 </file>
@@ -2341,7 +2356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2473,8 +2488,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2488,30 +2512,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2782,8 +2798,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1025" s="5" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="67"/>
-      <c r="B1" s="67"/>
+      <c r="A1" s="68"/>
+      <c r="B1" s="68"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -2792,10 +2808,10 @@
       <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:1025" s="5" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="68"/>
+      <c r="B2" s="71"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -2804,10 +2820,10 @@
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A3" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="69"/>
+      <c r="A3" s="72" t="s">
+        <v>555</v>
+      </c>
+      <c r="B3" s="72"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -2816,10 +2832,10 @@
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="70" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="70"/>
+      <c r="A4" s="73" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="73"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2828,10 +2844,10 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A5" s="71" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="71"/>
+      <c r="A5" s="74" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="74"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -2841,7 +2857,7 @@
     </row>
     <row r="6" spans="1:1025" s="5" customFormat="1" ht="80" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -2853,7 +2869,7 @@
     </row>
     <row r="7" spans="1:1025" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -3881,8 +3897,8 @@
       <c r="AMK7" s="5"/>
     </row>
     <row r="8" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="67"/>
-      <c r="B8" s="67"/>
+      <c r="A8" s="68"/>
+      <c r="B8" s="68"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -4908,10 +4924,10 @@
       <c r="AMK8" s="5"/>
     </row>
     <row r="9" spans="1:1025" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="73" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="73"/>
+      <c r="A9" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="69"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
@@ -5937,8 +5953,8 @@
       <c r="AMK9" s="5"/>
     </row>
     <row r="10" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="67"/>
-      <c r="B10" s="67"/>
+      <c r="A10" s="68"/>
+      <c r="B10" s="68"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -6964,65 +6980,65 @@
       <c r="AMK10" s="5"/>
     </row>
     <row r="11" spans="1:1025" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="74" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="74"/>
+      <c r="A11" s="70" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="70"/>
     </row>
     <row r="12" spans="1:1025" ht="20" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>8</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:1025" ht="20" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>10</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>11</v>
       </c>
       <c r="C13" s="14"/>
     </row>
     <row r="14" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
       <c r="A14" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>12</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
       <c r="A15" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>14</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:1025" ht="100" x14ac:dyDescent="0.2">
       <c r="A16" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>16</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:1025" ht="60" x14ac:dyDescent="0.2">
       <c r="A17" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="13" t="s">
+    </row>
+    <row r="19" spans="1:1025" s="5" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="67" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:1025" s="5" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="72" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="72"/>
+      <c r="B19" s="67"/>
       <c r="C19"/>
       <c r="D19"/>
       <c r="E19"/>
@@ -8048,22 +8064,22 @@
       <c r="AMK19"/>
     </row>
     <row r="20" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="72" t="s">
+      <c r="A20" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="67"/>
+    </row>
+    <row r="21" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="72"/>
-    </row>
-    <row r="21" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="72" t="s">
+      <c r="B21" s="67"/>
+    </row>
+    <row r="22" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="72"/>
-    </row>
-    <row r="22" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="72" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="72"/>
+      <c r="B22" s="67"/>
     </row>
     <row r="23" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="19"/>
@@ -9093,8 +9109,13 @@
       <c r="AMK23" s="5"/>
     </row>
   </sheetData>
-  <sheetProtection password="E50B" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="pKFT46AcXRrznfWpmO12FPPtk8Stkq83/gBYtpLA8HQFC7aZLAdf2WJU+dOj9PZT/L7JPEe68/xM25EHPxktXQ==" saltValue="g+GUymTOlW49z+xbPyQ28w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A22:B22"/>
@@ -9103,11 +9124,6 @@
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -9125,10 +9141,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -9171,1661 +9187,1678 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="64" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
       <c r="D1" s="64" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E1" s="40"/>
       <c r="F1" s="40"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B3" t="s">
         <v>198</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>199</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>200</v>
-      </c>
-      <c r="E3" t="s">
-        <v>201</v>
       </c>
       <c r="F3" s="65"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" t="s">
         <v>202</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>203</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>204</v>
-      </c>
-      <c r="E4" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B5" t="s">
         <v>206</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>207</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>208</v>
-      </c>
-      <c r="E5" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B6" t="s">
         <v>210</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>211</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>212</v>
-      </c>
-      <c r="E6" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" t="s">
         <v>214</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>215</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>216</v>
-      </c>
-      <c r="E7" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B8" t="s">
         <v>218</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
         <v>219</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>220</v>
-      </c>
-      <c r="E8" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>221</v>
+      </c>
+      <c r="B9" t="s">
         <v>222</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>223</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>224</v>
-      </c>
-      <c r="E9" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>225</v>
+      </c>
+      <c r="B10" t="s">
         <v>226</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
         <v>227</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>228</v>
-      </c>
-      <c r="E10" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" t="s">
         <v>230</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11" t="s">
         <v>231</v>
-      </c>
-      <c r="E11" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>232</v>
+      </c>
+      <c r="B12" t="s">
         <v>233</v>
       </c>
-      <c r="B12" t="s">
-        <v>234</v>
-      </c>
       <c r="E12" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
+        <v>234</v>
+      </c>
+      <c r="E13" t="s">
         <v>235</v>
-      </c>
-      <c r="E13" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
+        <v>236</v>
+      </c>
+      <c r="E14" t="s">
         <v>237</v>
-      </c>
-      <c r="E14" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
+        <v>238</v>
+      </c>
+      <c r="E15" t="s">
         <v>239</v>
-      </c>
-      <c r="E15" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
+        <v>240</v>
+      </c>
+      <c r="E16" t="s">
         <v>241</v>
-      </c>
-      <c r="E16" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
+        <v>242</v>
+      </c>
+      <c r="E17" t="s">
         <v>243</v>
-      </c>
-      <c r="E17" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
+        <v>244</v>
+      </c>
+      <c r="E18" t="s">
         <v>245</v>
-      </c>
-      <c r="E18" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
+        <v>246</v>
+      </c>
+      <c r="E19" t="s">
         <v>247</v>
-      </c>
-      <c r="E19" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
+        <v>248</v>
+      </c>
+      <c r="E20" t="s">
         <v>249</v>
-      </c>
-      <c r="E20" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
+        <v>250</v>
+      </c>
+      <c r="E21" t="s">
         <v>251</v>
-      </c>
-      <c r="E21" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
+        <v>252</v>
+      </c>
+      <c r="E22" t="s">
         <v>253</v>
-      </c>
-      <c r="E22" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
+        <v>254</v>
+      </c>
+      <c r="E23" t="s">
         <v>255</v>
-      </c>
-      <c r="E23" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
+        <v>256</v>
+      </c>
+      <c r="E24" t="s">
         <v>257</v>
-      </c>
-      <c r="E24" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
+        <v>258</v>
+      </c>
+      <c r="E25" t="s">
         <v>259</v>
-      </c>
-      <c r="E25" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
+        <v>260</v>
+      </c>
+      <c r="E26" t="s">
         <v>261</v>
-      </c>
-      <c r="E26" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
+        <v>262</v>
+      </c>
+      <c r="E27" t="s">
         <v>263</v>
-      </c>
-      <c r="E27" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
+        <v>264</v>
+      </c>
+      <c r="E28" t="s">
         <v>265</v>
-      </c>
-      <c r="E28" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
+        <v>266</v>
+      </c>
+      <c r="E29" t="s">
         <v>267</v>
-      </c>
-      <c r="E29" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
+        <v>268</v>
+      </c>
+      <c r="E30" t="s">
         <v>269</v>
-      </c>
-      <c r="E30" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
+        <v>270</v>
+      </c>
+      <c r="E31" t="s">
         <v>271</v>
-      </c>
-      <c r="E31" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
+        <v>272</v>
+      </c>
+      <c r="E32" t="s">
         <v>273</v>
-      </c>
-      <c r="E32" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
+        <v>274</v>
+      </c>
+      <c r="E33" t="s">
         <v>275</v>
-      </c>
-      <c r="E33" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E34" t="s">
         <v>277</v>
-      </c>
-      <c r="E34" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
+        <v>278</v>
+      </c>
+      <c r="E35" t="s">
         <v>279</v>
-      </c>
-      <c r="E35" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
+        <v>280</v>
+      </c>
+      <c r="E36" t="s">
         <v>281</v>
-      </c>
-      <c r="E36" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
+        <v>282</v>
+      </c>
+      <c r="E37" t="s">
         <v>283</v>
-      </c>
-      <c r="E37" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
+        <v>284</v>
+      </c>
+      <c r="E38" t="s">
         <v>285</v>
-      </c>
-      <c r="E38" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
+        <v>286</v>
+      </c>
+      <c r="E39" t="s">
         <v>287</v>
-      </c>
-      <c r="E39" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
+        <v>288</v>
+      </c>
+      <c r="E40" t="s">
         <v>289</v>
-      </c>
-      <c r="E40" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
+        <v>290</v>
+      </c>
+      <c r="E41" t="s">
         <v>291</v>
-      </c>
-      <c r="E41" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
+        <v>292</v>
+      </c>
+      <c r="E42" t="s">
         <v>293</v>
-      </c>
-      <c r="E42" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
+        <v>294</v>
+      </c>
+      <c r="E43" t="s">
         <v>295</v>
-      </c>
-      <c r="E43" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
+        <v>296</v>
+      </c>
+      <c r="E44" t="s">
         <v>297</v>
-      </c>
-      <c r="E44" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
+        <v>298</v>
+      </c>
+      <c r="E45" t="s">
         <v>299</v>
-      </c>
-      <c r="E45" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
+        <v>300</v>
+      </c>
+      <c r="E46" t="s">
         <v>301</v>
-      </c>
-      <c r="E46" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
+        <v>302</v>
+      </c>
+      <c r="E47" t="s">
         <v>303</v>
-      </c>
-      <c r="E47" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
+        <v>304</v>
+      </c>
+      <c r="E48" t="s">
         <v>305</v>
-      </c>
-      <c r="E48" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
+        <v>306</v>
+      </c>
+      <c r="E49" t="s">
         <v>307</v>
-      </c>
-      <c r="E49" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
+        <v>308</v>
+      </c>
+      <c r="E50" t="s">
         <v>309</v>
-      </c>
-      <c r="E50" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
+        <v>310</v>
+      </c>
+      <c r="E51" t="s">
         <v>311</v>
-      </c>
-      <c r="E51" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
+        <v>312</v>
+      </c>
+      <c r="E52" t="s">
         <v>313</v>
-      </c>
-      <c r="E52" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E53" t="s">
-        <v>316</v>
+        <v>553</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
-        <v>317</v>
+        <v>316</v>
+      </c>
+      <c r="E54" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
-        <v>318</v>
-      </c>
-      <c r="E55" s="40"/>
+        <v>317</v>
+      </c>
+      <c r="E55" s="80" t="s">
+        <v>551</v>
+      </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
-        <v>319</v>
+        <v>318</v>
+      </c>
+      <c r="E56" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
-        <v>320</v>
+        <v>319</v>
+      </c>
+      <c r="E57" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
-        <v>321</v>
+        <v>320</v>
+      </c>
+      <c r="E58" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B60" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B61" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B65" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B66" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="73" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B74" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B83" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="84" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B85" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B86" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B87" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B88" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B89" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="90" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B91" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B92" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B93" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="95" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B95" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B96" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B97" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B98" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B99" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B101" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B102" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="103" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B103" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B104" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B105" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="106" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B107" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="109" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="114" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B115" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B116" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="117" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="118" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="119" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="120" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B120" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B121" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="122" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B122" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="123" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="124" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="125" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="126" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B126" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="127" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B127" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="128" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B128" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="129" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="130" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="131" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="132" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="133" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B133" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="134" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B134" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="135" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="136" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="137" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="138" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B138" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="139" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="140" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B140" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="141" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="142" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="143" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="144" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B144" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="145" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B145" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="146" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B146" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="147" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B147" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="148" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B148" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="149" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B149" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="150" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B150" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="151" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B151" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="152" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B152" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="153" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B153" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="154" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B154" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="155" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B155" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="156" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B156" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="157" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B157" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="158" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B158" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="159" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B159" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="160" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B160" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="161" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B161" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="162" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B162" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="163" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B163" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="164" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B164" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="165" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B165" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="166" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B166" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="167" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B167" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="168" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B168" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="169" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B169" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="170" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B170" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="171" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B171" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="172" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B172" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="173" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B173" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="174" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B174" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="175" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B175" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="176" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B176" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="177" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B177" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="178" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B178" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="179" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B179" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="180" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B180" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="181" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B181" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="182" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B182" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="183" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B183" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="184" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B184" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="185" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B185" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="186" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B186" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="187" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B187" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="188" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B188" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="189" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B189" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="190" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B190" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="191" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B191" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="192" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B192" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="193" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B193" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="194" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B194" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="195" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B195" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="196" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B196" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="197" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B197" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="198" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B198" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="199" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B199" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="200" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B200" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="201" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B201" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="202" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B202" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="203" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B203" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="204" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B204" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="205" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B205" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="206" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B206" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="207" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B207" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="208" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B208" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="209" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B209" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="210" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B210" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="211" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B211" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="212" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B212" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="213" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B213" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="214" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B214" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="215" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B215" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="216" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B216" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="217" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B217" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="218" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B218" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="219" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B219" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="220" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B220" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="221" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B221" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="222" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B222" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="223" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B223" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="224" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B224" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="225" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B225" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="226" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B226" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="227" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B227" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="228" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B228" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="229" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B229" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="230" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B230" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="231" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B231" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="232" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B232" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="233" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B233" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="234" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B234" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="235" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B235" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="236" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B236" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="237" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B237" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="238" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B238" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="239" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B239" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="240" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B240" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="241" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B241" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="242" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B242" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="243" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B243" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="244" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B244" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="245" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B245" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="246" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B246" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="247" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B247" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="248" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B248" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="249" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B249" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="250" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B250" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="251" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B251" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="252" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B252" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="253" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B253" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="254" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B254" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="255" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B255" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="256" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B256" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="257" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B257" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="258" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B258" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="259" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B259" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="260" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B260" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="261" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B261" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="262" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B262" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="263" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B263" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="264" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B264" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
     </row>
     <row r="265" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B265" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="266" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B266" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="267" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B267" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="268" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B268" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="269" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B269" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="270" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B270" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="271" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B271" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="272" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B272" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
     </row>
     <row r="273" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B273" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="274" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B274" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="275" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B275" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="276" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B276" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="277" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B277" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="278" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B278" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="279" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B279" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="280" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B280" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="281" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B281" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="282" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B282" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="283" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B283" s="66" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="284" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B284" s="66" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="285" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B285" s="66" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
     </row>
     <row r="286" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B286" s="66" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="E50B" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="qp9rDPdjyVfO19PBWKfIfNZhhynpJZQsyvoWiYXbAJIAOmwCNMnLHqyBUqiXFFXNIXX8MGCI7qELdKTMmJUw4g==" saltValue="ylQiF++NX2Rl274PyCnWGg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E3:E58">
+    <sortCondition ref="E58"/>
+  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -10846,22 +10879,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="C1" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="E1" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="F1" s="22" t="s">
         <v>28</v>
-      </c>
-      <c r="F1" s="22" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -10881,129 +10914,129 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
         <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
         <v>37</v>
-      </c>
-      <c r="B6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
         <v>39</v>
-      </c>
-      <c r="B7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" t="s">
         <v>42</v>
-      </c>
-      <c r="B9" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
         <v>44</v>
-      </c>
-      <c r="B10" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
         <v>46</v>
-      </c>
-      <c r="B11" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="s">
         <v>48</v>
-      </c>
-      <c r="B12" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" t="s">
         <v>50</v>
-      </c>
-      <c r="B13" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
         <v>52</v>
-      </c>
-      <c r="B14" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s">
         <v>55</v>
-      </c>
-      <c r="B16" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="28" t="s">
         <v>57</v>
-      </c>
-      <c r="B17" s="28" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -11036,13 +11069,13 @@
   <sheetData>
     <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="75" t="s">
+      <c r="C1" s="30" t="s">
         <v>60</v>
-      </c>
-      <c r="C1" s="30" t="s">
-        <v>61</v>
       </c>
       <c r="D1" s="26"/>
       <c r="E1" s="26"/>
@@ -11053,7 +11086,7 @@
       <c r="A2" s="20"/>
       <c r="B2" s="75"/>
       <c r="C2" s="76" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="76"/>
       <c r="E2" s="76"/>
@@ -11069,44 +11102,44 @@
     </row>
     <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B3" s="75"/>
       <c r="C3" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H3" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L3" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="M3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="M3" s="22" t="s">
-        <v>55</v>
-      </c>
       <c r="N3" s="32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="16" x14ac:dyDescent="0.2"/>
@@ -11153,130 +11186,130 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
         <v>63</v>
-      </c>
-      <c r="B2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
         <v>65</v>
-      </c>
-      <c r="B3" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="26" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" t="s">
         <v>68</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" t="s">
         <v>70</v>
-      </c>
-      <c r="B6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" t="s">
         <v>72</v>
-      </c>
-      <c r="B7" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" t="s">
         <v>74</v>
-      </c>
-      <c r="B8" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" t="s">
         <v>76</v>
-      </c>
-      <c r="B9" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
         <v>78</v>
-      </c>
-      <c r="B10" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
         <v>80</v>
-      </c>
-      <c r="B11" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" t="s">
         <v>82</v>
-      </c>
-      <c r="B12" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" t="s">
         <v>84</v>
-      </c>
-      <c r="B13" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" t="s">
         <v>86</v>
-      </c>
-      <c r="B14" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" t="s">
         <v>89</v>
-      </c>
-      <c r="B16" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
@@ -11317,49 +11350,49 @@
   <sheetData>
     <row r="1" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H1" s="22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I1" s="22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K1" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L1" s="22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M1" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N1" s="22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O1" s="22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="16" x14ac:dyDescent="0.2">
@@ -11406,12 +11439,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" promptTitle="Platform" prompt="Please select from the available list of platforms._x000a_If your platform is not present, please enter it as a new entry and confirm warning message" xr:uid="{86898878-0656-0643-9D11-EC1AE19D11CB}">
-          <x14:formula1>
-            <xm:f>CVs!$E$3:$E$53</xm:f>
-          </x14:formula1>
-          <xm:sqref>G4:G1048576 G2</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Experiment type" prompt="Please select experiment type." xr:uid="{00000000-0002-0000-0500-000008000000}">
           <x14:formula1>
             <xm:f>CVs!$D$3:$D$10</xm:f>
@@ -11420,6 +11447,12 @@
             <xm:f>0</xm:f>
           </x14:formula2>
           <xm:sqref>D2:D1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" promptTitle="Platform" prompt="Please select from the available list of platforms._x000a_If your platform is not present, please enter it as a new entry and confirm warning message" xr:uid="{0A7314A8-3530-0D44-85F0-476834B4FE43}">
+          <x14:formula1>
+            <xm:f>CVs!$E$3:$E$58</xm:f>
+          </x14:formula1>
+          <xm:sqref>G2:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -11438,447 +11471,447 @@
   <sheetData>
     <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="36" t="s">
         <v>94</v>
-      </c>
-      <c r="B5" s="36" t="s">
-        <v>95</v>
       </c>
       <c r="C5" s="37"/>
     </row>
     <row r="6" spans="1:3" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="24" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="36" t="s">
         <v>98</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="36" t="s">
         <v>102</v>
-      </c>
-      <c r="B11" s="36" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" s="36" t="s">
         <v>104</v>
-      </c>
-      <c r="B12" s="36" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B13" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" s="36" t="s">
         <v>107</v>
-      </c>
-      <c r="B14" s="36" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="36" t="s">
         <v>109</v>
-      </c>
-      <c r="B15" s="36" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="36" t="s">
         <v>111</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="40" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B17" s="36"/>
     </row>
     <row r="18" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B18" s="41" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="36" t="s">
         <v>115</v>
-      </c>
-      <c r="B19" s="36" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="36" t="s">
         <v>117</v>
-      </c>
-      <c r="B20" s="36" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="40" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B21" s="36"/>
     </row>
     <row r="22" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" s="36" t="s">
         <v>120</v>
-      </c>
-      <c r="B22" s="36" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23" s="36" t="s">
         <v>122</v>
-      </c>
-      <c r="B23" s="36" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24" s="36" t="s">
         <v>124</v>
-      </c>
-      <c r="B24" s="36" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="40" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B25" s="36"/>
     </row>
     <row r="26" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>126</v>
+      </c>
+      <c r="B26" s="36" t="s">
         <v>127</v>
-      </c>
-      <c r="B26" s="36" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="36" t="s">
         <v>129</v>
-      </c>
-      <c r="B27" s="36" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" s="36" t="s">
         <v>131</v>
-      </c>
-      <c r="B28" s="36" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>132</v>
+      </c>
+      <c r="B29" s="36" t="s">
         <v>133</v>
-      </c>
-      <c r="B29" s="36" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>134</v>
+      </c>
+      <c r="B30" s="36" t="s">
         <v>135</v>
-      </c>
-      <c r="B30" s="36" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="40" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B31" s="36"/>
     </row>
     <row r="32" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>137</v>
+      </c>
+      <c r="B32" s="36" t="s">
         <v>138</v>
-      </c>
-      <c r="B32" s="36" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>139</v>
+      </c>
+      <c r="B33" s="36" t="s">
         <v>140</v>
-      </c>
-      <c r="B33" s="36" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>141</v>
+      </c>
+      <c r="B34" s="36" t="s">
         <v>142</v>
-      </c>
-      <c r="B34" s="36" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="40" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B35" s="36"/>
     </row>
     <row r="36" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>144</v>
+      </c>
+      <c r="B36" s="36" t="s">
         <v>145</v>
-      </c>
-      <c r="B36" s="36" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="B37" s="36" t="s">
         <v>147</v>
-      </c>
-      <c r="B37" s="36" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="36" t="s">
         <v>149</v>
-      </c>
-      <c r="B38" s="36" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>150</v>
+      </c>
+      <c r="B39" s="36" t="s">
         <v>151</v>
-      </c>
-      <c r="B39" s="36" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" s="36" t="s">
         <v>153</v>
-      </c>
-      <c r="B40" s="36" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
+        <v>154</v>
+      </c>
+      <c r="B41" s="36" t="s">
         <v>155</v>
-      </c>
-      <c r="B41" s="36" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>156</v>
+      </c>
+      <c r="B42" s="36" t="s">
         <v>157</v>
-      </c>
-      <c r="B42" s="36" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
+        <v>158</v>
+      </c>
+      <c r="B43" s="36" t="s">
         <v>159</v>
-      </c>
-      <c r="B43" s="36" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
+        <v>160</v>
+      </c>
+      <c r="B44" s="36" t="s">
         <v>161</v>
-      </c>
-      <c r="B44" s="36" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="51" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
+        <v>162</v>
+      </c>
+      <c r="B45" s="41" t="s">
         <v>163</v>
-      </c>
-      <c r="B45" s="41" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="40" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B46" s="36"/>
     </row>
     <row r="47" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
+        <v>165</v>
+      </c>
+      <c r="B47" s="36" t="s">
         <v>166</v>
-      </c>
-      <c r="B47" s="36" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>167</v>
+      </c>
+      <c r="B48" s="36" t="s">
         <v>168</v>
-      </c>
-      <c r="B48" s="36" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
+        <v>169</v>
+      </c>
+      <c r="B49" s="36" t="s">
         <v>170</v>
-      </c>
-      <c r="B49" s="36" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
+        <v>171</v>
+      </c>
+      <c r="B50" s="36" t="s">
         <v>172</v>
-      </c>
-      <c r="B50" s="36" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
+        <v>173</v>
+      </c>
+      <c r="B51" s="36" t="s">
         <v>174</v>
-      </c>
-      <c r="B51" s="36" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>175</v>
+      </c>
+      <c r="B52" s="36" t="s">
         <v>176</v>
-      </c>
-      <c r="B52" s="36" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
+        <v>177</v>
+      </c>
+      <c r="B53" s="36" t="s">
         <v>178</v>
-      </c>
-      <c r="B53" s="36" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
+        <v>179</v>
+      </c>
+      <c r="B54" s="36" t="s">
         <v>180</v>
-      </c>
-      <c r="B54" s="36" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
+        <v>181</v>
+      </c>
+      <c r="B55" s="36" t="s">
         <v>182</v>
-      </c>
-      <c r="B55" s="36" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
+        <v>183</v>
+      </c>
+      <c r="B56" s="36" t="s">
         <v>184</v>
-      </c>
-      <c r="B56" s="36" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B57" s="36"/>
     </row>
     <row r="58" spans="1:2" ht="24" x14ac:dyDescent="0.2">
       <c r="A58" s="34" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B58" s="36"/>
     </row>
     <row r="59" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="42" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B59" s="36"/>
     </row>
     <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
+        <v>188</v>
+      </c>
+      <c r="B60" s="36" t="s">
         <v>189</v>
-      </c>
-      <c r="B60" s="36" t="s">
-        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -11917,19 +11950,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A1" s="77" t="s">
-        <v>191</v>
-      </c>
-      <c r="B1" s="77"/>
+      <c r="A1" s="79" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="79"/>
       <c r="C1" s="75"/>
       <c r="D1" s="43" t="s">
+        <v>191</v>
+      </c>
+      <c r="E1" s="75" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="43" t="s">
         <v>192</v>
-      </c>
-      <c r="E1" s="75" t="s">
-        <v>60</v>
-      </c>
-      <c r="F1" s="43" t="s">
-        <v>193</v>
       </c>
       <c r="G1" s="44"/>
       <c r="H1" s="45"/>
@@ -11979,37 +12012,37 @@
       <c r="D2" s="51"/>
       <c r="E2" s="75"/>
       <c r="F2" s="78" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G2" s="78"/>
       <c r="H2" s="78"/>
       <c r="I2" s="78"/>
       <c r="J2" s="78"/>
       <c r="K2" s="78"/>
-      <c r="L2" s="79" t="s">
-        <v>113</v>
-      </c>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="79" t="s">
-        <v>119</v>
-      </c>
-      <c r="P2" s="79"/>
-      <c r="Q2" s="79"/>
+      <c r="L2" s="77" t="s">
+        <v>112</v>
+      </c>
+      <c r="M2" s="77"/>
+      <c r="N2" s="77"/>
+      <c r="O2" s="77" t="s">
+        <v>118</v>
+      </c>
+      <c r="P2" s="77"/>
+      <c r="Q2" s="77"/>
       <c r="R2" s="78" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="S2" s="78"/>
       <c r="T2" s="78"/>
       <c r="U2" s="78"/>
       <c r="V2" s="78"/>
       <c r="W2" s="78" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="X2" s="78"/>
       <c r="Y2" s="78"/>
       <c r="Z2" s="78" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AA2" s="78"/>
       <c r="AB2" s="78"/>
@@ -12021,7 +12054,7 @@
       <c r="AH2" s="78"/>
       <c r="AI2" s="78"/>
       <c r="AJ2" s="78" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AK2" s="78"/>
       <c r="AL2" s="78"/>
@@ -12035,138 +12068,138 @@
     </row>
     <row r="3" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A3" s="52" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C3" s="75"/>
       <c r="D3" s="54" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E3" s="75"/>
       <c r="F3" s="54" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G3" s="55" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H3" s="56" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I3" s="56" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J3" s="56" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K3" s="57" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L3" s="55" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M3" s="55" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="N3" s="57" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O3" s="56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P3" s="58" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q3" s="56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="R3" s="59" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="S3" s="56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="T3" s="56" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="U3" s="56" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="V3" s="57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="W3" s="59" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="X3" s="56" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Y3" s="57" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Z3" s="59" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AA3" s="60" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AB3" s="55" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AC3" s="56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AD3" s="56" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AE3" s="56" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AF3" s="56" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AG3" s="56" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AH3" s="56" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AI3" s="57" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AJ3" s="59" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AK3" s="56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AL3" s="56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AM3" s="56" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AN3" s="56" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AO3" s="56" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AP3" s="56" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AQ3" s="56" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AR3" s="56" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AS3" s="57" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AT3" s="61" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:46" x14ac:dyDescent="0.2">
@@ -12187,16 +12220,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="F2:K2"/>
+    <mergeCell ref="L2:N2"/>
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="R2:V2"/>
     <mergeCell ref="W2:Y2"/>
     <mergeCell ref="Z2:AI2"/>
     <mergeCell ref="AJ2:AS2"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="E1:E3"/>
-    <mergeCell ref="F2:K2"/>
-    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Metadata and VCF" prompt="These sample names must match those provided in the VCF file(s)" sqref="E1 B4:B1003" xr:uid="{00000000-0002-0000-0700-000000000000}">
@@ -12273,26 +12306,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" t="s">
         <v>195</v>
-      </c>
-      <c r="B3" t="s">
-        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add checkbox for data acknowledgement statements
</commit_message>
<xml_diff>
--- a/eva_sub_cli/etc/EVA_Submission_template.xlsx
+++ b/eva_sub_cli/etc/EVA_Submission_template.xlsx
@@ -1,31 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcezard/PycharmProjects/eva-sub-cli/eva_sub_cli/etc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkumar2/PycharmProjects/eva-sub-cli/eva_sub_cli/etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A9AA12-83B5-5F4E-A99B-DAAE6E8CF182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC01D75B-FA50-A942-89D0-656265DF7489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLEASE READ FIRST" sheetId="1" r:id="rId1"/>
     <sheet name="Submitter Details" sheetId="2" r:id="rId2"/>
-    <sheet name="Project HELP" sheetId="3" r:id="rId3"/>
-    <sheet name="Project" sheetId="4" r:id="rId4"/>
-    <sheet name="Analysis HELP" sheetId="5" r:id="rId5"/>
-    <sheet name="Analysis" sheetId="6" r:id="rId6"/>
-    <sheet name="Sample HELP" sheetId="7" r:id="rId7"/>
-    <sheet name="Sample" sheetId="8" r:id="rId8"/>
-    <sheet name="Files HELP" sheetId="9" r:id="rId9"/>
-    <sheet name="Files" sheetId="10" r:id="rId10"/>
-    <sheet name="CVs" sheetId="11" r:id="rId11"/>
+    <sheet name="Data Acknowledgement" sheetId="13" r:id="rId3"/>
+    <sheet name="Project HELP" sheetId="3" r:id="rId4"/>
+    <sheet name="Project" sheetId="4" r:id="rId5"/>
+    <sheet name="Analysis HELP" sheetId="5" r:id="rId6"/>
+    <sheet name="Analysis" sheetId="6" r:id="rId7"/>
+    <sheet name="Sample HELP" sheetId="7" r:id="rId8"/>
+    <sheet name="Sample" sheetId="8" r:id="rId9"/>
+    <sheet name="Files HELP" sheetId="9" r:id="rId10"/>
+    <sheet name="Files" sheetId="10" r:id="rId11"/>
+    <sheet name="CVs" sheetId="11" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="561">
   <si>
     <t>PLEASE READ FIRST</t>
   </si>
@@ -1911,7 +1912,22 @@
     <t>PacBio Vega</t>
   </si>
   <si>
-    <t>V3.0.1 Jun 2026</t>
+    <t>Submitters must confirm they have the right to openly share the submitted data and that the submission complies with applicable access and benefit-sharing obligations. See the "Data Access Acknowledgement" worksheet for the full statement.</t>
+  </si>
+  <si>
+    <t>To the best of my knowledge, the data being submitted are not subject to any restrictions that prohibit their open sharing and are submitted in compliance with applicable national and international access and benefit-sharing obligations, in accordance with the EMBL-EBI Terms of Use (https://www.ebi.ac.uk/about/terms-of-use/).</t>
+  </si>
+  <si>
+    <t>Statement</t>
+  </si>
+  <si>
+    <t>Acknowledgement</t>
+  </si>
+  <si>
+    <t>Data Acknowledgement</t>
+  </si>
+  <si>
+    <t>V3.1.0 Sep 2026</t>
   </si>
 </sst>
 </file>
@@ -1921,7 +1937,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -2132,6 +2148,27 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="36"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -2356,7 +2393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2489,16 +2526,33 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2512,22 +2566,30 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2611,6 +2673,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2789,7 +2868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMK23"/>
+  <dimension ref="A1:AMK24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="61.6640625" customWidth="1"/>
@@ -2798,8 +2877,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1025" s="5" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="68"/>
-      <c r="B1" s="68"/>
+      <c r="A1" s="73"/>
+      <c r="B1" s="73"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -2808,10 +2887,10 @@
       <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:1025" s="5" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="71"/>
+      <c r="B2" s="74"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -2820,10 +2899,10 @@
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A3" s="72" t="s">
-        <v>555</v>
-      </c>
-      <c r="B3" s="72"/>
+      <c r="A3" s="75" t="s">
+        <v>560</v>
+      </c>
+      <c r="B3" s="75"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -2832,10 +2911,10 @@
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="73"/>
+      <c r="B4" s="76"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2844,10 +2923,10 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="74"/>
+      <c r="B5" s="77"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -3897,8 +3976,8 @@
       <c r="AMK7" s="5"/>
     </row>
     <row r="8" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="68"/>
-      <c r="B8" s="68"/>
+      <c r="A8" s="73"/>
+      <c r="B8" s="73"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -4924,10 +5003,10 @@
       <c r="AMK8" s="5"/>
     </row>
     <row r="9" spans="1:1025" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="69" t="s">
+      <c r="A9" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="69"/>
+      <c r="B9" s="79"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
@@ -5953,8 +6032,8 @@
       <c r="AMK9" s="5"/>
     </row>
     <row r="10" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="68"/>
-      <c r="B10" s="68"/>
+      <c r="A10" s="73"/>
+      <c r="B10" s="73"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -6980,10 +7059,10 @@
       <c r="AMK10" s="5"/>
     </row>
     <row r="11" spans="1:1025" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="70" t="s">
+      <c r="A11" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="70"/>
+      <c r="B11" s="80"/>
     </row>
     <row r="12" spans="1:1025" ht="20" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
@@ -7002,2128 +7081,2136 @@
       </c>
       <c r="C13" s="14"/>
     </row>
-    <row r="14" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:1025" ht="60" x14ac:dyDescent="0.2">
+      <c r="A14" s="16" t="s">
+        <v>559</v>
+      </c>
+      <c r="B14" s="67" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
+      <c r="A15" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B15" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
-      <c r="A15" s="16" t="s">
+    <row r="16" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B16" s="13" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:1025" ht="100" x14ac:dyDescent="0.2">
-      <c r="A16" s="17" t="s">
+    <row r="17" spans="1:1025" ht="100" x14ac:dyDescent="0.2">
+      <c r="A17" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B17" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:1025" ht="60" x14ac:dyDescent="0.2">
-      <c r="A17" s="18" t="s">
+    <row r="18" spans="1:1025" ht="60" x14ac:dyDescent="0.2">
+      <c r="A18" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B18" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:1025" s="5" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="67" t="s">
+    <row r="20" spans="1:1025" s="5" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="67"/>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-      <c r="G19"/>
-      <c r="H19"/>
-      <c r="I19"/>
-      <c r="J19"/>
-      <c r="K19"/>
-      <c r="L19"/>
-      <c r="M19"/>
-      <c r="N19"/>
-      <c r="O19"/>
-      <c r="P19"/>
-      <c r="Q19"/>
-      <c r="R19"/>
-      <c r="S19"/>
-      <c r="T19"/>
-      <c r="U19"/>
-      <c r="V19"/>
-      <c r="W19"/>
-      <c r="X19"/>
-      <c r="Y19"/>
-      <c r="Z19"/>
-      <c r="AA19"/>
-      <c r="AB19"/>
-      <c r="AC19"/>
-      <c r="AD19"/>
-      <c r="AE19"/>
-      <c r="AF19"/>
-      <c r="AG19"/>
-      <c r="AH19"/>
-      <c r="AI19"/>
-      <c r="AJ19"/>
-      <c r="AK19"/>
-      <c r="AL19"/>
-      <c r="AM19"/>
-      <c r="AN19"/>
-      <c r="AO19"/>
-      <c r="AP19"/>
-      <c r="AQ19"/>
-      <c r="AR19"/>
-      <c r="AS19"/>
-      <c r="AT19"/>
-      <c r="AU19"/>
-      <c r="AV19"/>
-      <c r="AW19"/>
-      <c r="AX19"/>
-      <c r="AY19"/>
-      <c r="AZ19"/>
-      <c r="BA19"/>
-      <c r="BB19"/>
-      <c r="BC19"/>
-      <c r="BD19"/>
-      <c r="BE19"/>
-      <c r="BF19"/>
-      <c r="BG19"/>
-      <c r="BH19"/>
-      <c r="BI19"/>
-      <c r="BJ19"/>
-      <c r="BK19"/>
-      <c r="BL19"/>
-      <c r="BM19"/>
-      <c r="BN19"/>
-      <c r="BO19"/>
-      <c r="BP19"/>
-      <c r="BQ19"/>
-      <c r="BR19"/>
-      <c r="BS19"/>
-      <c r="BT19"/>
-      <c r="BU19"/>
-      <c r="BV19"/>
-      <c r="BW19"/>
-      <c r="BX19"/>
-      <c r="BY19"/>
-      <c r="BZ19"/>
-      <c r="CA19"/>
-      <c r="CB19"/>
-      <c r="CC19"/>
-      <c r="CD19"/>
-      <c r="CE19"/>
-      <c r="CF19"/>
-      <c r="CG19"/>
-      <c r="CH19"/>
-      <c r="CI19"/>
-      <c r="CJ19"/>
-      <c r="CK19"/>
-      <c r="CL19"/>
-      <c r="CM19"/>
-      <c r="CN19"/>
-      <c r="CO19"/>
-      <c r="CP19"/>
-      <c r="CQ19"/>
-      <c r="CR19"/>
-      <c r="CS19"/>
-      <c r="CT19"/>
-      <c r="CU19"/>
-      <c r="CV19"/>
-      <c r="CW19"/>
-      <c r="CX19"/>
-      <c r="CY19"/>
-      <c r="CZ19"/>
-      <c r="DA19"/>
-      <c r="DB19"/>
-      <c r="DC19"/>
-      <c r="DD19"/>
-      <c r="DE19"/>
-      <c r="DF19"/>
-      <c r="DG19"/>
-      <c r="DH19"/>
-      <c r="DI19"/>
-      <c r="DJ19"/>
-      <c r="DK19"/>
-      <c r="DL19"/>
-      <c r="DM19"/>
-      <c r="DN19"/>
-      <c r="DO19"/>
-      <c r="DP19"/>
-      <c r="DQ19"/>
-      <c r="DR19"/>
-      <c r="DS19"/>
-      <c r="DT19"/>
-      <c r="DU19"/>
-      <c r="DV19"/>
-      <c r="DW19"/>
-      <c r="DX19"/>
-      <c r="DY19"/>
-      <c r="DZ19"/>
-      <c r="EA19"/>
-      <c r="EB19"/>
-      <c r="EC19"/>
-      <c r="ED19"/>
-      <c r="EE19"/>
-      <c r="EF19"/>
-      <c r="EG19"/>
-      <c r="EH19"/>
-      <c r="EI19"/>
-      <c r="EJ19"/>
-      <c r="EK19"/>
-      <c r="EL19"/>
-      <c r="EM19"/>
-      <c r="EN19"/>
-      <c r="EO19"/>
-      <c r="EP19"/>
-      <c r="EQ19"/>
-      <c r="ER19"/>
-      <c r="ES19"/>
-      <c r="ET19"/>
-      <c r="EU19"/>
-      <c r="EV19"/>
-      <c r="EW19"/>
-      <c r="EX19"/>
-      <c r="EY19"/>
-      <c r="EZ19"/>
-      <c r="FA19"/>
-      <c r="FB19"/>
-      <c r="FC19"/>
-      <c r="FD19"/>
-      <c r="FE19"/>
-      <c r="FF19"/>
-      <c r="FG19"/>
-      <c r="FH19"/>
-      <c r="FI19"/>
-      <c r="FJ19"/>
-      <c r="FK19"/>
-      <c r="FL19"/>
-      <c r="FM19"/>
-      <c r="FN19"/>
-      <c r="FO19"/>
-      <c r="FP19"/>
-      <c r="FQ19"/>
-      <c r="FR19"/>
-      <c r="FS19"/>
-      <c r="FT19"/>
-      <c r="FU19"/>
-      <c r="FV19"/>
-      <c r="FW19"/>
-      <c r="FX19"/>
-      <c r="FY19"/>
-      <c r="FZ19"/>
-      <c r="GA19"/>
-      <c r="GB19"/>
-      <c r="GC19"/>
-      <c r="GD19"/>
-      <c r="GE19"/>
-      <c r="GF19"/>
-      <c r="GG19"/>
-      <c r="GH19"/>
-      <c r="GI19"/>
-      <c r="GJ19"/>
-      <c r="GK19"/>
-      <c r="GL19"/>
-      <c r="GM19"/>
-      <c r="GN19"/>
-      <c r="GO19"/>
-      <c r="GP19"/>
-      <c r="GQ19"/>
-      <c r="GR19"/>
-      <c r="GS19"/>
-      <c r="GT19"/>
-      <c r="GU19"/>
-      <c r="GV19"/>
-      <c r="GW19"/>
-      <c r="GX19"/>
-      <c r="GY19"/>
-      <c r="GZ19"/>
-      <c r="HA19"/>
-      <c r="HB19"/>
-      <c r="HC19"/>
-      <c r="HD19"/>
-      <c r="HE19"/>
-      <c r="HF19"/>
-      <c r="HG19"/>
-      <c r="HH19"/>
-      <c r="HI19"/>
-      <c r="HJ19"/>
-      <c r="HK19"/>
-      <c r="HL19"/>
-      <c r="HM19"/>
-      <c r="HN19"/>
-      <c r="HO19"/>
-      <c r="HP19"/>
-      <c r="HQ19"/>
-      <c r="HR19"/>
-      <c r="HS19"/>
-      <c r="HT19"/>
-      <c r="HU19"/>
-      <c r="HV19"/>
-      <c r="HW19"/>
-      <c r="HX19"/>
-      <c r="HY19"/>
-      <c r="HZ19"/>
-      <c r="IA19"/>
-      <c r="IB19"/>
-      <c r="IC19"/>
-      <c r="ID19"/>
-      <c r="IE19"/>
-      <c r="IF19"/>
-      <c r="IG19"/>
-      <c r="IH19"/>
-      <c r="II19"/>
-      <c r="IJ19"/>
-      <c r="IK19"/>
-      <c r="IL19"/>
-      <c r="IM19"/>
-      <c r="IN19"/>
-      <c r="IO19"/>
-      <c r="IP19"/>
-      <c r="IQ19"/>
-      <c r="IR19"/>
-      <c r="IS19"/>
-      <c r="IT19"/>
-      <c r="IU19"/>
-      <c r="IV19"/>
-      <c r="IW19"/>
-      <c r="IX19"/>
-      <c r="IY19"/>
-      <c r="IZ19"/>
-      <c r="JA19"/>
-      <c r="JB19"/>
-      <c r="JC19"/>
-      <c r="JD19"/>
-      <c r="JE19"/>
-      <c r="JF19"/>
-      <c r="JG19"/>
-      <c r="JH19"/>
-      <c r="JI19"/>
-      <c r="JJ19"/>
-      <c r="JK19"/>
-      <c r="JL19"/>
-      <c r="JM19"/>
-      <c r="JN19"/>
-      <c r="JO19"/>
-      <c r="JP19"/>
-      <c r="JQ19"/>
-      <c r="JR19"/>
-      <c r="JS19"/>
-      <c r="JT19"/>
-      <c r="JU19"/>
-      <c r="JV19"/>
-      <c r="JW19"/>
-      <c r="JX19"/>
-      <c r="JY19"/>
-      <c r="JZ19"/>
-      <c r="KA19"/>
-      <c r="KB19"/>
-      <c r="KC19"/>
-      <c r="KD19"/>
-      <c r="KE19"/>
-      <c r="KF19"/>
-      <c r="KG19"/>
-      <c r="KH19"/>
-      <c r="KI19"/>
-      <c r="KJ19"/>
-      <c r="KK19"/>
-      <c r="KL19"/>
-      <c r="KM19"/>
-      <c r="KN19"/>
-      <c r="KO19"/>
-      <c r="KP19"/>
-      <c r="KQ19"/>
-      <c r="KR19"/>
-      <c r="KS19"/>
-      <c r="KT19"/>
-      <c r="KU19"/>
-      <c r="KV19"/>
-      <c r="KW19"/>
-      <c r="KX19"/>
-      <c r="KY19"/>
-      <c r="KZ19"/>
-      <c r="LA19"/>
-      <c r="LB19"/>
-      <c r="LC19"/>
-      <c r="LD19"/>
-      <c r="LE19"/>
-      <c r="LF19"/>
-      <c r="LG19"/>
-      <c r="LH19"/>
-      <c r="LI19"/>
-      <c r="LJ19"/>
-      <c r="LK19"/>
-      <c r="LL19"/>
-      <c r="LM19"/>
-      <c r="LN19"/>
-      <c r="LO19"/>
-      <c r="LP19"/>
-      <c r="LQ19"/>
-      <c r="LR19"/>
-      <c r="LS19"/>
-      <c r="LT19"/>
-      <c r="LU19"/>
-      <c r="LV19"/>
-      <c r="LW19"/>
-      <c r="LX19"/>
-      <c r="LY19"/>
-      <c r="LZ19"/>
-      <c r="MA19"/>
-      <c r="MB19"/>
-      <c r="MC19"/>
-      <c r="MD19"/>
-      <c r="ME19"/>
-      <c r="MF19"/>
-      <c r="MG19"/>
-      <c r="MH19"/>
-      <c r="MI19"/>
-      <c r="MJ19"/>
-      <c r="MK19"/>
-      <c r="ML19"/>
-      <c r="MM19"/>
-      <c r="MN19"/>
-      <c r="MO19"/>
-      <c r="MP19"/>
-      <c r="MQ19"/>
-      <c r="MR19"/>
-      <c r="MS19"/>
-      <c r="MT19"/>
-      <c r="MU19"/>
-      <c r="MV19"/>
-      <c r="MW19"/>
-      <c r="MX19"/>
-      <c r="MY19"/>
-      <c r="MZ19"/>
-      <c r="NA19"/>
-      <c r="NB19"/>
-      <c r="NC19"/>
-      <c r="ND19"/>
-      <c r="NE19"/>
-      <c r="NF19"/>
-      <c r="NG19"/>
-      <c r="NH19"/>
-      <c r="NI19"/>
-      <c r="NJ19"/>
-      <c r="NK19"/>
-      <c r="NL19"/>
-      <c r="NM19"/>
-      <c r="NN19"/>
-      <c r="NO19"/>
-      <c r="NP19"/>
-      <c r="NQ19"/>
-      <c r="NR19"/>
-      <c r="NS19"/>
-      <c r="NT19"/>
-      <c r="NU19"/>
-      <c r="NV19"/>
-      <c r="NW19"/>
-      <c r="NX19"/>
-      <c r="NY19"/>
-      <c r="NZ19"/>
-      <c r="OA19"/>
-      <c r="OB19"/>
-      <c r="OC19"/>
-      <c r="OD19"/>
-      <c r="OE19"/>
-      <c r="OF19"/>
-      <c r="OG19"/>
-      <c r="OH19"/>
-      <c r="OI19"/>
-      <c r="OJ19"/>
-      <c r="OK19"/>
-      <c r="OL19"/>
-      <c r="OM19"/>
-      <c r="ON19"/>
-      <c r="OO19"/>
-      <c r="OP19"/>
-      <c r="OQ19"/>
-      <c r="OR19"/>
-      <c r="OS19"/>
-      <c r="OT19"/>
-      <c r="OU19"/>
-      <c r="OV19"/>
-      <c r="OW19"/>
-      <c r="OX19"/>
-      <c r="OY19"/>
-      <c r="OZ19"/>
-      <c r="PA19"/>
-      <c r="PB19"/>
-      <c r="PC19"/>
-      <c r="PD19"/>
-      <c r="PE19"/>
-      <c r="PF19"/>
-      <c r="PG19"/>
-      <c r="PH19"/>
-      <c r="PI19"/>
-      <c r="PJ19"/>
-      <c r="PK19"/>
-      <c r="PL19"/>
-      <c r="PM19"/>
-      <c r="PN19"/>
-      <c r="PO19"/>
-      <c r="PP19"/>
-      <c r="PQ19"/>
-      <c r="PR19"/>
-      <c r="PS19"/>
-      <c r="PT19"/>
-      <c r="PU19"/>
-      <c r="PV19"/>
-      <c r="PW19"/>
-      <c r="PX19"/>
-      <c r="PY19"/>
-      <c r="PZ19"/>
-      <c r="QA19"/>
-      <c r="QB19"/>
-      <c r="QC19"/>
-      <c r="QD19"/>
-      <c r="QE19"/>
-      <c r="QF19"/>
-      <c r="QG19"/>
-      <c r="QH19"/>
-      <c r="QI19"/>
-      <c r="QJ19"/>
-      <c r="QK19"/>
-      <c r="QL19"/>
-      <c r="QM19"/>
-      <c r="QN19"/>
-      <c r="QO19"/>
-      <c r="QP19"/>
-      <c r="QQ19"/>
-      <c r="QR19"/>
-      <c r="QS19"/>
-      <c r="QT19"/>
-      <c r="QU19"/>
-      <c r="QV19"/>
-      <c r="QW19"/>
-      <c r="QX19"/>
-      <c r="QY19"/>
-      <c r="QZ19"/>
-      <c r="RA19"/>
-      <c r="RB19"/>
-      <c r="RC19"/>
-      <c r="RD19"/>
-      <c r="RE19"/>
-      <c r="RF19"/>
-      <c r="RG19"/>
-      <c r="RH19"/>
-      <c r="RI19"/>
-      <c r="RJ19"/>
-      <c r="RK19"/>
-      <c r="RL19"/>
-      <c r="RM19"/>
-      <c r="RN19"/>
-      <c r="RO19"/>
-      <c r="RP19"/>
-      <c r="RQ19"/>
-      <c r="RR19"/>
-      <c r="RS19"/>
-      <c r="RT19"/>
-      <c r="RU19"/>
-      <c r="RV19"/>
-      <c r="RW19"/>
-      <c r="RX19"/>
-      <c r="RY19"/>
-      <c r="RZ19"/>
-      <c r="SA19"/>
-      <c r="SB19"/>
-      <c r="SC19"/>
-      <c r="SD19"/>
-      <c r="SE19"/>
-      <c r="SF19"/>
-      <c r="SG19"/>
-      <c r="SH19"/>
-      <c r="SI19"/>
-      <c r="SJ19"/>
-      <c r="SK19"/>
-      <c r="SL19"/>
-      <c r="SM19"/>
-      <c r="SN19"/>
-      <c r="SO19"/>
-      <c r="SP19"/>
-      <c r="SQ19"/>
-      <c r="SR19"/>
-      <c r="SS19"/>
-      <c r="ST19"/>
-      <c r="SU19"/>
-      <c r="SV19"/>
-      <c r="SW19"/>
-      <c r="SX19"/>
-      <c r="SY19"/>
-      <c r="SZ19"/>
-      <c r="TA19"/>
-      <c r="TB19"/>
-      <c r="TC19"/>
-      <c r="TD19"/>
-      <c r="TE19"/>
-      <c r="TF19"/>
-      <c r="TG19"/>
-      <c r="TH19"/>
-      <c r="TI19"/>
-      <c r="TJ19"/>
-      <c r="TK19"/>
-      <c r="TL19"/>
-      <c r="TM19"/>
-      <c r="TN19"/>
-      <c r="TO19"/>
-      <c r="TP19"/>
-      <c r="TQ19"/>
-      <c r="TR19"/>
-      <c r="TS19"/>
-      <c r="TT19"/>
-      <c r="TU19"/>
-      <c r="TV19"/>
-      <c r="TW19"/>
-      <c r="TX19"/>
-      <c r="TY19"/>
-      <c r="TZ19"/>
-      <c r="UA19"/>
-      <c r="UB19"/>
-      <c r="UC19"/>
-      <c r="UD19"/>
-      <c r="UE19"/>
-      <c r="UF19"/>
-      <c r="UG19"/>
-      <c r="UH19"/>
-      <c r="UI19"/>
-      <c r="UJ19"/>
-      <c r="UK19"/>
-      <c r="UL19"/>
-      <c r="UM19"/>
-      <c r="UN19"/>
-      <c r="UO19"/>
-      <c r="UP19"/>
-      <c r="UQ19"/>
-      <c r="UR19"/>
-      <c r="US19"/>
-      <c r="UT19"/>
-      <c r="UU19"/>
-      <c r="UV19"/>
-      <c r="UW19"/>
-      <c r="UX19"/>
-      <c r="UY19"/>
-      <c r="UZ19"/>
-      <c r="VA19"/>
-      <c r="VB19"/>
-      <c r="VC19"/>
-      <c r="VD19"/>
-      <c r="VE19"/>
-      <c r="VF19"/>
-      <c r="VG19"/>
-      <c r="VH19"/>
-      <c r="VI19"/>
-      <c r="VJ19"/>
-      <c r="VK19"/>
-      <c r="VL19"/>
-      <c r="VM19"/>
-      <c r="VN19"/>
-      <c r="VO19"/>
-      <c r="VP19"/>
-      <c r="VQ19"/>
-      <c r="VR19"/>
-      <c r="VS19"/>
-      <c r="VT19"/>
-      <c r="VU19"/>
-      <c r="VV19"/>
-      <c r="VW19"/>
-      <c r="VX19"/>
-      <c r="VY19"/>
-      <c r="VZ19"/>
-      <c r="WA19"/>
-      <c r="WB19"/>
-      <c r="WC19"/>
-      <c r="WD19"/>
-      <c r="WE19"/>
-      <c r="WF19"/>
-      <c r="WG19"/>
-      <c r="WH19"/>
-      <c r="WI19"/>
-      <c r="WJ19"/>
-      <c r="WK19"/>
-      <c r="WL19"/>
-      <c r="WM19"/>
-      <c r="WN19"/>
-      <c r="WO19"/>
-      <c r="WP19"/>
-      <c r="WQ19"/>
-      <c r="WR19"/>
-      <c r="WS19"/>
-      <c r="WT19"/>
-      <c r="WU19"/>
-      <c r="WV19"/>
-      <c r="WW19"/>
-      <c r="WX19"/>
-      <c r="WY19"/>
-      <c r="WZ19"/>
-      <c r="XA19"/>
-      <c r="XB19"/>
-      <c r="XC19"/>
-      <c r="XD19"/>
-      <c r="XE19"/>
-      <c r="XF19"/>
-      <c r="XG19"/>
-      <c r="XH19"/>
-      <c r="XI19"/>
-      <c r="XJ19"/>
-      <c r="XK19"/>
-      <c r="XL19"/>
-      <c r="XM19"/>
-      <c r="XN19"/>
-      <c r="XO19"/>
-      <c r="XP19"/>
-      <c r="XQ19"/>
-      <c r="XR19"/>
-      <c r="XS19"/>
-      <c r="XT19"/>
-      <c r="XU19"/>
-      <c r="XV19"/>
-      <c r="XW19"/>
-      <c r="XX19"/>
-      <c r="XY19"/>
-      <c r="XZ19"/>
-      <c r="YA19"/>
-      <c r="YB19"/>
-      <c r="YC19"/>
-      <c r="YD19"/>
-      <c r="YE19"/>
-      <c r="YF19"/>
-      <c r="YG19"/>
-      <c r="YH19"/>
-      <c r="YI19"/>
-      <c r="YJ19"/>
-      <c r="YK19"/>
-      <c r="YL19"/>
-      <c r="YM19"/>
-      <c r="YN19"/>
-      <c r="YO19"/>
-      <c r="YP19"/>
-      <c r="YQ19"/>
-      <c r="YR19"/>
-      <c r="YS19"/>
-      <c r="YT19"/>
-      <c r="YU19"/>
-      <c r="YV19"/>
-      <c r="YW19"/>
-      <c r="YX19"/>
-      <c r="YY19"/>
-      <c r="YZ19"/>
-      <c r="ZA19"/>
-      <c r="ZB19"/>
-      <c r="ZC19"/>
-      <c r="ZD19"/>
-      <c r="ZE19"/>
-      <c r="ZF19"/>
-      <c r="ZG19"/>
-      <c r="ZH19"/>
-      <c r="ZI19"/>
-      <c r="ZJ19"/>
-      <c r="ZK19"/>
-      <c r="ZL19"/>
-      <c r="ZM19"/>
-      <c r="ZN19"/>
-      <c r="ZO19"/>
-      <c r="ZP19"/>
-      <c r="ZQ19"/>
-      <c r="ZR19"/>
-      <c r="ZS19"/>
-      <c r="ZT19"/>
-      <c r="ZU19"/>
-      <c r="ZV19"/>
-      <c r="ZW19"/>
-      <c r="ZX19"/>
-      <c r="ZY19"/>
-      <c r="ZZ19"/>
-      <c r="AAA19"/>
-      <c r="AAB19"/>
-      <c r="AAC19"/>
-      <c r="AAD19"/>
-      <c r="AAE19"/>
-      <c r="AAF19"/>
-      <c r="AAG19"/>
-      <c r="AAH19"/>
-      <c r="AAI19"/>
-      <c r="AAJ19"/>
-      <c r="AAK19"/>
-      <c r="AAL19"/>
-      <c r="AAM19"/>
-      <c r="AAN19"/>
-      <c r="AAO19"/>
-      <c r="AAP19"/>
-      <c r="AAQ19"/>
-      <c r="AAR19"/>
-      <c r="AAS19"/>
-      <c r="AAT19"/>
-      <c r="AAU19"/>
-      <c r="AAV19"/>
-      <c r="AAW19"/>
-      <c r="AAX19"/>
-      <c r="AAY19"/>
-      <c r="AAZ19"/>
-      <c r="ABA19"/>
-      <c r="ABB19"/>
-      <c r="ABC19"/>
-      <c r="ABD19"/>
-      <c r="ABE19"/>
-      <c r="ABF19"/>
-      <c r="ABG19"/>
-      <c r="ABH19"/>
-      <c r="ABI19"/>
-      <c r="ABJ19"/>
-      <c r="ABK19"/>
-      <c r="ABL19"/>
-      <c r="ABM19"/>
-      <c r="ABN19"/>
-      <c r="ABO19"/>
-      <c r="ABP19"/>
-      <c r="ABQ19"/>
-      <c r="ABR19"/>
-      <c r="ABS19"/>
-      <c r="ABT19"/>
-      <c r="ABU19"/>
-      <c r="ABV19"/>
-      <c r="ABW19"/>
-      <c r="ABX19"/>
-      <c r="ABY19"/>
-      <c r="ABZ19"/>
-      <c r="ACA19"/>
-      <c r="ACB19"/>
-      <c r="ACC19"/>
-      <c r="ACD19"/>
-      <c r="ACE19"/>
-      <c r="ACF19"/>
-      <c r="ACG19"/>
-      <c r="ACH19"/>
-      <c r="ACI19"/>
-      <c r="ACJ19"/>
-      <c r="ACK19"/>
-      <c r="ACL19"/>
-      <c r="ACM19"/>
-      <c r="ACN19"/>
-      <c r="ACO19"/>
-      <c r="ACP19"/>
-      <c r="ACQ19"/>
-      <c r="ACR19"/>
-      <c r="ACS19"/>
-      <c r="ACT19"/>
-      <c r="ACU19"/>
-      <c r="ACV19"/>
-      <c r="ACW19"/>
-      <c r="ACX19"/>
-      <c r="ACY19"/>
-      <c r="ACZ19"/>
-      <c r="ADA19"/>
-      <c r="ADB19"/>
-      <c r="ADC19"/>
-      <c r="ADD19"/>
-      <c r="ADE19"/>
-      <c r="ADF19"/>
-      <c r="ADG19"/>
-      <c r="ADH19"/>
-      <c r="ADI19"/>
-      <c r="ADJ19"/>
-      <c r="ADK19"/>
-      <c r="ADL19"/>
-      <c r="ADM19"/>
-      <c r="ADN19"/>
-      <c r="ADO19"/>
-      <c r="ADP19"/>
-      <c r="ADQ19"/>
-      <c r="ADR19"/>
-      <c r="ADS19"/>
-      <c r="ADT19"/>
-      <c r="ADU19"/>
-      <c r="ADV19"/>
-      <c r="ADW19"/>
-      <c r="ADX19"/>
-      <c r="ADY19"/>
-      <c r="ADZ19"/>
-      <c r="AEA19"/>
-      <c r="AEB19"/>
-      <c r="AEC19"/>
-      <c r="AED19"/>
-      <c r="AEE19"/>
-      <c r="AEF19"/>
-      <c r="AEG19"/>
-      <c r="AEH19"/>
-      <c r="AEI19"/>
-      <c r="AEJ19"/>
-      <c r="AEK19"/>
-      <c r="AEL19"/>
-      <c r="AEM19"/>
-      <c r="AEN19"/>
-      <c r="AEO19"/>
-      <c r="AEP19"/>
-      <c r="AEQ19"/>
-      <c r="AER19"/>
-      <c r="AES19"/>
-      <c r="AET19"/>
-      <c r="AEU19"/>
-      <c r="AEV19"/>
-      <c r="AEW19"/>
-      <c r="AEX19"/>
-      <c r="AEY19"/>
-      <c r="AEZ19"/>
-      <c r="AFA19"/>
-      <c r="AFB19"/>
-      <c r="AFC19"/>
-      <c r="AFD19"/>
-      <c r="AFE19"/>
-      <c r="AFF19"/>
-      <c r="AFG19"/>
-      <c r="AFH19"/>
-      <c r="AFI19"/>
-      <c r="AFJ19"/>
-      <c r="AFK19"/>
-      <c r="AFL19"/>
-      <c r="AFM19"/>
-      <c r="AFN19"/>
-      <c r="AFO19"/>
-      <c r="AFP19"/>
-      <c r="AFQ19"/>
-      <c r="AFR19"/>
-      <c r="AFS19"/>
-      <c r="AFT19"/>
-      <c r="AFU19"/>
-      <c r="AFV19"/>
-      <c r="AFW19"/>
-      <c r="AFX19"/>
-      <c r="AFY19"/>
-      <c r="AFZ19"/>
-      <c r="AGA19"/>
-      <c r="AGB19"/>
-      <c r="AGC19"/>
-      <c r="AGD19"/>
-      <c r="AGE19"/>
-      <c r="AGF19"/>
-      <c r="AGG19"/>
-      <c r="AGH19"/>
-      <c r="AGI19"/>
-      <c r="AGJ19"/>
-      <c r="AGK19"/>
-      <c r="AGL19"/>
-      <c r="AGM19"/>
-      <c r="AGN19"/>
-      <c r="AGO19"/>
-      <c r="AGP19"/>
-      <c r="AGQ19"/>
-      <c r="AGR19"/>
-      <c r="AGS19"/>
-      <c r="AGT19"/>
-      <c r="AGU19"/>
-      <c r="AGV19"/>
-      <c r="AGW19"/>
-      <c r="AGX19"/>
-      <c r="AGY19"/>
-      <c r="AGZ19"/>
-      <c r="AHA19"/>
-      <c r="AHB19"/>
-      <c r="AHC19"/>
-      <c r="AHD19"/>
-      <c r="AHE19"/>
-      <c r="AHF19"/>
-      <c r="AHG19"/>
-      <c r="AHH19"/>
-      <c r="AHI19"/>
-      <c r="AHJ19"/>
-      <c r="AHK19"/>
-      <c r="AHL19"/>
-      <c r="AHM19"/>
-      <c r="AHN19"/>
-      <c r="AHO19"/>
-      <c r="AHP19"/>
-      <c r="AHQ19"/>
-      <c r="AHR19"/>
-      <c r="AHS19"/>
-      <c r="AHT19"/>
-      <c r="AHU19"/>
-      <c r="AHV19"/>
-      <c r="AHW19"/>
-      <c r="AHX19"/>
-      <c r="AHY19"/>
-      <c r="AHZ19"/>
-      <c r="AIA19"/>
-      <c r="AIB19"/>
-      <c r="AIC19"/>
-      <c r="AID19"/>
-      <c r="AIE19"/>
-      <c r="AIF19"/>
-      <c r="AIG19"/>
-      <c r="AIH19"/>
-      <c r="AII19"/>
-      <c r="AIJ19"/>
-      <c r="AIK19"/>
-      <c r="AIL19"/>
-      <c r="AIM19"/>
-      <c r="AIN19"/>
-      <c r="AIO19"/>
-      <c r="AIP19"/>
-      <c r="AIQ19"/>
-      <c r="AIR19"/>
-      <c r="AIS19"/>
-      <c r="AIT19"/>
-      <c r="AIU19"/>
-      <c r="AIV19"/>
-      <c r="AIW19"/>
-      <c r="AIX19"/>
-      <c r="AIY19"/>
-      <c r="AIZ19"/>
-      <c r="AJA19"/>
-      <c r="AJB19"/>
-      <c r="AJC19"/>
-      <c r="AJD19"/>
-      <c r="AJE19"/>
-      <c r="AJF19"/>
-      <c r="AJG19"/>
-      <c r="AJH19"/>
-      <c r="AJI19"/>
-      <c r="AJJ19"/>
-      <c r="AJK19"/>
-      <c r="AJL19"/>
-      <c r="AJM19"/>
-      <c r="AJN19"/>
-      <c r="AJO19"/>
-      <c r="AJP19"/>
-      <c r="AJQ19"/>
-      <c r="AJR19"/>
-      <c r="AJS19"/>
-      <c r="AJT19"/>
-      <c r="AJU19"/>
-      <c r="AJV19"/>
-      <c r="AJW19"/>
-      <c r="AJX19"/>
-      <c r="AJY19"/>
-      <c r="AJZ19"/>
-      <c r="AKA19"/>
-      <c r="AKB19"/>
-      <c r="AKC19"/>
-      <c r="AKD19"/>
-      <c r="AKE19"/>
-      <c r="AKF19"/>
-      <c r="AKG19"/>
-      <c r="AKH19"/>
-      <c r="AKI19"/>
-      <c r="AKJ19"/>
-      <c r="AKK19"/>
-      <c r="AKL19"/>
-      <c r="AKM19"/>
-      <c r="AKN19"/>
-      <c r="AKO19"/>
-      <c r="AKP19"/>
-      <c r="AKQ19"/>
-      <c r="AKR19"/>
-      <c r="AKS19"/>
-      <c r="AKT19"/>
-      <c r="AKU19"/>
-      <c r="AKV19"/>
-      <c r="AKW19"/>
-      <c r="AKX19"/>
-      <c r="AKY19"/>
-      <c r="AKZ19"/>
-      <c r="ALA19"/>
-      <c r="ALB19"/>
-      <c r="ALC19"/>
-      <c r="ALD19"/>
-      <c r="ALE19"/>
-      <c r="ALF19"/>
-      <c r="ALG19"/>
-      <c r="ALH19"/>
-      <c r="ALI19"/>
-      <c r="ALJ19"/>
-      <c r="ALK19"/>
-      <c r="ALL19"/>
-      <c r="ALM19"/>
-      <c r="ALN19"/>
-      <c r="ALO19"/>
-      <c r="ALP19"/>
-      <c r="ALQ19"/>
-      <c r="ALR19"/>
-      <c r="ALS19"/>
-      <c r="ALT19"/>
-      <c r="ALU19"/>
-      <c r="ALV19"/>
-      <c r="ALW19"/>
-      <c r="ALX19"/>
-      <c r="ALY19"/>
-      <c r="ALZ19"/>
-      <c r="AMA19"/>
-      <c r="AMB19"/>
-      <c r="AMC19"/>
-      <c r="AMD19"/>
-      <c r="AME19"/>
-      <c r="AMF19"/>
-      <c r="AMG19"/>
-      <c r="AMH19"/>
-      <c r="AMI19"/>
-      <c r="AMJ19"/>
-      <c r="AMK19"/>
-    </row>
-    <row r="20" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="67" t="s">
+      <c r="B20" s="78"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+      <c r="AR20"/>
+      <c r="AS20"/>
+      <c r="AT20"/>
+      <c r="AU20"/>
+      <c r="AV20"/>
+      <c r="AW20"/>
+      <c r="AX20"/>
+      <c r="AY20"/>
+      <c r="AZ20"/>
+      <c r="BA20"/>
+      <c r="BB20"/>
+      <c r="BC20"/>
+      <c r="BD20"/>
+      <c r="BE20"/>
+      <c r="BF20"/>
+      <c r="BG20"/>
+      <c r="BH20"/>
+      <c r="BI20"/>
+      <c r="BJ20"/>
+      <c r="BK20"/>
+      <c r="BL20"/>
+      <c r="BM20"/>
+      <c r="BN20"/>
+      <c r="BO20"/>
+      <c r="BP20"/>
+      <c r="BQ20"/>
+      <c r="BR20"/>
+      <c r="BS20"/>
+      <c r="BT20"/>
+      <c r="BU20"/>
+      <c r="BV20"/>
+      <c r="BW20"/>
+      <c r="BX20"/>
+      <c r="BY20"/>
+      <c r="BZ20"/>
+      <c r="CA20"/>
+      <c r="CB20"/>
+      <c r="CC20"/>
+      <c r="CD20"/>
+      <c r="CE20"/>
+      <c r="CF20"/>
+      <c r="CG20"/>
+      <c r="CH20"/>
+      <c r="CI20"/>
+      <c r="CJ20"/>
+      <c r="CK20"/>
+      <c r="CL20"/>
+      <c r="CM20"/>
+      <c r="CN20"/>
+      <c r="CO20"/>
+      <c r="CP20"/>
+      <c r="CQ20"/>
+      <c r="CR20"/>
+      <c r="CS20"/>
+      <c r="CT20"/>
+      <c r="CU20"/>
+      <c r="CV20"/>
+      <c r="CW20"/>
+      <c r="CX20"/>
+      <c r="CY20"/>
+      <c r="CZ20"/>
+      <c r="DA20"/>
+      <c r="DB20"/>
+      <c r="DC20"/>
+      <c r="DD20"/>
+      <c r="DE20"/>
+      <c r="DF20"/>
+      <c r="DG20"/>
+      <c r="DH20"/>
+      <c r="DI20"/>
+      <c r="DJ20"/>
+      <c r="DK20"/>
+      <c r="DL20"/>
+      <c r="DM20"/>
+      <c r="DN20"/>
+      <c r="DO20"/>
+      <c r="DP20"/>
+      <c r="DQ20"/>
+      <c r="DR20"/>
+      <c r="DS20"/>
+      <c r="DT20"/>
+      <c r="DU20"/>
+      <c r="DV20"/>
+      <c r="DW20"/>
+      <c r="DX20"/>
+      <c r="DY20"/>
+      <c r="DZ20"/>
+      <c r="EA20"/>
+      <c r="EB20"/>
+      <c r="EC20"/>
+      <c r="ED20"/>
+      <c r="EE20"/>
+      <c r="EF20"/>
+      <c r="EG20"/>
+      <c r="EH20"/>
+      <c r="EI20"/>
+      <c r="EJ20"/>
+      <c r="EK20"/>
+      <c r="EL20"/>
+      <c r="EM20"/>
+      <c r="EN20"/>
+      <c r="EO20"/>
+      <c r="EP20"/>
+      <c r="EQ20"/>
+      <c r="ER20"/>
+      <c r="ES20"/>
+      <c r="ET20"/>
+      <c r="EU20"/>
+      <c r="EV20"/>
+      <c r="EW20"/>
+      <c r="EX20"/>
+      <c r="EY20"/>
+      <c r="EZ20"/>
+      <c r="FA20"/>
+      <c r="FB20"/>
+      <c r="FC20"/>
+      <c r="FD20"/>
+      <c r="FE20"/>
+      <c r="FF20"/>
+      <c r="FG20"/>
+      <c r="FH20"/>
+      <c r="FI20"/>
+      <c r="FJ20"/>
+      <c r="FK20"/>
+      <c r="FL20"/>
+      <c r="FM20"/>
+      <c r="FN20"/>
+      <c r="FO20"/>
+      <c r="FP20"/>
+      <c r="FQ20"/>
+      <c r="FR20"/>
+      <c r="FS20"/>
+      <c r="FT20"/>
+      <c r="FU20"/>
+      <c r="FV20"/>
+      <c r="FW20"/>
+      <c r="FX20"/>
+      <c r="FY20"/>
+      <c r="FZ20"/>
+      <c r="GA20"/>
+      <c r="GB20"/>
+      <c r="GC20"/>
+      <c r="GD20"/>
+      <c r="GE20"/>
+      <c r="GF20"/>
+      <c r="GG20"/>
+      <c r="GH20"/>
+      <c r="GI20"/>
+      <c r="GJ20"/>
+      <c r="GK20"/>
+      <c r="GL20"/>
+      <c r="GM20"/>
+      <c r="GN20"/>
+      <c r="GO20"/>
+      <c r="GP20"/>
+      <c r="GQ20"/>
+      <c r="GR20"/>
+      <c r="GS20"/>
+      <c r="GT20"/>
+      <c r="GU20"/>
+      <c r="GV20"/>
+      <c r="GW20"/>
+      <c r="GX20"/>
+      <c r="GY20"/>
+      <c r="GZ20"/>
+      <c r="HA20"/>
+      <c r="HB20"/>
+      <c r="HC20"/>
+      <c r="HD20"/>
+      <c r="HE20"/>
+      <c r="HF20"/>
+      <c r="HG20"/>
+      <c r="HH20"/>
+      <c r="HI20"/>
+      <c r="HJ20"/>
+      <c r="HK20"/>
+      <c r="HL20"/>
+      <c r="HM20"/>
+      <c r="HN20"/>
+      <c r="HO20"/>
+      <c r="HP20"/>
+      <c r="HQ20"/>
+      <c r="HR20"/>
+      <c r="HS20"/>
+      <c r="HT20"/>
+      <c r="HU20"/>
+      <c r="HV20"/>
+      <c r="HW20"/>
+      <c r="HX20"/>
+      <c r="HY20"/>
+      <c r="HZ20"/>
+      <c r="IA20"/>
+      <c r="IB20"/>
+      <c r="IC20"/>
+      <c r="ID20"/>
+      <c r="IE20"/>
+      <c r="IF20"/>
+      <c r="IG20"/>
+      <c r="IH20"/>
+      <c r="II20"/>
+      <c r="IJ20"/>
+      <c r="IK20"/>
+      <c r="IL20"/>
+      <c r="IM20"/>
+      <c r="IN20"/>
+      <c r="IO20"/>
+      <c r="IP20"/>
+      <c r="IQ20"/>
+      <c r="IR20"/>
+      <c r="IS20"/>
+      <c r="IT20"/>
+      <c r="IU20"/>
+      <c r="IV20"/>
+      <c r="IW20"/>
+      <c r="IX20"/>
+      <c r="IY20"/>
+      <c r="IZ20"/>
+      <c r="JA20"/>
+      <c r="JB20"/>
+      <c r="JC20"/>
+      <c r="JD20"/>
+      <c r="JE20"/>
+      <c r="JF20"/>
+      <c r="JG20"/>
+      <c r="JH20"/>
+      <c r="JI20"/>
+      <c r="JJ20"/>
+      <c r="JK20"/>
+      <c r="JL20"/>
+      <c r="JM20"/>
+      <c r="JN20"/>
+      <c r="JO20"/>
+      <c r="JP20"/>
+      <c r="JQ20"/>
+      <c r="JR20"/>
+      <c r="JS20"/>
+      <c r="JT20"/>
+      <c r="JU20"/>
+      <c r="JV20"/>
+      <c r="JW20"/>
+      <c r="JX20"/>
+      <c r="JY20"/>
+      <c r="JZ20"/>
+      <c r="KA20"/>
+      <c r="KB20"/>
+      <c r="KC20"/>
+      <c r="KD20"/>
+      <c r="KE20"/>
+      <c r="KF20"/>
+      <c r="KG20"/>
+      <c r="KH20"/>
+      <c r="KI20"/>
+      <c r="KJ20"/>
+      <c r="KK20"/>
+      <c r="KL20"/>
+      <c r="KM20"/>
+      <c r="KN20"/>
+      <c r="KO20"/>
+      <c r="KP20"/>
+      <c r="KQ20"/>
+      <c r="KR20"/>
+      <c r="KS20"/>
+      <c r="KT20"/>
+      <c r="KU20"/>
+      <c r="KV20"/>
+      <c r="KW20"/>
+      <c r="KX20"/>
+      <c r="KY20"/>
+      <c r="KZ20"/>
+      <c r="LA20"/>
+      <c r="LB20"/>
+      <c r="LC20"/>
+      <c r="LD20"/>
+      <c r="LE20"/>
+      <c r="LF20"/>
+      <c r="LG20"/>
+      <c r="LH20"/>
+      <c r="LI20"/>
+      <c r="LJ20"/>
+      <c r="LK20"/>
+      <c r="LL20"/>
+      <c r="LM20"/>
+      <c r="LN20"/>
+      <c r="LO20"/>
+      <c r="LP20"/>
+      <c r="LQ20"/>
+      <c r="LR20"/>
+      <c r="LS20"/>
+      <c r="LT20"/>
+      <c r="LU20"/>
+      <c r="LV20"/>
+      <c r="LW20"/>
+      <c r="LX20"/>
+      <c r="LY20"/>
+      <c r="LZ20"/>
+      <c r="MA20"/>
+      <c r="MB20"/>
+      <c r="MC20"/>
+      <c r="MD20"/>
+      <c r="ME20"/>
+      <c r="MF20"/>
+      <c r="MG20"/>
+      <c r="MH20"/>
+      <c r="MI20"/>
+      <c r="MJ20"/>
+      <c r="MK20"/>
+      <c r="ML20"/>
+      <c r="MM20"/>
+      <c r="MN20"/>
+      <c r="MO20"/>
+      <c r="MP20"/>
+      <c r="MQ20"/>
+      <c r="MR20"/>
+      <c r="MS20"/>
+      <c r="MT20"/>
+      <c r="MU20"/>
+      <c r="MV20"/>
+      <c r="MW20"/>
+      <c r="MX20"/>
+      <c r="MY20"/>
+      <c r="MZ20"/>
+      <c r="NA20"/>
+      <c r="NB20"/>
+      <c r="NC20"/>
+      <c r="ND20"/>
+      <c r="NE20"/>
+      <c r="NF20"/>
+      <c r="NG20"/>
+      <c r="NH20"/>
+      <c r="NI20"/>
+      <c r="NJ20"/>
+      <c r="NK20"/>
+      <c r="NL20"/>
+      <c r="NM20"/>
+      <c r="NN20"/>
+      <c r="NO20"/>
+      <c r="NP20"/>
+      <c r="NQ20"/>
+      <c r="NR20"/>
+      <c r="NS20"/>
+      <c r="NT20"/>
+      <c r="NU20"/>
+      <c r="NV20"/>
+      <c r="NW20"/>
+      <c r="NX20"/>
+      <c r="NY20"/>
+      <c r="NZ20"/>
+      <c r="OA20"/>
+      <c r="OB20"/>
+      <c r="OC20"/>
+      <c r="OD20"/>
+      <c r="OE20"/>
+      <c r="OF20"/>
+      <c r="OG20"/>
+      <c r="OH20"/>
+      <c r="OI20"/>
+      <c r="OJ20"/>
+      <c r="OK20"/>
+      <c r="OL20"/>
+      <c r="OM20"/>
+      <c r="ON20"/>
+      <c r="OO20"/>
+      <c r="OP20"/>
+      <c r="OQ20"/>
+      <c r="OR20"/>
+      <c r="OS20"/>
+      <c r="OT20"/>
+      <c r="OU20"/>
+      <c r="OV20"/>
+      <c r="OW20"/>
+      <c r="OX20"/>
+      <c r="OY20"/>
+      <c r="OZ20"/>
+      <c r="PA20"/>
+      <c r="PB20"/>
+      <c r="PC20"/>
+      <c r="PD20"/>
+      <c r="PE20"/>
+      <c r="PF20"/>
+      <c r="PG20"/>
+      <c r="PH20"/>
+      <c r="PI20"/>
+      <c r="PJ20"/>
+      <c r="PK20"/>
+      <c r="PL20"/>
+      <c r="PM20"/>
+      <c r="PN20"/>
+      <c r="PO20"/>
+      <c r="PP20"/>
+      <c r="PQ20"/>
+      <c r="PR20"/>
+      <c r="PS20"/>
+      <c r="PT20"/>
+      <c r="PU20"/>
+      <c r="PV20"/>
+      <c r="PW20"/>
+      <c r="PX20"/>
+      <c r="PY20"/>
+      <c r="PZ20"/>
+      <c r="QA20"/>
+      <c r="QB20"/>
+      <c r="QC20"/>
+      <c r="QD20"/>
+      <c r="QE20"/>
+      <c r="QF20"/>
+      <c r="QG20"/>
+      <c r="QH20"/>
+      <c r="QI20"/>
+      <c r="QJ20"/>
+      <c r="QK20"/>
+      <c r="QL20"/>
+      <c r="QM20"/>
+      <c r="QN20"/>
+      <c r="QO20"/>
+      <c r="QP20"/>
+      <c r="QQ20"/>
+      <c r="QR20"/>
+      <c r="QS20"/>
+      <c r="QT20"/>
+      <c r="QU20"/>
+      <c r="QV20"/>
+      <c r="QW20"/>
+      <c r="QX20"/>
+      <c r="QY20"/>
+      <c r="QZ20"/>
+      <c r="RA20"/>
+      <c r="RB20"/>
+      <c r="RC20"/>
+      <c r="RD20"/>
+      <c r="RE20"/>
+      <c r="RF20"/>
+      <c r="RG20"/>
+      <c r="RH20"/>
+      <c r="RI20"/>
+      <c r="RJ20"/>
+      <c r="RK20"/>
+      <c r="RL20"/>
+      <c r="RM20"/>
+      <c r="RN20"/>
+      <c r="RO20"/>
+      <c r="RP20"/>
+      <c r="RQ20"/>
+      <c r="RR20"/>
+      <c r="RS20"/>
+      <c r="RT20"/>
+      <c r="RU20"/>
+      <c r="RV20"/>
+      <c r="RW20"/>
+      <c r="RX20"/>
+      <c r="RY20"/>
+      <c r="RZ20"/>
+      <c r="SA20"/>
+      <c r="SB20"/>
+      <c r="SC20"/>
+      <c r="SD20"/>
+      <c r="SE20"/>
+      <c r="SF20"/>
+      <c r="SG20"/>
+      <c r="SH20"/>
+      <c r="SI20"/>
+      <c r="SJ20"/>
+      <c r="SK20"/>
+      <c r="SL20"/>
+      <c r="SM20"/>
+      <c r="SN20"/>
+      <c r="SO20"/>
+      <c r="SP20"/>
+      <c r="SQ20"/>
+      <c r="SR20"/>
+      <c r="SS20"/>
+      <c r="ST20"/>
+      <c r="SU20"/>
+      <c r="SV20"/>
+      <c r="SW20"/>
+      <c r="SX20"/>
+      <c r="SY20"/>
+      <c r="SZ20"/>
+      <c r="TA20"/>
+      <c r="TB20"/>
+      <c r="TC20"/>
+      <c r="TD20"/>
+      <c r="TE20"/>
+      <c r="TF20"/>
+      <c r="TG20"/>
+      <c r="TH20"/>
+      <c r="TI20"/>
+      <c r="TJ20"/>
+      <c r="TK20"/>
+      <c r="TL20"/>
+      <c r="TM20"/>
+      <c r="TN20"/>
+      <c r="TO20"/>
+      <c r="TP20"/>
+      <c r="TQ20"/>
+      <c r="TR20"/>
+      <c r="TS20"/>
+      <c r="TT20"/>
+      <c r="TU20"/>
+      <c r="TV20"/>
+      <c r="TW20"/>
+      <c r="TX20"/>
+      <c r="TY20"/>
+      <c r="TZ20"/>
+      <c r="UA20"/>
+      <c r="UB20"/>
+      <c r="UC20"/>
+      <c r="UD20"/>
+      <c r="UE20"/>
+      <c r="UF20"/>
+      <c r="UG20"/>
+      <c r="UH20"/>
+      <c r="UI20"/>
+      <c r="UJ20"/>
+      <c r="UK20"/>
+      <c r="UL20"/>
+      <c r="UM20"/>
+      <c r="UN20"/>
+      <c r="UO20"/>
+      <c r="UP20"/>
+      <c r="UQ20"/>
+      <c r="UR20"/>
+      <c r="US20"/>
+      <c r="UT20"/>
+      <c r="UU20"/>
+      <c r="UV20"/>
+      <c r="UW20"/>
+      <c r="UX20"/>
+      <c r="UY20"/>
+      <c r="UZ20"/>
+      <c r="VA20"/>
+      <c r="VB20"/>
+      <c r="VC20"/>
+      <c r="VD20"/>
+      <c r="VE20"/>
+      <c r="VF20"/>
+      <c r="VG20"/>
+      <c r="VH20"/>
+      <c r="VI20"/>
+      <c r="VJ20"/>
+      <c r="VK20"/>
+      <c r="VL20"/>
+      <c r="VM20"/>
+      <c r="VN20"/>
+      <c r="VO20"/>
+      <c r="VP20"/>
+      <c r="VQ20"/>
+      <c r="VR20"/>
+      <c r="VS20"/>
+      <c r="VT20"/>
+      <c r="VU20"/>
+      <c r="VV20"/>
+      <c r="VW20"/>
+      <c r="VX20"/>
+      <c r="VY20"/>
+      <c r="VZ20"/>
+      <c r="WA20"/>
+      <c r="WB20"/>
+      <c r="WC20"/>
+      <c r="WD20"/>
+      <c r="WE20"/>
+      <c r="WF20"/>
+      <c r="WG20"/>
+      <c r="WH20"/>
+      <c r="WI20"/>
+      <c r="WJ20"/>
+      <c r="WK20"/>
+      <c r="WL20"/>
+      <c r="WM20"/>
+      <c r="WN20"/>
+      <c r="WO20"/>
+      <c r="WP20"/>
+      <c r="WQ20"/>
+      <c r="WR20"/>
+      <c r="WS20"/>
+      <c r="WT20"/>
+      <c r="WU20"/>
+      <c r="WV20"/>
+      <c r="WW20"/>
+      <c r="WX20"/>
+      <c r="WY20"/>
+      <c r="WZ20"/>
+      <c r="XA20"/>
+      <c r="XB20"/>
+      <c r="XC20"/>
+      <c r="XD20"/>
+      <c r="XE20"/>
+      <c r="XF20"/>
+      <c r="XG20"/>
+      <c r="XH20"/>
+      <c r="XI20"/>
+      <c r="XJ20"/>
+      <c r="XK20"/>
+      <c r="XL20"/>
+      <c r="XM20"/>
+      <c r="XN20"/>
+      <c r="XO20"/>
+      <c r="XP20"/>
+      <c r="XQ20"/>
+      <c r="XR20"/>
+      <c r="XS20"/>
+      <c r="XT20"/>
+      <c r="XU20"/>
+      <c r="XV20"/>
+      <c r="XW20"/>
+      <c r="XX20"/>
+      <c r="XY20"/>
+      <c r="XZ20"/>
+      <c r="YA20"/>
+      <c r="YB20"/>
+      <c r="YC20"/>
+      <c r="YD20"/>
+      <c r="YE20"/>
+      <c r="YF20"/>
+      <c r="YG20"/>
+      <c r="YH20"/>
+      <c r="YI20"/>
+      <c r="YJ20"/>
+      <c r="YK20"/>
+      <c r="YL20"/>
+      <c r="YM20"/>
+      <c r="YN20"/>
+      <c r="YO20"/>
+      <c r="YP20"/>
+      <c r="YQ20"/>
+      <c r="YR20"/>
+      <c r="YS20"/>
+      <c r="YT20"/>
+      <c r="YU20"/>
+      <c r="YV20"/>
+      <c r="YW20"/>
+      <c r="YX20"/>
+      <c r="YY20"/>
+      <c r="YZ20"/>
+      <c r="ZA20"/>
+      <c r="ZB20"/>
+      <c r="ZC20"/>
+      <c r="ZD20"/>
+      <c r="ZE20"/>
+      <c r="ZF20"/>
+      <c r="ZG20"/>
+      <c r="ZH20"/>
+      <c r="ZI20"/>
+      <c r="ZJ20"/>
+      <c r="ZK20"/>
+      <c r="ZL20"/>
+      <c r="ZM20"/>
+      <c r="ZN20"/>
+      <c r="ZO20"/>
+      <c r="ZP20"/>
+      <c r="ZQ20"/>
+      <c r="ZR20"/>
+      <c r="ZS20"/>
+      <c r="ZT20"/>
+      <c r="ZU20"/>
+      <c r="ZV20"/>
+      <c r="ZW20"/>
+      <c r="ZX20"/>
+      <c r="ZY20"/>
+      <c r="ZZ20"/>
+      <c r="AAA20"/>
+      <c r="AAB20"/>
+      <c r="AAC20"/>
+      <c r="AAD20"/>
+      <c r="AAE20"/>
+      <c r="AAF20"/>
+      <c r="AAG20"/>
+      <c r="AAH20"/>
+      <c r="AAI20"/>
+      <c r="AAJ20"/>
+      <c r="AAK20"/>
+      <c r="AAL20"/>
+      <c r="AAM20"/>
+      <c r="AAN20"/>
+      <c r="AAO20"/>
+      <c r="AAP20"/>
+      <c r="AAQ20"/>
+      <c r="AAR20"/>
+      <c r="AAS20"/>
+      <c r="AAT20"/>
+      <c r="AAU20"/>
+      <c r="AAV20"/>
+      <c r="AAW20"/>
+      <c r="AAX20"/>
+      <c r="AAY20"/>
+      <c r="AAZ20"/>
+      <c r="ABA20"/>
+      <c r="ABB20"/>
+      <c r="ABC20"/>
+      <c r="ABD20"/>
+      <c r="ABE20"/>
+      <c r="ABF20"/>
+      <c r="ABG20"/>
+      <c r="ABH20"/>
+      <c r="ABI20"/>
+      <c r="ABJ20"/>
+      <c r="ABK20"/>
+      <c r="ABL20"/>
+      <c r="ABM20"/>
+      <c r="ABN20"/>
+      <c r="ABO20"/>
+      <c r="ABP20"/>
+      <c r="ABQ20"/>
+      <c r="ABR20"/>
+      <c r="ABS20"/>
+      <c r="ABT20"/>
+      <c r="ABU20"/>
+      <c r="ABV20"/>
+      <c r="ABW20"/>
+      <c r="ABX20"/>
+      <c r="ABY20"/>
+      <c r="ABZ20"/>
+      <c r="ACA20"/>
+      <c r="ACB20"/>
+      <c r="ACC20"/>
+      <c r="ACD20"/>
+      <c r="ACE20"/>
+      <c r="ACF20"/>
+      <c r="ACG20"/>
+      <c r="ACH20"/>
+      <c r="ACI20"/>
+      <c r="ACJ20"/>
+      <c r="ACK20"/>
+      <c r="ACL20"/>
+      <c r="ACM20"/>
+      <c r="ACN20"/>
+      <c r="ACO20"/>
+      <c r="ACP20"/>
+      <c r="ACQ20"/>
+      <c r="ACR20"/>
+      <c r="ACS20"/>
+      <c r="ACT20"/>
+      <c r="ACU20"/>
+      <c r="ACV20"/>
+      <c r="ACW20"/>
+      <c r="ACX20"/>
+      <c r="ACY20"/>
+      <c r="ACZ20"/>
+      <c r="ADA20"/>
+      <c r="ADB20"/>
+      <c r="ADC20"/>
+      <c r="ADD20"/>
+      <c r="ADE20"/>
+      <c r="ADF20"/>
+      <c r="ADG20"/>
+      <c r="ADH20"/>
+      <c r="ADI20"/>
+      <c r="ADJ20"/>
+      <c r="ADK20"/>
+      <c r="ADL20"/>
+      <c r="ADM20"/>
+      <c r="ADN20"/>
+      <c r="ADO20"/>
+      <c r="ADP20"/>
+      <c r="ADQ20"/>
+      <c r="ADR20"/>
+      <c r="ADS20"/>
+      <c r="ADT20"/>
+      <c r="ADU20"/>
+      <c r="ADV20"/>
+      <c r="ADW20"/>
+      <c r="ADX20"/>
+      <c r="ADY20"/>
+      <c r="ADZ20"/>
+      <c r="AEA20"/>
+      <c r="AEB20"/>
+      <c r="AEC20"/>
+      <c r="AED20"/>
+      <c r="AEE20"/>
+      <c r="AEF20"/>
+      <c r="AEG20"/>
+      <c r="AEH20"/>
+      <c r="AEI20"/>
+      <c r="AEJ20"/>
+      <c r="AEK20"/>
+      <c r="AEL20"/>
+      <c r="AEM20"/>
+      <c r="AEN20"/>
+      <c r="AEO20"/>
+      <c r="AEP20"/>
+      <c r="AEQ20"/>
+      <c r="AER20"/>
+      <c r="AES20"/>
+      <c r="AET20"/>
+      <c r="AEU20"/>
+      <c r="AEV20"/>
+      <c r="AEW20"/>
+      <c r="AEX20"/>
+      <c r="AEY20"/>
+      <c r="AEZ20"/>
+      <c r="AFA20"/>
+      <c r="AFB20"/>
+      <c r="AFC20"/>
+      <c r="AFD20"/>
+      <c r="AFE20"/>
+      <c r="AFF20"/>
+      <c r="AFG20"/>
+      <c r="AFH20"/>
+      <c r="AFI20"/>
+      <c r="AFJ20"/>
+      <c r="AFK20"/>
+      <c r="AFL20"/>
+      <c r="AFM20"/>
+      <c r="AFN20"/>
+      <c r="AFO20"/>
+      <c r="AFP20"/>
+      <c r="AFQ20"/>
+      <c r="AFR20"/>
+      <c r="AFS20"/>
+      <c r="AFT20"/>
+      <c r="AFU20"/>
+      <c r="AFV20"/>
+      <c r="AFW20"/>
+      <c r="AFX20"/>
+      <c r="AFY20"/>
+      <c r="AFZ20"/>
+      <c r="AGA20"/>
+      <c r="AGB20"/>
+      <c r="AGC20"/>
+      <c r="AGD20"/>
+      <c r="AGE20"/>
+      <c r="AGF20"/>
+      <c r="AGG20"/>
+      <c r="AGH20"/>
+      <c r="AGI20"/>
+      <c r="AGJ20"/>
+      <c r="AGK20"/>
+      <c r="AGL20"/>
+      <c r="AGM20"/>
+      <c r="AGN20"/>
+      <c r="AGO20"/>
+      <c r="AGP20"/>
+      <c r="AGQ20"/>
+      <c r="AGR20"/>
+      <c r="AGS20"/>
+      <c r="AGT20"/>
+      <c r="AGU20"/>
+      <c r="AGV20"/>
+      <c r="AGW20"/>
+      <c r="AGX20"/>
+      <c r="AGY20"/>
+      <c r="AGZ20"/>
+      <c r="AHA20"/>
+      <c r="AHB20"/>
+      <c r="AHC20"/>
+      <c r="AHD20"/>
+      <c r="AHE20"/>
+      <c r="AHF20"/>
+      <c r="AHG20"/>
+      <c r="AHH20"/>
+      <c r="AHI20"/>
+      <c r="AHJ20"/>
+      <c r="AHK20"/>
+      <c r="AHL20"/>
+      <c r="AHM20"/>
+      <c r="AHN20"/>
+      <c r="AHO20"/>
+      <c r="AHP20"/>
+      <c r="AHQ20"/>
+      <c r="AHR20"/>
+      <c r="AHS20"/>
+      <c r="AHT20"/>
+      <c r="AHU20"/>
+      <c r="AHV20"/>
+      <c r="AHW20"/>
+      <c r="AHX20"/>
+      <c r="AHY20"/>
+      <c r="AHZ20"/>
+      <c r="AIA20"/>
+      <c r="AIB20"/>
+      <c r="AIC20"/>
+      <c r="AID20"/>
+      <c r="AIE20"/>
+      <c r="AIF20"/>
+      <c r="AIG20"/>
+      <c r="AIH20"/>
+      <c r="AII20"/>
+      <c r="AIJ20"/>
+      <c r="AIK20"/>
+      <c r="AIL20"/>
+      <c r="AIM20"/>
+      <c r="AIN20"/>
+      <c r="AIO20"/>
+      <c r="AIP20"/>
+      <c r="AIQ20"/>
+      <c r="AIR20"/>
+      <c r="AIS20"/>
+      <c r="AIT20"/>
+      <c r="AIU20"/>
+      <c r="AIV20"/>
+      <c r="AIW20"/>
+      <c r="AIX20"/>
+      <c r="AIY20"/>
+      <c r="AIZ20"/>
+      <c r="AJA20"/>
+      <c r="AJB20"/>
+      <c r="AJC20"/>
+      <c r="AJD20"/>
+      <c r="AJE20"/>
+      <c r="AJF20"/>
+      <c r="AJG20"/>
+      <c r="AJH20"/>
+      <c r="AJI20"/>
+      <c r="AJJ20"/>
+      <c r="AJK20"/>
+      <c r="AJL20"/>
+      <c r="AJM20"/>
+      <c r="AJN20"/>
+      <c r="AJO20"/>
+      <c r="AJP20"/>
+      <c r="AJQ20"/>
+      <c r="AJR20"/>
+      <c r="AJS20"/>
+      <c r="AJT20"/>
+      <c r="AJU20"/>
+      <c r="AJV20"/>
+      <c r="AJW20"/>
+      <c r="AJX20"/>
+      <c r="AJY20"/>
+      <c r="AJZ20"/>
+      <c r="AKA20"/>
+      <c r="AKB20"/>
+      <c r="AKC20"/>
+      <c r="AKD20"/>
+      <c r="AKE20"/>
+      <c r="AKF20"/>
+      <c r="AKG20"/>
+      <c r="AKH20"/>
+      <c r="AKI20"/>
+      <c r="AKJ20"/>
+      <c r="AKK20"/>
+      <c r="AKL20"/>
+      <c r="AKM20"/>
+      <c r="AKN20"/>
+      <c r="AKO20"/>
+      <c r="AKP20"/>
+      <c r="AKQ20"/>
+      <c r="AKR20"/>
+      <c r="AKS20"/>
+      <c r="AKT20"/>
+      <c r="AKU20"/>
+      <c r="AKV20"/>
+      <c r="AKW20"/>
+      <c r="AKX20"/>
+      <c r="AKY20"/>
+      <c r="AKZ20"/>
+      <c r="ALA20"/>
+      <c r="ALB20"/>
+      <c r="ALC20"/>
+      <c r="ALD20"/>
+      <c r="ALE20"/>
+      <c r="ALF20"/>
+      <c r="ALG20"/>
+      <c r="ALH20"/>
+      <c r="ALI20"/>
+      <c r="ALJ20"/>
+      <c r="ALK20"/>
+      <c r="ALL20"/>
+      <c r="ALM20"/>
+      <c r="ALN20"/>
+      <c r="ALO20"/>
+      <c r="ALP20"/>
+      <c r="ALQ20"/>
+      <c r="ALR20"/>
+      <c r="ALS20"/>
+      <c r="ALT20"/>
+      <c r="ALU20"/>
+      <c r="ALV20"/>
+      <c r="ALW20"/>
+      <c r="ALX20"/>
+      <c r="ALY20"/>
+      <c r="ALZ20"/>
+      <c r="AMA20"/>
+      <c r="AMB20"/>
+      <c r="AMC20"/>
+      <c r="AMD20"/>
+      <c r="AME20"/>
+      <c r="AMF20"/>
+      <c r="AMG20"/>
+      <c r="AMH20"/>
+      <c r="AMI20"/>
+      <c r="AMJ20"/>
+      <c r="AMK20"/>
+    </row>
+    <row r="21" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="67"/>
-    </row>
-    <row r="21" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="67" t="s">
+      <c r="B21" s="78"/>
+    </row>
+    <row r="22" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="78" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="67"/>
-    </row>
-    <row r="22" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="67" t="s">
+      <c r="B22" s="78"/>
+    </row>
+    <row r="23" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="78" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="67"/>
-    </row>
-    <row r="23" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="19"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="5"/>
-      <c r="W23" s="5"/>
-      <c r="X23" s="5"/>
-      <c r="Y23" s="5"/>
-      <c r="Z23" s="5"/>
-      <c r="AA23" s="5"/>
-      <c r="AB23" s="5"/>
-      <c r="AC23" s="5"/>
-      <c r="AD23" s="5"/>
-      <c r="AE23" s="5"/>
-      <c r="AF23" s="5"/>
-      <c r="AG23" s="5"/>
-      <c r="AH23" s="5"/>
-      <c r="AI23" s="5"/>
-      <c r="AJ23" s="5"/>
-      <c r="AK23" s="5"/>
-      <c r="AL23" s="5"/>
-      <c r="AM23" s="5"/>
-      <c r="AN23" s="5"/>
-      <c r="AO23" s="5"/>
-      <c r="AP23" s="5"/>
-      <c r="AQ23" s="5"/>
-      <c r="AR23" s="5"/>
-      <c r="AS23" s="5"/>
-      <c r="AT23" s="5"/>
-      <c r="AU23" s="5"/>
-      <c r="AV23" s="5"/>
-      <c r="AW23" s="5"/>
-      <c r="AX23" s="5"/>
-      <c r="AY23" s="5"/>
-      <c r="AZ23" s="5"/>
-      <c r="BA23" s="5"/>
-      <c r="BB23" s="5"/>
-      <c r="BC23" s="5"/>
-      <c r="BD23" s="5"/>
-      <c r="BE23" s="5"/>
-      <c r="BF23" s="5"/>
-      <c r="BG23" s="5"/>
-      <c r="BH23" s="5"/>
-      <c r="BI23" s="5"/>
-      <c r="BJ23" s="5"/>
-      <c r="BK23" s="5"/>
-      <c r="BL23" s="5"/>
-      <c r="BM23" s="5"/>
-      <c r="BN23" s="5"/>
-      <c r="BO23" s="5"/>
-      <c r="BP23" s="5"/>
-      <c r="BQ23" s="5"/>
-      <c r="BR23" s="5"/>
-      <c r="BS23" s="5"/>
-      <c r="BT23" s="5"/>
-      <c r="BU23" s="5"/>
-      <c r="BV23" s="5"/>
-      <c r="BW23" s="5"/>
-      <c r="BX23" s="5"/>
-      <c r="BY23" s="5"/>
-      <c r="BZ23" s="5"/>
-      <c r="CA23" s="5"/>
-      <c r="CB23" s="5"/>
-      <c r="CC23" s="5"/>
-      <c r="CD23" s="5"/>
-      <c r="CE23" s="5"/>
-      <c r="CF23" s="5"/>
-      <c r="CG23" s="5"/>
-      <c r="CH23" s="5"/>
-      <c r="CI23" s="5"/>
-      <c r="CJ23" s="5"/>
-      <c r="CK23" s="5"/>
-      <c r="CL23" s="5"/>
-      <c r="CM23" s="5"/>
-      <c r="CN23" s="5"/>
-      <c r="CO23" s="5"/>
-      <c r="CP23" s="5"/>
-      <c r="CQ23" s="5"/>
-      <c r="CR23" s="5"/>
-      <c r="CS23" s="5"/>
-      <c r="CT23" s="5"/>
-      <c r="CU23" s="5"/>
-      <c r="CV23" s="5"/>
-      <c r="CW23" s="5"/>
-      <c r="CX23" s="5"/>
-      <c r="CY23" s="5"/>
-      <c r="CZ23" s="5"/>
-      <c r="DA23" s="5"/>
-      <c r="DB23" s="5"/>
-      <c r="DC23" s="5"/>
-      <c r="DD23" s="5"/>
-      <c r="DE23" s="5"/>
-      <c r="DF23" s="5"/>
-      <c r="DG23" s="5"/>
-      <c r="DH23" s="5"/>
-      <c r="DI23" s="5"/>
-      <c r="DJ23" s="5"/>
-      <c r="DK23" s="5"/>
-      <c r="DL23" s="5"/>
-      <c r="DM23" s="5"/>
-      <c r="DN23" s="5"/>
-      <c r="DO23" s="5"/>
-      <c r="DP23" s="5"/>
-      <c r="DQ23" s="5"/>
-      <c r="DR23" s="5"/>
-      <c r="DS23" s="5"/>
-      <c r="DT23" s="5"/>
-      <c r="DU23" s="5"/>
-      <c r="DV23" s="5"/>
-      <c r="DW23" s="5"/>
-      <c r="DX23" s="5"/>
-      <c r="DY23" s="5"/>
-      <c r="DZ23" s="5"/>
-      <c r="EA23" s="5"/>
-      <c r="EB23" s="5"/>
-      <c r="EC23" s="5"/>
-      <c r="ED23" s="5"/>
-      <c r="EE23" s="5"/>
-      <c r="EF23" s="5"/>
-      <c r="EG23" s="5"/>
-      <c r="EH23" s="5"/>
-      <c r="EI23" s="5"/>
-      <c r="EJ23" s="5"/>
-      <c r="EK23" s="5"/>
-      <c r="EL23" s="5"/>
-      <c r="EM23" s="5"/>
-      <c r="EN23" s="5"/>
-      <c r="EO23" s="5"/>
-      <c r="EP23" s="5"/>
-      <c r="EQ23" s="5"/>
-      <c r="ER23" s="5"/>
-      <c r="ES23" s="5"/>
-      <c r="ET23" s="5"/>
-      <c r="EU23" s="5"/>
-      <c r="EV23" s="5"/>
-      <c r="EW23" s="5"/>
-      <c r="EX23" s="5"/>
-      <c r="EY23" s="5"/>
-      <c r="EZ23" s="5"/>
-      <c r="FA23" s="5"/>
-      <c r="FB23" s="5"/>
-      <c r="FC23" s="5"/>
-      <c r="FD23" s="5"/>
-      <c r="FE23" s="5"/>
-      <c r="FF23" s="5"/>
-      <c r="FG23" s="5"/>
-      <c r="FH23" s="5"/>
-      <c r="FI23" s="5"/>
-      <c r="FJ23" s="5"/>
-      <c r="FK23" s="5"/>
-      <c r="FL23" s="5"/>
-      <c r="FM23" s="5"/>
-      <c r="FN23" s="5"/>
-      <c r="FO23" s="5"/>
-      <c r="FP23" s="5"/>
-      <c r="FQ23" s="5"/>
-      <c r="FR23" s="5"/>
-      <c r="FS23" s="5"/>
-      <c r="FT23" s="5"/>
-      <c r="FU23" s="5"/>
-      <c r="FV23" s="5"/>
-      <c r="FW23" s="5"/>
-      <c r="FX23" s="5"/>
-      <c r="FY23" s="5"/>
-      <c r="FZ23" s="5"/>
-      <c r="GA23" s="5"/>
-      <c r="GB23" s="5"/>
-      <c r="GC23" s="5"/>
-      <c r="GD23" s="5"/>
-      <c r="GE23" s="5"/>
-      <c r="GF23" s="5"/>
-      <c r="GG23" s="5"/>
-      <c r="GH23" s="5"/>
-      <c r="GI23" s="5"/>
-      <c r="GJ23" s="5"/>
-      <c r="GK23" s="5"/>
-      <c r="GL23" s="5"/>
-      <c r="GM23" s="5"/>
-      <c r="GN23" s="5"/>
-      <c r="GO23" s="5"/>
-      <c r="GP23" s="5"/>
-      <c r="GQ23" s="5"/>
-      <c r="GR23" s="5"/>
-      <c r="GS23" s="5"/>
-      <c r="GT23" s="5"/>
-      <c r="GU23" s="5"/>
-      <c r="GV23" s="5"/>
-      <c r="GW23" s="5"/>
-      <c r="GX23" s="5"/>
-      <c r="GY23" s="5"/>
-      <c r="GZ23" s="5"/>
-      <c r="HA23" s="5"/>
-      <c r="HB23" s="5"/>
-      <c r="HC23" s="5"/>
-      <c r="HD23" s="5"/>
-      <c r="HE23" s="5"/>
-      <c r="HF23" s="5"/>
-      <c r="HG23" s="5"/>
-      <c r="HH23" s="5"/>
-      <c r="HI23" s="5"/>
-      <c r="HJ23" s="5"/>
-      <c r="HK23" s="5"/>
-      <c r="HL23" s="5"/>
-      <c r="HM23" s="5"/>
-      <c r="HN23" s="5"/>
-      <c r="HO23" s="5"/>
-      <c r="HP23" s="5"/>
-      <c r="HQ23" s="5"/>
-      <c r="HR23" s="5"/>
-      <c r="HS23" s="5"/>
-      <c r="HT23" s="5"/>
-      <c r="HU23" s="5"/>
-      <c r="HV23" s="5"/>
-      <c r="HW23" s="5"/>
-      <c r="HX23" s="5"/>
-      <c r="HY23" s="5"/>
-      <c r="HZ23" s="5"/>
-      <c r="IA23" s="5"/>
-      <c r="IB23" s="5"/>
-      <c r="IC23" s="5"/>
-      <c r="ID23" s="5"/>
-      <c r="IE23" s="5"/>
-      <c r="IF23" s="5"/>
-      <c r="IG23" s="5"/>
-      <c r="IH23" s="5"/>
-      <c r="II23" s="5"/>
-      <c r="IJ23" s="5"/>
-      <c r="IK23" s="5"/>
-      <c r="IL23" s="5"/>
-      <c r="IM23" s="5"/>
-      <c r="IN23" s="5"/>
-      <c r="IO23" s="5"/>
-      <c r="IP23" s="5"/>
-      <c r="IQ23" s="5"/>
-      <c r="IR23" s="5"/>
-      <c r="IS23" s="5"/>
-      <c r="IT23" s="5"/>
-      <c r="IU23" s="5"/>
-      <c r="IV23" s="5"/>
-      <c r="IW23" s="5"/>
-      <c r="IX23" s="5"/>
-      <c r="IY23" s="5"/>
-      <c r="IZ23" s="5"/>
-      <c r="JA23" s="5"/>
-      <c r="JB23" s="5"/>
-      <c r="JC23" s="5"/>
-      <c r="JD23" s="5"/>
-      <c r="JE23" s="5"/>
-      <c r="JF23" s="5"/>
-      <c r="JG23" s="5"/>
-      <c r="JH23" s="5"/>
-      <c r="JI23" s="5"/>
-      <c r="JJ23" s="5"/>
-      <c r="JK23" s="5"/>
-      <c r="JL23" s="5"/>
-      <c r="JM23" s="5"/>
-      <c r="JN23" s="5"/>
-      <c r="JO23" s="5"/>
-      <c r="JP23" s="5"/>
-      <c r="JQ23" s="5"/>
-      <c r="JR23" s="5"/>
-      <c r="JS23" s="5"/>
-      <c r="JT23" s="5"/>
-      <c r="JU23" s="5"/>
-      <c r="JV23" s="5"/>
-      <c r="JW23" s="5"/>
-      <c r="JX23" s="5"/>
-      <c r="JY23" s="5"/>
-      <c r="JZ23" s="5"/>
-      <c r="KA23" s="5"/>
-      <c r="KB23" s="5"/>
-      <c r="KC23" s="5"/>
-      <c r="KD23" s="5"/>
-      <c r="KE23" s="5"/>
-      <c r="KF23" s="5"/>
-      <c r="KG23" s="5"/>
-      <c r="KH23" s="5"/>
-      <c r="KI23" s="5"/>
-      <c r="KJ23" s="5"/>
-      <c r="KK23" s="5"/>
-      <c r="KL23" s="5"/>
-      <c r="KM23" s="5"/>
-      <c r="KN23" s="5"/>
-      <c r="KO23" s="5"/>
-      <c r="KP23" s="5"/>
-      <c r="KQ23" s="5"/>
-      <c r="KR23" s="5"/>
-      <c r="KS23" s="5"/>
-      <c r="KT23" s="5"/>
-      <c r="KU23" s="5"/>
-      <c r="KV23" s="5"/>
-      <c r="KW23" s="5"/>
-      <c r="KX23" s="5"/>
-      <c r="KY23" s="5"/>
-      <c r="KZ23" s="5"/>
-      <c r="LA23" s="5"/>
-      <c r="LB23" s="5"/>
-      <c r="LC23" s="5"/>
-      <c r="LD23" s="5"/>
-      <c r="LE23" s="5"/>
-      <c r="LF23" s="5"/>
-      <c r="LG23" s="5"/>
-      <c r="LH23" s="5"/>
-      <c r="LI23" s="5"/>
-      <c r="LJ23" s="5"/>
-      <c r="LK23" s="5"/>
-      <c r="LL23" s="5"/>
-      <c r="LM23" s="5"/>
-      <c r="LN23" s="5"/>
-      <c r="LO23" s="5"/>
-      <c r="LP23" s="5"/>
-      <c r="LQ23" s="5"/>
-      <c r="LR23" s="5"/>
-      <c r="LS23" s="5"/>
-      <c r="LT23" s="5"/>
-      <c r="LU23" s="5"/>
-      <c r="LV23" s="5"/>
-      <c r="LW23" s="5"/>
-      <c r="LX23" s="5"/>
-      <c r="LY23" s="5"/>
-      <c r="LZ23" s="5"/>
-      <c r="MA23" s="5"/>
-      <c r="MB23" s="5"/>
-      <c r="MC23" s="5"/>
-      <c r="MD23" s="5"/>
-      <c r="ME23" s="5"/>
-      <c r="MF23" s="5"/>
-      <c r="MG23" s="5"/>
-      <c r="MH23" s="5"/>
-      <c r="MI23" s="5"/>
-      <c r="MJ23" s="5"/>
-      <c r="MK23" s="5"/>
-      <c r="ML23" s="5"/>
-      <c r="MM23" s="5"/>
-      <c r="MN23" s="5"/>
-      <c r="MO23" s="5"/>
-      <c r="MP23" s="5"/>
-      <c r="MQ23" s="5"/>
-      <c r="MR23" s="5"/>
-      <c r="MS23" s="5"/>
-      <c r="MT23" s="5"/>
-      <c r="MU23" s="5"/>
-      <c r="MV23" s="5"/>
-      <c r="MW23" s="5"/>
-      <c r="MX23" s="5"/>
-      <c r="MY23" s="5"/>
-      <c r="MZ23" s="5"/>
-      <c r="NA23" s="5"/>
-      <c r="NB23" s="5"/>
-      <c r="NC23" s="5"/>
-      <c r="ND23" s="5"/>
-      <c r="NE23" s="5"/>
-      <c r="NF23" s="5"/>
-      <c r="NG23" s="5"/>
-      <c r="NH23" s="5"/>
-      <c r="NI23" s="5"/>
-      <c r="NJ23" s="5"/>
-      <c r="NK23" s="5"/>
-      <c r="NL23" s="5"/>
-      <c r="NM23" s="5"/>
-      <c r="NN23" s="5"/>
-      <c r="NO23" s="5"/>
-      <c r="NP23" s="5"/>
-      <c r="NQ23" s="5"/>
-      <c r="NR23" s="5"/>
-      <c r="NS23" s="5"/>
-      <c r="NT23" s="5"/>
-      <c r="NU23" s="5"/>
-      <c r="NV23" s="5"/>
-      <c r="NW23" s="5"/>
-      <c r="NX23" s="5"/>
-      <c r="NY23" s="5"/>
-      <c r="NZ23" s="5"/>
-      <c r="OA23" s="5"/>
-      <c r="OB23" s="5"/>
-      <c r="OC23" s="5"/>
-      <c r="OD23" s="5"/>
-      <c r="OE23" s="5"/>
-      <c r="OF23" s="5"/>
-      <c r="OG23" s="5"/>
-      <c r="OH23" s="5"/>
-      <c r="OI23" s="5"/>
-      <c r="OJ23" s="5"/>
-      <c r="OK23" s="5"/>
-      <c r="OL23" s="5"/>
-      <c r="OM23" s="5"/>
-      <c r="ON23" s="5"/>
-      <c r="OO23" s="5"/>
-      <c r="OP23" s="5"/>
-      <c r="OQ23" s="5"/>
-      <c r="OR23" s="5"/>
-      <c r="OS23" s="5"/>
-      <c r="OT23" s="5"/>
-      <c r="OU23" s="5"/>
-      <c r="OV23" s="5"/>
-      <c r="OW23" s="5"/>
-      <c r="OX23" s="5"/>
-      <c r="OY23" s="5"/>
-      <c r="OZ23" s="5"/>
-      <c r="PA23" s="5"/>
-      <c r="PB23" s="5"/>
-      <c r="PC23" s="5"/>
-      <c r="PD23" s="5"/>
-      <c r="PE23" s="5"/>
-      <c r="PF23" s="5"/>
-      <c r="PG23" s="5"/>
-      <c r="PH23" s="5"/>
-      <c r="PI23" s="5"/>
-      <c r="PJ23" s="5"/>
-      <c r="PK23" s="5"/>
-      <c r="PL23" s="5"/>
-      <c r="PM23" s="5"/>
-      <c r="PN23" s="5"/>
-      <c r="PO23" s="5"/>
-      <c r="PP23" s="5"/>
-      <c r="PQ23" s="5"/>
-      <c r="PR23" s="5"/>
-      <c r="PS23" s="5"/>
-      <c r="PT23" s="5"/>
-      <c r="PU23" s="5"/>
-      <c r="PV23" s="5"/>
-      <c r="PW23" s="5"/>
-      <c r="PX23" s="5"/>
-      <c r="PY23" s="5"/>
-      <c r="PZ23" s="5"/>
-      <c r="QA23" s="5"/>
-      <c r="QB23" s="5"/>
-      <c r="QC23" s="5"/>
-      <c r="QD23" s="5"/>
-      <c r="QE23" s="5"/>
-      <c r="QF23" s="5"/>
-      <c r="QG23" s="5"/>
-      <c r="QH23" s="5"/>
-      <c r="QI23" s="5"/>
-      <c r="QJ23" s="5"/>
-      <c r="QK23" s="5"/>
-      <c r="QL23" s="5"/>
-      <c r="QM23" s="5"/>
-      <c r="QN23" s="5"/>
-      <c r="QO23" s="5"/>
-      <c r="QP23" s="5"/>
-      <c r="QQ23" s="5"/>
-      <c r="QR23" s="5"/>
-      <c r="QS23" s="5"/>
-      <c r="QT23" s="5"/>
-      <c r="QU23" s="5"/>
-      <c r="QV23" s="5"/>
-      <c r="QW23" s="5"/>
-      <c r="QX23" s="5"/>
-      <c r="QY23" s="5"/>
-      <c r="QZ23" s="5"/>
-      <c r="RA23" s="5"/>
-      <c r="RB23" s="5"/>
-      <c r="RC23" s="5"/>
-      <c r="RD23" s="5"/>
-      <c r="RE23" s="5"/>
-      <c r="RF23" s="5"/>
-      <c r="RG23" s="5"/>
-      <c r="RH23" s="5"/>
-      <c r="RI23" s="5"/>
-      <c r="RJ23" s="5"/>
-      <c r="RK23" s="5"/>
-      <c r="RL23" s="5"/>
-      <c r="RM23" s="5"/>
-      <c r="RN23" s="5"/>
-      <c r="RO23" s="5"/>
-      <c r="RP23" s="5"/>
-      <c r="RQ23" s="5"/>
-      <c r="RR23" s="5"/>
-      <c r="RS23" s="5"/>
-      <c r="RT23" s="5"/>
-      <c r="RU23" s="5"/>
-      <c r="RV23" s="5"/>
-      <c r="RW23" s="5"/>
-      <c r="RX23" s="5"/>
-      <c r="RY23" s="5"/>
-      <c r="RZ23" s="5"/>
-      <c r="SA23" s="5"/>
-      <c r="SB23" s="5"/>
-      <c r="SC23" s="5"/>
-      <c r="SD23" s="5"/>
-      <c r="SE23" s="5"/>
-      <c r="SF23" s="5"/>
-      <c r="SG23" s="5"/>
-      <c r="SH23" s="5"/>
-      <c r="SI23" s="5"/>
-      <c r="SJ23" s="5"/>
-      <c r="SK23" s="5"/>
-      <c r="SL23" s="5"/>
-      <c r="SM23" s="5"/>
-      <c r="SN23" s="5"/>
-      <c r="SO23" s="5"/>
-      <c r="SP23" s="5"/>
-      <c r="SQ23" s="5"/>
-      <c r="SR23" s="5"/>
-      <c r="SS23" s="5"/>
-      <c r="ST23" s="5"/>
-      <c r="SU23" s="5"/>
-      <c r="SV23" s="5"/>
-      <c r="SW23" s="5"/>
-      <c r="SX23" s="5"/>
-      <c r="SY23" s="5"/>
-      <c r="SZ23" s="5"/>
-      <c r="TA23" s="5"/>
-      <c r="TB23" s="5"/>
-      <c r="TC23" s="5"/>
-      <c r="TD23" s="5"/>
-      <c r="TE23" s="5"/>
-      <c r="TF23" s="5"/>
-      <c r="TG23" s="5"/>
-      <c r="TH23" s="5"/>
-      <c r="TI23" s="5"/>
-      <c r="TJ23" s="5"/>
-      <c r="TK23" s="5"/>
-      <c r="TL23" s="5"/>
-      <c r="TM23" s="5"/>
-      <c r="TN23" s="5"/>
-      <c r="TO23" s="5"/>
-      <c r="TP23" s="5"/>
-      <c r="TQ23" s="5"/>
-      <c r="TR23" s="5"/>
-      <c r="TS23" s="5"/>
-      <c r="TT23" s="5"/>
-      <c r="TU23" s="5"/>
-      <c r="TV23" s="5"/>
-      <c r="TW23" s="5"/>
-      <c r="TX23" s="5"/>
-      <c r="TY23" s="5"/>
-      <c r="TZ23" s="5"/>
-      <c r="UA23" s="5"/>
-      <c r="UB23" s="5"/>
-      <c r="UC23" s="5"/>
-      <c r="UD23" s="5"/>
-      <c r="UE23" s="5"/>
-      <c r="UF23" s="5"/>
-      <c r="UG23" s="5"/>
-      <c r="UH23" s="5"/>
-      <c r="UI23" s="5"/>
-      <c r="UJ23" s="5"/>
-      <c r="UK23" s="5"/>
-      <c r="UL23" s="5"/>
-      <c r="UM23" s="5"/>
-      <c r="UN23" s="5"/>
-      <c r="UO23" s="5"/>
-      <c r="UP23" s="5"/>
-      <c r="UQ23" s="5"/>
-      <c r="UR23" s="5"/>
-      <c r="US23" s="5"/>
-      <c r="UT23" s="5"/>
-      <c r="UU23" s="5"/>
-      <c r="UV23" s="5"/>
-      <c r="UW23" s="5"/>
-      <c r="UX23" s="5"/>
-      <c r="UY23" s="5"/>
-      <c r="UZ23" s="5"/>
-      <c r="VA23" s="5"/>
-      <c r="VB23" s="5"/>
-      <c r="VC23" s="5"/>
-      <c r="VD23" s="5"/>
-      <c r="VE23" s="5"/>
-      <c r="VF23" s="5"/>
-      <c r="VG23" s="5"/>
-      <c r="VH23" s="5"/>
-      <c r="VI23" s="5"/>
-      <c r="VJ23" s="5"/>
-      <c r="VK23" s="5"/>
-      <c r="VL23" s="5"/>
-      <c r="VM23" s="5"/>
-      <c r="VN23" s="5"/>
-      <c r="VO23" s="5"/>
-      <c r="VP23" s="5"/>
-      <c r="VQ23" s="5"/>
-      <c r="VR23" s="5"/>
-      <c r="VS23" s="5"/>
-      <c r="VT23" s="5"/>
-      <c r="VU23" s="5"/>
-      <c r="VV23" s="5"/>
-      <c r="VW23" s="5"/>
-      <c r="VX23" s="5"/>
-      <c r="VY23" s="5"/>
-      <c r="VZ23" s="5"/>
-      <c r="WA23" s="5"/>
-      <c r="WB23" s="5"/>
-      <c r="WC23" s="5"/>
-      <c r="WD23" s="5"/>
-      <c r="WE23" s="5"/>
-      <c r="WF23" s="5"/>
-      <c r="WG23" s="5"/>
-      <c r="WH23" s="5"/>
-      <c r="WI23" s="5"/>
-      <c r="WJ23" s="5"/>
-      <c r="WK23" s="5"/>
-      <c r="WL23" s="5"/>
-      <c r="WM23" s="5"/>
-      <c r="WN23" s="5"/>
-      <c r="WO23" s="5"/>
-      <c r="WP23" s="5"/>
-      <c r="WQ23" s="5"/>
-      <c r="WR23" s="5"/>
-      <c r="WS23" s="5"/>
-      <c r="WT23" s="5"/>
-      <c r="WU23" s="5"/>
-      <c r="WV23" s="5"/>
-      <c r="WW23" s="5"/>
-      <c r="WX23" s="5"/>
-      <c r="WY23" s="5"/>
-      <c r="WZ23" s="5"/>
-      <c r="XA23" s="5"/>
-      <c r="XB23" s="5"/>
-      <c r="XC23" s="5"/>
-      <c r="XD23" s="5"/>
-      <c r="XE23" s="5"/>
-      <c r="XF23" s="5"/>
-      <c r="XG23" s="5"/>
-      <c r="XH23" s="5"/>
-      <c r="XI23" s="5"/>
-      <c r="XJ23" s="5"/>
-      <c r="XK23" s="5"/>
-      <c r="XL23" s="5"/>
-      <c r="XM23" s="5"/>
-      <c r="XN23" s="5"/>
-      <c r="XO23" s="5"/>
-      <c r="XP23" s="5"/>
-      <c r="XQ23" s="5"/>
-      <c r="XR23" s="5"/>
-      <c r="XS23" s="5"/>
-      <c r="XT23" s="5"/>
-      <c r="XU23" s="5"/>
-      <c r="XV23" s="5"/>
-      <c r="XW23" s="5"/>
-      <c r="XX23" s="5"/>
-      <c r="XY23" s="5"/>
-      <c r="XZ23" s="5"/>
-      <c r="YA23" s="5"/>
-      <c r="YB23" s="5"/>
-      <c r="YC23" s="5"/>
-      <c r="YD23" s="5"/>
-      <c r="YE23" s="5"/>
-      <c r="YF23" s="5"/>
-      <c r="YG23" s="5"/>
-      <c r="YH23" s="5"/>
-      <c r="YI23" s="5"/>
-      <c r="YJ23" s="5"/>
-      <c r="YK23" s="5"/>
-      <c r="YL23" s="5"/>
-      <c r="YM23" s="5"/>
-      <c r="YN23" s="5"/>
-      <c r="YO23" s="5"/>
-      <c r="YP23" s="5"/>
-      <c r="YQ23" s="5"/>
-      <c r="YR23" s="5"/>
-      <c r="YS23" s="5"/>
-      <c r="YT23" s="5"/>
-      <c r="YU23" s="5"/>
-      <c r="YV23" s="5"/>
-      <c r="YW23" s="5"/>
-      <c r="YX23" s="5"/>
-      <c r="YY23" s="5"/>
-      <c r="YZ23" s="5"/>
-      <c r="ZA23" s="5"/>
-      <c r="ZB23" s="5"/>
-      <c r="ZC23" s="5"/>
-      <c r="ZD23" s="5"/>
-      <c r="ZE23" s="5"/>
-      <c r="ZF23" s="5"/>
-      <c r="ZG23" s="5"/>
-      <c r="ZH23" s="5"/>
-      <c r="ZI23" s="5"/>
-      <c r="ZJ23" s="5"/>
-      <c r="ZK23" s="5"/>
-      <c r="ZL23" s="5"/>
-      <c r="ZM23" s="5"/>
-      <c r="ZN23" s="5"/>
-      <c r="ZO23" s="5"/>
-      <c r="ZP23" s="5"/>
-      <c r="ZQ23" s="5"/>
-      <c r="ZR23" s="5"/>
-      <c r="ZS23" s="5"/>
-      <c r="ZT23" s="5"/>
-      <c r="ZU23" s="5"/>
-      <c r="ZV23" s="5"/>
-      <c r="ZW23" s="5"/>
-      <c r="ZX23" s="5"/>
-      <c r="ZY23" s="5"/>
-      <c r="ZZ23" s="5"/>
-      <c r="AAA23" s="5"/>
-      <c r="AAB23" s="5"/>
-      <c r="AAC23" s="5"/>
-      <c r="AAD23" s="5"/>
-      <c r="AAE23" s="5"/>
-      <c r="AAF23" s="5"/>
-      <c r="AAG23" s="5"/>
-      <c r="AAH23" s="5"/>
-      <c r="AAI23" s="5"/>
-      <c r="AAJ23" s="5"/>
-      <c r="AAK23" s="5"/>
-      <c r="AAL23" s="5"/>
-      <c r="AAM23" s="5"/>
-      <c r="AAN23" s="5"/>
-      <c r="AAO23" s="5"/>
-      <c r="AAP23" s="5"/>
-      <c r="AAQ23" s="5"/>
-      <c r="AAR23" s="5"/>
-      <c r="AAS23" s="5"/>
-      <c r="AAT23" s="5"/>
-      <c r="AAU23" s="5"/>
-      <c r="AAV23" s="5"/>
-      <c r="AAW23" s="5"/>
-      <c r="AAX23" s="5"/>
-      <c r="AAY23" s="5"/>
-      <c r="AAZ23" s="5"/>
-      <c r="ABA23" s="5"/>
-      <c r="ABB23" s="5"/>
-      <c r="ABC23" s="5"/>
-      <c r="ABD23" s="5"/>
-      <c r="ABE23" s="5"/>
-      <c r="ABF23" s="5"/>
-      <c r="ABG23" s="5"/>
-      <c r="ABH23" s="5"/>
-      <c r="ABI23" s="5"/>
-      <c r="ABJ23" s="5"/>
-      <c r="ABK23" s="5"/>
-      <c r="ABL23" s="5"/>
-      <c r="ABM23" s="5"/>
-      <c r="ABN23" s="5"/>
-      <c r="ABO23" s="5"/>
-      <c r="ABP23" s="5"/>
-      <c r="ABQ23" s="5"/>
-      <c r="ABR23" s="5"/>
-      <c r="ABS23" s="5"/>
-      <c r="ABT23" s="5"/>
-      <c r="ABU23" s="5"/>
-      <c r="ABV23" s="5"/>
-      <c r="ABW23" s="5"/>
-      <c r="ABX23" s="5"/>
-      <c r="ABY23" s="5"/>
-      <c r="ABZ23" s="5"/>
-      <c r="ACA23" s="5"/>
-      <c r="ACB23" s="5"/>
-      <c r="ACC23" s="5"/>
-      <c r="ACD23" s="5"/>
-      <c r="ACE23" s="5"/>
-      <c r="ACF23" s="5"/>
-      <c r="ACG23" s="5"/>
-      <c r="ACH23" s="5"/>
-      <c r="ACI23" s="5"/>
-      <c r="ACJ23" s="5"/>
-      <c r="ACK23" s="5"/>
-      <c r="ACL23" s="5"/>
-      <c r="ACM23" s="5"/>
-      <c r="ACN23" s="5"/>
-      <c r="ACO23" s="5"/>
-      <c r="ACP23" s="5"/>
-      <c r="ACQ23" s="5"/>
-      <c r="ACR23" s="5"/>
-      <c r="ACS23" s="5"/>
-      <c r="ACT23" s="5"/>
-      <c r="ACU23" s="5"/>
-      <c r="ACV23" s="5"/>
-      <c r="ACW23" s="5"/>
-      <c r="ACX23" s="5"/>
-      <c r="ACY23" s="5"/>
-      <c r="ACZ23" s="5"/>
-      <c r="ADA23" s="5"/>
-      <c r="ADB23" s="5"/>
-      <c r="ADC23" s="5"/>
-      <c r="ADD23" s="5"/>
-      <c r="ADE23" s="5"/>
-      <c r="ADF23" s="5"/>
-      <c r="ADG23" s="5"/>
-      <c r="ADH23" s="5"/>
-      <c r="ADI23" s="5"/>
-      <c r="ADJ23" s="5"/>
-      <c r="ADK23" s="5"/>
-      <c r="ADL23" s="5"/>
-      <c r="ADM23" s="5"/>
-      <c r="ADN23" s="5"/>
-      <c r="ADO23" s="5"/>
-      <c r="ADP23" s="5"/>
-      <c r="ADQ23" s="5"/>
-      <c r="ADR23" s="5"/>
-      <c r="ADS23" s="5"/>
-      <c r="ADT23" s="5"/>
-      <c r="ADU23" s="5"/>
-      <c r="ADV23" s="5"/>
-      <c r="ADW23" s="5"/>
-      <c r="ADX23" s="5"/>
-      <c r="ADY23" s="5"/>
-      <c r="ADZ23" s="5"/>
-      <c r="AEA23" s="5"/>
-      <c r="AEB23" s="5"/>
-      <c r="AEC23" s="5"/>
-      <c r="AED23" s="5"/>
-      <c r="AEE23" s="5"/>
-      <c r="AEF23" s="5"/>
-      <c r="AEG23" s="5"/>
-      <c r="AEH23" s="5"/>
-      <c r="AEI23" s="5"/>
-      <c r="AEJ23" s="5"/>
-      <c r="AEK23" s="5"/>
-      <c r="AEL23" s="5"/>
-      <c r="AEM23" s="5"/>
-      <c r="AEN23" s="5"/>
-      <c r="AEO23" s="5"/>
-      <c r="AEP23" s="5"/>
-      <c r="AEQ23" s="5"/>
-      <c r="AER23" s="5"/>
-      <c r="AES23" s="5"/>
-      <c r="AET23" s="5"/>
-      <c r="AEU23" s="5"/>
-      <c r="AEV23" s="5"/>
-      <c r="AEW23" s="5"/>
-      <c r="AEX23" s="5"/>
-      <c r="AEY23" s="5"/>
-      <c r="AEZ23" s="5"/>
-      <c r="AFA23" s="5"/>
-      <c r="AFB23" s="5"/>
-      <c r="AFC23" s="5"/>
-      <c r="AFD23" s="5"/>
-      <c r="AFE23" s="5"/>
-      <c r="AFF23" s="5"/>
-      <c r="AFG23" s="5"/>
-      <c r="AFH23" s="5"/>
-      <c r="AFI23" s="5"/>
-      <c r="AFJ23" s="5"/>
-      <c r="AFK23" s="5"/>
-      <c r="AFL23" s="5"/>
-      <c r="AFM23" s="5"/>
-      <c r="AFN23" s="5"/>
-      <c r="AFO23" s="5"/>
-      <c r="AFP23" s="5"/>
-      <c r="AFQ23" s="5"/>
-      <c r="AFR23" s="5"/>
-      <c r="AFS23" s="5"/>
-      <c r="AFT23" s="5"/>
-      <c r="AFU23" s="5"/>
-      <c r="AFV23" s="5"/>
-      <c r="AFW23" s="5"/>
-      <c r="AFX23" s="5"/>
-      <c r="AFY23" s="5"/>
-      <c r="AFZ23" s="5"/>
-      <c r="AGA23" s="5"/>
-      <c r="AGB23" s="5"/>
-      <c r="AGC23" s="5"/>
-      <c r="AGD23" s="5"/>
-      <c r="AGE23" s="5"/>
-      <c r="AGF23" s="5"/>
-      <c r="AGG23" s="5"/>
-      <c r="AGH23" s="5"/>
-      <c r="AGI23" s="5"/>
-      <c r="AGJ23" s="5"/>
-      <c r="AGK23" s="5"/>
-      <c r="AGL23" s="5"/>
-      <c r="AGM23" s="5"/>
-      <c r="AGN23" s="5"/>
-      <c r="AGO23" s="5"/>
-      <c r="AGP23" s="5"/>
-      <c r="AGQ23" s="5"/>
-      <c r="AGR23" s="5"/>
-      <c r="AGS23" s="5"/>
-      <c r="AGT23" s="5"/>
-      <c r="AGU23" s="5"/>
-      <c r="AGV23" s="5"/>
-      <c r="AGW23" s="5"/>
-      <c r="AGX23" s="5"/>
-      <c r="AGY23" s="5"/>
-      <c r="AGZ23" s="5"/>
-      <c r="AHA23" s="5"/>
-      <c r="AHB23" s="5"/>
-      <c r="AHC23" s="5"/>
-      <c r="AHD23" s="5"/>
-      <c r="AHE23" s="5"/>
-      <c r="AHF23" s="5"/>
-      <c r="AHG23" s="5"/>
-      <c r="AHH23" s="5"/>
-      <c r="AHI23" s="5"/>
-      <c r="AHJ23" s="5"/>
-      <c r="AHK23" s="5"/>
-      <c r="AHL23" s="5"/>
-      <c r="AHM23" s="5"/>
-      <c r="AHN23" s="5"/>
-      <c r="AHO23" s="5"/>
-      <c r="AHP23" s="5"/>
-      <c r="AHQ23" s="5"/>
-      <c r="AHR23" s="5"/>
-      <c r="AHS23" s="5"/>
-      <c r="AHT23" s="5"/>
-      <c r="AHU23" s="5"/>
-      <c r="AHV23" s="5"/>
-      <c r="AHW23" s="5"/>
-      <c r="AHX23" s="5"/>
-      <c r="AHY23" s="5"/>
-      <c r="AHZ23" s="5"/>
-      <c r="AIA23" s="5"/>
-      <c r="AIB23" s="5"/>
-      <c r="AIC23" s="5"/>
-      <c r="AID23" s="5"/>
-      <c r="AIE23" s="5"/>
-      <c r="AIF23" s="5"/>
-      <c r="AIG23" s="5"/>
-      <c r="AIH23" s="5"/>
-      <c r="AII23" s="5"/>
-      <c r="AIJ23" s="5"/>
-      <c r="AIK23" s="5"/>
-      <c r="AIL23" s="5"/>
-      <c r="AIM23" s="5"/>
-      <c r="AIN23" s="5"/>
-      <c r="AIO23" s="5"/>
-      <c r="AIP23" s="5"/>
-      <c r="AIQ23" s="5"/>
-      <c r="AIR23" s="5"/>
-      <c r="AIS23" s="5"/>
-      <c r="AIT23" s="5"/>
-      <c r="AIU23" s="5"/>
-      <c r="AIV23" s="5"/>
-      <c r="AIW23" s="5"/>
-      <c r="AIX23" s="5"/>
-      <c r="AIY23" s="5"/>
-      <c r="AIZ23" s="5"/>
-      <c r="AJA23" s="5"/>
-      <c r="AJB23" s="5"/>
-      <c r="AJC23" s="5"/>
-      <c r="AJD23" s="5"/>
-      <c r="AJE23" s="5"/>
-      <c r="AJF23" s="5"/>
-      <c r="AJG23" s="5"/>
-      <c r="AJH23" s="5"/>
-      <c r="AJI23" s="5"/>
-      <c r="AJJ23" s="5"/>
-      <c r="AJK23" s="5"/>
-      <c r="AJL23" s="5"/>
-      <c r="AJM23" s="5"/>
-      <c r="AJN23" s="5"/>
-      <c r="AJO23" s="5"/>
-      <c r="AJP23" s="5"/>
-      <c r="AJQ23" s="5"/>
-      <c r="AJR23" s="5"/>
-      <c r="AJS23" s="5"/>
-      <c r="AJT23" s="5"/>
-      <c r="AJU23" s="5"/>
-      <c r="AJV23" s="5"/>
-      <c r="AJW23" s="5"/>
-      <c r="AJX23" s="5"/>
-      <c r="AJY23" s="5"/>
-      <c r="AJZ23" s="5"/>
-      <c r="AKA23" s="5"/>
-      <c r="AKB23" s="5"/>
-      <c r="AKC23" s="5"/>
-      <c r="AKD23" s="5"/>
-      <c r="AKE23" s="5"/>
-      <c r="AKF23" s="5"/>
-      <c r="AKG23" s="5"/>
-      <c r="AKH23" s="5"/>
-      <c r="AKI23" s="5"/>
-      <c r="AKJ23" s="5"/>
-      <c r="AKK23" s="5"/>
-      <c r="AKL23" s="5"/>
-      <c r="AKM23" s="5"/>
-      <c r="AKN23" s="5"/>
-      <c r="AKO23" s="5"/>
-      <c r="AKP23" s="5"/>
-      <c r="AKQ23" s="5"/>
-      <c r="AKR23" s="5"/>
-      <c r="AKS23" s="5"/>
-      <c r="AKT23" s="5"/>
-      <c r="AKU23" s="5"/>
-      <c r="AKV23" s="5"/>
-      <c r="AKW23" s="5"/>
-      <c r="AKX23" s="5"/>
-      <c r="AKY23" s="5"/>
-      <c r="AKZ23" s="5"/>
-      <c r="ALA23" s="5"/>
-      <c r="ALB23" s="5"/>
-      <c r="ALC23" s="5"/>
-      <c r="ALD23" s="5"/>
-      <c r="ALE23" s="5"/>
-      <c r="ALF23" s="5"/>
-      <c r="ALG23" s="5"/>
-      <c r="ALH23" s="5"/>
-      <c r="ALI23" s="5"/>
-      <c r="ALJ23" s="5"/>
-      <c r="ALK23" s="5"/>
-      <c r="ALL23" s="5"/>
-      <c r="ALM23" s="5"/>
-      <c r="ALN23" s="5"/>
-      <c r="ALO23" s="5"/>
-      <c r="ALP23" s="5"/>
-      <c r="ALQ23" s="5"/>
-      <c r="ALR23" s="5"/>
-      <c r="ALS23" s="5"/>
-      <c r="ALT23" s="5"/>
-      <c r="ALU23" s="5"/>
-      <c r="ALV23" s="5"/>
-      <c r="ALW23" s="5"/>
-      <c r="ALX23" s="5"/>
-      <c r="ALY23" s="5"/>
-      <c r="ALZ23" s="5"/>
-      <c r="AMA23" s="5"/>
-      <c r="AMB23" s="5"/>
-      <c r="AMC23" s="5"/>
-      <c r="AMD23" s="5"/>
-      <c r="AME23" s="5"/>
-      <c r="AMF23" s="5"/>
-      <c r="AMG23" s="5"/>
-      <c r="AMH23" s="5"/>
-      <c r="AMI23" s="5"/>
-      <c r="AMJ23" s="5"/>
-      <c r="AMK23" s="5"/>
+      <c r="B23" s="78"/>
+    </row>
+    <row r="24" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+      <c r="S24" s="5"/>
+      <c r="T24" s="5"/>
+      <c r="U24" s="5"/>
+      <c r="V24" s="5"/>
+      <c r="W24" s="5"/>
+      <c r="X24" s="5"/>
+      <c r="Y24" s="5"/>
+      <c r="Z24" s="5"/>
+      <c r="AA24" s="5"/>
+      <c r="AB24" s="5"/>
+      <c r="AC24" s="5"/>
+      <c r="AD24" s="5"/>
+      <c r="AE24" s="5"/>
+      <c r="AF24" s="5"/>
+      <c r="AG24" s="5"/>
+      <c r="AH24" s="5"/>
+      <c r="AI24" s="5"/>
+      <c r="AJ24" s="5"/>
+      <c r="AK24" s="5"/>
+      <c r="AL24" s="5"/>
+      <c r="AM24" s="5"/>
+      <c r="AN24" s="5"/>
+      <c r="AO24" s="5"/>
+      <c r="AP24" s="5"/>
+      <c r="AQ24" s="5"/>
+      <c r="AR24" s="5"/>
+      <c r="AS24" s="5"/>
+      <c r="AT24" s="5"/>
+      <c r="AU24" s="5"/>
+      <c r="AV24" s="5"/>
+      <c r="AW24" s="5"/>
+      <c r="AX24" s="5"/>
+      <c r="AY24" s="5"/>
+      <c r="AZ24" s="5"/>
+      <c r="BA24" s="5"/>
+      <c r="BB24" s="5"/>
+      <c r="BC24" s="5"/>
+      <c r="BD24" s="5"/>
+      <c r="BE24" s="5"/>
+      <c r="BF24" s="5"/>
+      <c r="BG24" s="5"/>
+      <c r="BH24" s="5"/>
+      <c r="BI24" s="5"/>
+      <c r="BJ24" s="5"/>
+      <c r="BK24" s="5"/>
+      <c r="BL24" s="5"/>
+      <c r="BM24" s="5"/>
+      <c r="BN24" s="5"/>
+      <c r="BO24" s="5"/>
+      <c r="BP24" s="5"/>
+      <c r="BQ24" s="5"/>
+      <c r="BR24" s="5"/>
+      <c r="BS24" s="5"/>
+      <c r="BT24" s="5"/>
+      <c r="BU24" s="5"/>
+      <c r="BV24" s="5"/>
+      <c r="BW24" s="5"/>
+      <c r="BX24" s="5"/>
+      <c r="BY24" s="5"/>
+      <c r="BZ24" s="5"/>
+      <c r="CA24" s="5"/>
+      <c r="CB24" s="5"/>
+      <c r="CC24" s="5"/>
+      <c r="CD24" s="5"/>
+      <c r="CE24" s="5"/>
+      <c r="CF24" s="5"/>
+      <c r="CG24" s="5"/>
+      <c r="CH24" s="5"/>
+      <c r="CI24" s="5"/>
+      <c r="CJ24" s="5"/>
+      <c r="CK24" s="5"/>
+      <c r="CL24" s="5"/>
+      <c r="CM24" s="5"/>
+      <c r="CN24" s="5"/>
+      <c r="CO24" s="5"/>
+      <c r="CP24" s="5"/>
+      <c r="CQ24" s="5"/>
+      <c r="CR24" s="5"/>
+      <c r="CS24" s="5"/>
+      <c r="CT24" s="5"/>
+      <c r="CU24" s="5"/>
+      <c r="CV24" s="5"/>
+      <c r="CW24" s="5"/>
+      <c r="CX24" s="5"/>
+      <c r="CY24" s="5"/>
+      <c r="CZ24" s="5"/>
+      <c r="DA24" s="5"/>
+      <c r="DB24" s="5"/>
+      <c r="DC24" s="5"/>
+      <c r="DD24" s="5"/>
+      <c r="DE24" s="5"/>
+      <c r="DF24" s="5"/>
+      <c r="DG24" s="5"/>
+      <c r="DH24" s="5"/>
+      <c r="DI24" s="5"/>
+      <c r="DJ24" s="5"/>
+      <c r="DK24" s="5"/>
+      <c r="DL24" s="5"/>
+      <c r="DM24" s="5"/>
+      <c r="DN24" s="5"/>
+      <c r="DO24" s="5"/>
+      <c r="DP24" s="5"/>
+      <c r="DQ24" s="5"/>
+      <c r="DR24" s="5"/>
+      <c r="DS24" s="5"/>
+      <c r="DT24" s="5"/>
+      <c r="DU24" s="5"/>
+      <c r="DV24" s="5"/>
+      <c r="DW24" s="5"/>
+      <c r="DX24" s="5"/>
+      <c r="DY24" s="5"/>
+      <c r="DZ24" s="5"/>
+      <c r="EA24" s="5"/>
+      <c r="EB24" s="5"/>
+      <c r="EC24" s="5"/>
+      <c r="ED24" s="5"/>
+      <c r="EE24" s="5"/>
+      <c r="EF24" s="5"/>
+      <c r="EG24" s="5"/>
+      <c r="EH24" s="5"/>
+      <c r="EI24" s="5"/>
+      <c r="EJ24" s="5"/>
+      <c r="EK24" s="5"/>
+      <c r="EL24" s="5"/>
+      <c r="EM24" s="5"/>
+      <c r="EN24" s="5"/>
+      <c r="EO24" s="5"/>
+      <c r="EP24" s="5"/>
+      <c r="EQ24" s="5"/>
+      <c r="ER24" s="5"/>
+      <c r="ES24" s="5"/>
+      <c r="ET24" s="5"/>
+      <c r="EU24" s="5"/>
+      <c r="EV24" s="5"/>
+      <c r="EW24" s="5"/>
+      <c r="EX24" s="5"/>
+      <c r="EY24" s="5"/>
+      <c r="EZ24" s="5"/>
+      <c r="FA24" s="5"/>
+      <c r="FB24" s="5"/>
+      <c r="FC24" s="5"/>
+      <c r="FD24" s="5"/>
+      <c r="FE24" s="5"/>
+      <c r="FF24" s="5"/>
+      <c r="FG24" s="5"/>
+      <c r="FH24" s="5"/>
+      <c r="FI24" s="5"/>
+      <c r="FJ24" s="5"/>
+      <c r="FK24" s="5"/>
+      <c r="FL24" s="5"/>
+      <c r="FM24" s="5"/>
+      <c r="FN24" s="5"/>
+      <c r="FO24" s="5"/>
+      <c r="FP24" s="5"/>
+      <c r="FQ24" s="5"/>
+      <c r="FR24" s="5"/>
+      <c r="FS24" s="5"/>
+      <c r="FT24" s="5"/>
+      <c r="FU24" s="5"/>
+      <c r="FV24" s="5"/>
+      <c r="FW24" s="5"/>
+      <c r="FX24" s="5"/>
+      <c r="FY24" s="5"/>
+      <c r="FZ24" s="5"/>
+      <c r="GA24" s="5"/>
+      <c r="GB24" s="5"/>
+      <c r="GC24" s="5"/>
+      <c r="GD24" s="5"/>
+      <c r="GE24" s="5"/>
+      <c r="GF24" s="5"/>
+      <c r="GG24" s="5"/>
+      <c r="GH24" s="5"/>
+      <c r="GI24" s="5"/>
+      <c r="GJ24" s="5"/>
+      <c r="GK24" s="5"/>
+      <c r="GL24" s="5"/>
+      <c r="GM24" s="5"/>
+      <c r="GN24" s="5"/>
+      <c r="GO24" s="5"/>
+      <c r="GP24" s="5"/>
+      <c r="GQ24" s="5"/>
+      <c r="GR24" s="5"/>
+      <c r="GS24" s="5"/>
+      <c r="GT24" s="5"/>
+      <c r="GU24" s="5"/>
+      <c r="GV24" s="5"/>
+      <c r="GW24" s="5"/>
+      <c r="GX24" s="5"/>
+      <c r="GY24" s="5"/>
+      <c r="GZ24" s="5"/>
+      <c r="HA24" s="5"/>
+      <c r="HB24" s="5"/>
+      <c r="HC24" s="5"/>
+      <c r="HD24" s="5"/>
+      <c r="HE24" s="5"/>
+      <c r="HF24" s="5"/>
+      <c r="HG24" s="5"/>
+      <c r="HH24" s="5"/>
+      <c r="HI24" s="5"/>
+      <c r="HJ24" s="5"/>
+      <c r="HK24" s="5"/>
+      <c r="HL24" s="5"/>
+      <c r="HM24" s="5"/>
+      <c r="HN24" s="5"/>
+      <c r="HO24" s="5"/>
+      <c r="HP24" s="5"/>
+      <c r="HQ24" s="5"/>
+      <c r="HR24" s="5"/>
+      <c r="HS24" s="5"/>
+      <c r="HT24" s="5"/>
+      <c r="HU24" s="5"/>
+      <c r="HV24" s="5"/>
+      <c r="HW24" s="5"/>
+      <c r="HX24" s="5"/>
+      <c r="HY24" s="5"/>
+      <c r="HZ24" s="5"/>
+      <c r="IA24" s="5"/>
+      <c r="IB24" s="5"/>
+      <c r="IC24" s="5"/>
+      <c r="ID24" s="5"/>
+      <c r="IE24" s="5"/>
+      <c r="IF24" s="5"/>
+      <c r="IG24" s="5"/>
+      <c r="IH24" s="5"/>
+      <c r="II24" s="5"/>
+      <c r="IJ24" s="5"/>
+      <c r="IK24" s="5"/>
+      <c r="IL24" s="5"/>
+      <c r="IM24" s="5"/>
+      <c r="IN24" s="5"/>
+      <c r="IO24" s="5"/>
+      <c r="IP24" s="5"/>
+      <c r="IQ24" s="5"/>
+      <c r="IR24" s="5"/>
+      <c r="IS24" s="5"/>
+      <c r="IT24" s="5"/>
+      <c r="IU24" s="5"/>
+      <c r="IV24" s="5"/>
+      <c r="IW24" s="5"/>
+      <c r="IX24" s="5"/>
+      <c r="IY24" s="5"/>
+      <c r="IZ24" s="5"/>
+      <c r="JA24" s="5"/>
+      <c r="JB24" s="5"/>
+      <c r="JC24" s="5"/>
+      <c r="JD24" s="5"/>
+      <c r="JE24" s="5"/>
+      <c r="JF24" s="5"/>
+      <c r="JG24" s="5"/>
+      <c r="JH24" s="5"/>
+      <c r="JI24" s="5"/>
+      <c r="JJ24" s="5"/>
+      <c r="JK24" s="5"/>
+      <c r="JL24" s="5"/>
+      <c r="JM24" s="5"/>
+      <c r="JN24" s="5"/>
+      <c r="JO24" s="5"/>
+      <c r="JP24" s="5"/>
+      <c r="JQ24" s="5"/>
+      <c r="JR24" s="5"/>
+      <c r="JS24" s="5"/>
+      <c r="JT24" s="5"/>
+      <c r="JU24" s="5"/>
+      <c r="JV24" s="5"/>
+      <c r="JW24" s="5"/>
+      <c r="JX24" s="5"/>
+      <c r="JY24" s="5"/>
+      <c r="JZ24" s="5"/>
+      <c r="KA24" s="5"/>
+      <c r="KB24" s="5"/>
+      <c r="KC24" s="5"/>
+      <c r="KD24" s="5"/>
+      <c r="KE24" s="5"/>
+      <c r="KF24" s="5"/>
+      <c r="KG24" s="5"/>
+      <c r="KH24" s="5"/>
+      <c r="KI24" s="5"/>
+      <c r="KJ24" s="5"/>
+      <c r="KK24" s="5"/>
+      <c r="KL24" s="5"/>
+      <c r="KM24" s="5"/>
+      <c r="KN24" s="5"/>
+      <c r="KO24" s="5"/>
+      <c r="KP24" s="5"/>
+      <c r="KQ24" s="5"/>
+      <c r="KR24" s="5"/>
+      <c r="KS24" s="5"/>
+      <c r="KT24" s="5"/>
+      <c r="KU24" s="5"/>
+      <c r="KV24" s="5"/>
+      <c r="KW24" s="5"/>
+      <c r="KX24" s="5"/>
+      <c r="KY24" s="5"/>
+      <c r="KZ24" s="5"/>
+      <c r="LA24" s="5"/>
+      <c r="LB24" s="5"/>
+      <c r="LC24" s="5"/>
+      <c r="LD24" s="5"/>
+      <c r="LE24" s="5"/>
+      <c r="LF24" s="5"/>
+      <c r="LG24" s="5"/>
+      <c r="LH24" s="5"/>
+      <c r="LI24" s="5"/>
+      <c r="LJ24" s="5"/>
+      <c r="LK24" s="5"/>
+      <c r="LL24" s="5"/>
+      <c r="LM24" s="5"/>
+      <c r="LN24" s="5"/>
+      <c r="LO24" s="5"/>
+      <c r="LP24" s="5"/>
+      <c r="LQ24" s="5"/>
+      <c r="LR24" s="5"/>
+      <c r="LS24" s="5"/>
+      <c r="LT24" s="5"/>
+      <c r="LU24" s="5"/>
+      <c r="LV24" s="5"/>
+      <c r="LW24" s="5"/>
+      <c r="LX24" s="5"/>
+      <c r="LY24" s="5"/>
+      <c r="LZ24" s="5"/>
+      <c r="MA24" s="5"/>
+      <c r="MB24" s="5"/>
+      <c r="MC24" s="5"/>
+      <c r="MD24" s="5"/>
+      <c r="ME24" s="5"/>
+      <c r="MF24" s="5"/>
+      <c r="MG24" s="5"/>
+      <c r="MH24" s="5"/>
+      <c r="MI24" s="5"/>
+      <c r="MJ24" s="5"/>
+      <c r="MK24" s="5"/>
+      <c r="ML24" s="5"/>
+      <c r="MM24" s="5"/>
+      <c r="MN24" s="5"/>
+      <c r="MO24" s="5"/>
+      <c r="MP24" s="5"/>
+      <c r="MQ24" s="5"/>
+      <c r="MR24" s="5"/>
+      <c r="MS24" s="5"/>
+      <c r="MT24" s="5"/>
+      <c r="MU24" s="5"/>
+      <c r="MV24" s="5"/>
+      <c r="MW24" s="5"/>
+      <c r="MX24" s="5"/>
+      <c r="MY24" s="5"/>
+      <c r="MZ24" s="5"/>
+      <c r="NA24" s="5"/>
+      <c r="NB24" s="5"/>
+      <c r="NC24" s="5"/>
+      <c r="ND24" s="5"/>
+      <c r="NE24" s="5"/>
+      <c r="NF24" s="5"/>
+      <c r="NG24" s="5"/>
+      <c r="NH24" s="5"/>
+      <c r="NI24" s="5"/>
+      <c r="NJ24" s="5"/>
+      <c r="NK24" s="5"/>
+      <c r="NL24" s="5"/>
+      <c r="NM24" s="5"/>
+      <c r="NN24" s="5"/>
+      <c r="NO24" s="5"/>
+      <c r="NP24" s="5"/>
+      <c r="NQ24" s="5"/>
+      <c r="NR24" s="5"/>
+      <c r="NS24" s="5"/>
+      <c r="NT24" s="5"/>
+      <c r="NU24" s="5"/>
+      <c r="NV24" s="5"/>
+      <c r="NW24" s="5"/>
+      <c r="NX24" s="5"/>
+      <c r="NY24" s="5"/>
+      <c r="NZ24" s="5"/>
+      <c r="OA24" s="5"/>
+      <c r="OB24" s="5"/>
+      <c r="OC24" s="5"/>
+      <c r="OD24" s="5"/>
+      <c r="OE24" s="5"/>
+      <c r="OF24" s="5"/>
+      <c r="OG24" s="5"/>
+      <c r="OH24" s="5"/>
+      <c r="OI24" s="5"/>
+      <c r="OJ24" s="5"/>
+      <c r="OK24" s="5"/>
+      <c r="OL24" s="5"/>
+      <c r="OM24" s="5"/>
+      <c r="ON24" s="5"/>
+      <c r="OO24" s="5"/>
+      <c r="OP24" s="5"/>
+      <c r="OQ24" s="5"/>
+      <c r="OR24" s="5"/>
+      <c r="OS24" s="5"/>
+      <c r="OT24" s="5"/>
+      <c r="OU24" s="5"/>
+      <c r="OV24" s="5"/>
+      <c r="OW24" s="5"/>
+      <c r="OX24" s="5"/>
+      <c r="OY24" s="5"/>
+      <c r="OZ24" s="5"/>
+      <c r="PA24" s="5"/>
+      <c r="PB24" s="5"/>
+      <c r="PC24" s="5"/>
+      <c r="PD24" s="5"/>
+      <c r="PE24" s="5"/>
+      <c r="PF24" s="5"/>
+      <c r="PG24" s="5"/>
+      <c r="PH24" s="5"/>
+      <c r="PI24" s="5"/>
+      <c r="PJ24" s="5"/>
+      <c r="PK24" s="5"/>
+      <c r="PL24" s="5"/>
+      <c r="PM24" s="5"/>
+      <c r="PN24" s="5"/>
+      <c r="PO24" s="5"/>
+      <c r="PP24" s="5"/>
+      <c r="PQ24" s="5"/>
+      <c r="PR24" s="5"/>
+      <c r="PS24" s="5"/>
+      <c r="PT24" s="5"/>
+      <c r="PU24" s="5"/>
+      <c r="PV24" s="5"/>
+      <c r="PW24" s="5"/>
+      <c r="PX24" s="5"/>
+      <c r="PY24" s="5"/>
+      <c r="PZ24" s="5"/>
+      <c r="QA24" s="5"/>
+      <c r="QB24" s="5"/>
+      <c r="QC24" s="5"/>
+      <c r="QD24" s="5"/>
+      <c r="QE24" s="5"/>
+      <c r="QF24" s="5"/>
+      <c r="QG24" s="5"/>
+      <c r="QH24" s="5"/>
+      <c r="QI24" s="5"/>
+      <c r="QJ24" s="5"/>
+      <c r="QK24" s="5"/>
+      <c r="QL24" s="5"/>
+      <c r="QM24" s="5"/>
+      <c r="QN24" s="5"/>
+      <c r="QO24" s="5"/>
+      <c r="QP24" s="5"/>
+      <c r="QQ24" s="5"/>
+      <c r="QR24" s="5"/>
+      <c r="QS24" s="5"/>
+      <c r="QT24" s="5"/>
+      <c r="QU24" s="5"/>
+      <c r="QV24" s="5"/>
+      <c r="QW24" s="5"/>
+      <c r="QX24" s="5"/>
+      <c r="QY24" s="5"/>
+      <c r="QZ24" s="5"/>
+      <c r="RA24" s="5"/>
+      <c r="RB24" s="5"/>
+      <c r="RC24" s="5"/>
+      <c r="RD24" s="5"/>
+      <c r="RE24" s="5"/>
+      <c r="RF24" s="5"/>
+      <c r="RG24" s="5"/>
+      <c r="RH24" s="5"/>
+      <c r="RI24" s="5"/>
+      <c r="RJ24" s="5"/>
+      <c r="RK24" s="5"/>
+      <c r="RL24" s="5"/>
+      <c r="RM24" s="5"/>
+      <c r="RN24" s="5"/>
+      <c r="RO24" s="5"/>
+      <c r="RP24" s="5"/>
+      <c r="RQ24" s="5"/>
+      <c r="RR24" s="5"/>
+      <c r="RS24" s="5"/>
+      <c r="RT24" s="5"/>
+      <c r="RU24" s="5"/>
+      <c r="RV24" s="5"/>
+      <c r="RW24" s="5"/>
+      <c r="RX24" s="5"/>
+      <c r="RY24" s="5"/>
+      <c r="RZ24" s="5"/>
+      <c r="SA24" s="5"/>
+      <c r="SB24" s="5"/>
+      <c r="SC24" s="5"/>
+      <c r="SD24" s="5"/>
+      <c r="SE24" s="5"/>
+      <c r="SF24" s="5"/>
+      <c r="SG24" s="5"/>
+      <c r="SH24" s="5"/>
+      <c r="SI24" s="5"/>
+      <c r="SJ24" s="5"/>
+      <c r="SK24" s="5"/>
+      <c r="SL24" s="5"/>
+      <c r="SM24" s="5"/>
+      <c r="SN24" s="5"/>
+      <c r="SO24" s="5"/>
+      <c r="SP24" s="5"/>
+      <c r="SQ24" s="5"/>
+      <c r="SR24" s="5"/>
+      <c r="SS24" s="5"/>
+      <c r="ST24" s="5"/>
+      <c r="SU24" s="5"/>
+      <c r="SV24" s="5"/>
+      <c r="SW24" s="5"/>
+      <c r="SX24" s="5"/>
+      <c r="SY24" s="5"/>
+      <c r="SZ24" s="5"/>
+      <c r="TA24" s="5"/>
+      <c r="TB24" s="5"/>
+      <c r="TC24" s="5"/>
+      <c r="TD24" s="5"/>
+      <c r="TE24" s="5"/>
+      <c r="TF24" s="5"/>
+      <c r="TG24" s="5"/>
+      <c r="TH24" s="5"/>
+      <c r="TI24" s="5"/>
+      <c r="TJ24" s="5"/>
+      <c r="TK24" s="5"/>
+      <c r="TL24" s="5"/>
+      <c r="TM24" s="5"/>
+      <c r="TN24" s="5"/>
+      <c r="TO24" s="5"/>
+      <c r="TP24" s="5"/>
+      <c r="TQ24" s="5"/>
+      <c r="TR24" s="5"/>
+      <c r="TS24" s="5"/>
+      <c r="TT24" s="5"/>
+      <c r="TU24" s="5"/>
+      <c r="TV24" s="5"/>
+      <c r="TW24" s="5"/>
+      <c r="TX24" s="5"/>
+      <c r="TY24" s="5"/>
+      <c r="TZ24" s="5"/>
+      <c r="UA24" s="5"/>
+      <c r="UB24" s="5"/>
+      <c r="UC24" s="5"/>
+      <c r="UD24" s="5"/>
+      <c r="UE24" s="5"/>
+      <c r="UF24" s="5"/>
+      <c r="UG24" s="5"/>
+      <c r="UH24" s="5"/>
+      <c r="UI24" s="5"/>
+      <c r="UJ24" s="5"/>
+      <c r="UK24" s="5"/>
+      <c r="UL24" s="5"/>
+      <c r="UM24" s="5"/>
+      <c r="UN24" s="5"/>
+      <c r="UO24" s="5"/>
+      <c r="UP24" s="5"/>
+      <c r="UQ24" s="5"/>
+      <c r="UR24" s="5"/>
+      <c r="US24" s="5"/>
+      <c r="UT24" s="5"/>
+      <c r="UU24" s="5"/>
+      <c r="UV24" s="5"/>
+      <c r="UW24" s="5"/>
+      <c r="UX24" s="5"/>
+      <c r="UY24" s="5"/>
+      <c r="UZ24" s="5"/>
+      <c r="VA24" s="5"/>
+      <c r="VB24" s="5"/>
+      <c r="VC24" s="5"/>
+      <c r="VD24" s="5"/>
+      <c r="VE24" s="5"/>
+      <c r="VF24" s="5"/>
+      <c r="VG24" s="5"/>
+      <c r="VH24" s="5"/>
+      <c r="VI24" s="5"/>
+      <c r="VJ24" s="5"/>
+      <c r="VK24" s="5"/>
+      <c r="VL24" s="5"/>
+      <c r="VM24" s="5"/>
+      <c r="VN24" s="5"/>
+      <c r="VO24" s="5"/>
+      <c r="VP24" s="5"/>
+      <c r="VQ24" s="5"/>
+      <c r="VR24" s="5"/>
+      <c r="VS24" s="5"/>
+      <c r="VT24" s="5"/>
+      <c r="VU24" s="5"/>
+      <c r="VV24" s="5"/>
+      <c r="VW24" s="5"/>
+      <c r="VX24" s="5"/>
+      <c r="VY24" s="5"/>
+      <c r="VZ24" s="5"/>
+      <c r="WA24" s="5"/>
+      <c r="WB24" s="5"/>
+      <c r="WC24" s="5"/>
+      <c r="WD24" s="5"/>
+      <c r="WE24" s="5"/>
+      <c r="WF24" s="5"/>
+      <c r="WG24" s="5"/>
+      <c r="WH24" s="5"/>
+      <c r="WI24" s="5"/>
+      <c r="WJ24" s="5"/>
+      <c r="WK24" s="5"/>
+      <c r="WL24" s="5"/>
+      <c r="WM24" s="5"/>
+      <c r="WN24" s="5"/>
+      <c r="WO24" s="5"/>
+      <c r="WP24" s="5"/>
+      <c r="WQ24" s="5"/>
+      <c r="WR24" s="5"/>
+      <c r="WS24" s="5"/>
+      <c r="WT24" s="5"/>
+      <c r="WU24" s="5"/>
+      <c r="WV24" s="5"/>
+      <c r="WW24" s="5"/>
+      <c r="WX24" s="5"/>
+      <c r="WY24" s="5"/>
+      <c r="WZ24" s="5"/>
+      <c r="XA24" s="5"/>
+      <c r="XB24" s="5"/>
+      <c r="XC24" s="5"/>
+      <c r="XD24" s="5"/>
+      <c r="XE24" s="5"/>
+      <c r="XF24" s="5"/>
+      <c r="XG24" s="5"/>
+      <c r="XH24" s="5"/>
+      <c r="XI24" s="5"/>
+      <c r="XJ24" s="5"/>
+      <c r="XK24" s="5"/>
+      <c r="XL24" s="5"/>
+      <c r="XM24" s="5"/>
+      <c r="XN24" s="5"/>
+      <c r="XO24" s="5"/>
+      <c r="XP24" s="5"/>
+      <c r="XQ24" s="5"/>
+      <c r="XR24" s="5"/>
+      <c r="XS24" s="5"/>
+      <c r="XT24" s="5"/>
+      <c r="XU24" s="5"/>
+      <c r="XV24" s="5"/>
+      <c r="XW24" s="5"/>
+      <c r="XX24" s="5"/>
+      <c r="XY24" s="5"/>
+      <c r="XZ24" s="5"/>
+      <c r="YA24" s="5"/>
+      <c r="YB24" s="5"/>
+      <c r="YC24" s="5"/>
+      <c r="YD24" s="5"/>
+      <c r="YE24" s="5"/>
+      <c r="YF24" s="5"/>
+      <c r="YG24" s="5"/>
+      <c r="YH24" s="5"/>
+      <c r="YI24" s="5"/>
+      <c r="YJ24" s="5"/>
+      <c r="YK24" s="5"/>
+      <c r="YL24" s="5"/>
+      <c r="YM24" s="5"/>
+      <c r="YN24" s="5"/>
+      <c r="YO24" s="5"/>
+      <c r="YP24" s="5"/>
+      <c r="YQ24" s="5"/>
+      <c r="YR24" s="5"/>
+      <c r="YS24" s="5"/>
+      <c r="YT24" s="5"/>
+      <c r="YU24" s="5"/>
+      <c r="YV24" s="5"/>
+      <c r="YW24" s="5"/>
+      <c r="YX24" s="5"/>
+      <c r="YY24" s="5"/>
+      <c r="YZ24" s="5"/>
+      <c r="ZA24" s="5"/>
+      <c r="ZB24" s="5"/>
+      <c r="ZC24" s="5"/>
+      <c r="ZD24" s="5"/>
+      <c r="ZE24" s="5"/>
+      <c r="ZF24" s="5"/>
+      <c r="ZG24" s="5"/>
+      <c r="ZH24" s="5"/>
+      <c r="ZI24" s="5"/>
+      <c r="ZJ24" s="5"/>
+      <c r="ZK24" s="5"/>
+      <c r="ZL24" s="5"/>
+      <c r="ZM24" s="5"/>
+      <c r="ZN24" s="5"/>
+      <c r="ZO24" s="5"/>
+      <c r="ZP24" s="5"/>
+      <c r="ZQ24" s="5"/>
+      <c r="ZR24" s="5"/>
+      <c r="ZS24" s="5"/>
+      <c r="ZT24" s="5"/>
+      <c r="ZU24" s="5"/>
+      <c r="ZV24" s="5"/>
+      <c r="ZW24" s="5"/>
+      <c r="ZX24" s="5"/>
+      <c r="ZY24" s="5"/>
+      <c r="ZZ24" s="5"/>
+      <c r="AAA24" s="5"/>
+      <c r="AAB24" s="5"/>
+      <c r="AAC24" s="5"/>
+      <c r="AAD24" s="5"/>
+      <c r="AAE24" s="5"/>
+      <c r="AAF24" s="5"/>
+      <c r="AAG24" s="5"/>
+      <c r="AAH24" s="5"/>
+      <c r="AAI24" s="5"/>
+      <c r="AAJ24" s="5"/>
+      <c r="AAK24" s="5"/>
+      <c r="AAL24" s="5"/>
+      <c r="AAM24" s="5"/>
+      <c r="AAN24" s="5"/>
+      <c r="AAO24" s="5"/>
+      <c r="AAP24" s="5"/>
+      <c r="AAQ24" s="5"/>
+      <c r="AAR24" s="5"/>
+      <c r="AAS24" s="5"/>
+      <c r="AAT24" s="5"/>
+      <c r="AAU24" s="5"/>
+      <c r="AAV24" s="5"/>
+      <c r="AAW24" s="5"/>
+      <c r="AAX24" s="5"/>
+      <c r="AAY24" s="5"/>
+      <c r="AAZ24" s="5"/>
+      <c r="ABA24" s="5"/>
+      <c r="ABB24" s="5"/>
+      <c r="ABC24" s="5"/>
+      <c r="ABD24" s="5"/>
+      <c r="ABE24" s="5"/>
+      <c r="ABF24" s="5"/>
+      <c r="ABG24" s="5"/>
+      <c r="ABH24" s="5"/>
+      <c r="ABI24" s="5"/>
+      <c r="ABJ24" s="5"/>
+      <c r="ABK24" s="5"/>
+      <c r="ABL24" s="5"/>
+      <c r="ABM24" s="5"/>
+      <c r="ABN24" s="5"/>
+      <c r="ABO24" s="5"/>
+      <c r="ABP24" s="5"/>
+      <c r="ABQ24" s="5"/>
+      <c r="ABR24" s="5"/>
+      <c r="ABS24" s="5"/>
+      <c r="ABT24" s="5"/>
+      <c r="ABU24" s="5"/>
+      <c r="ABV24" s="5"/>
+      <c r="ABW24" s="5"/>
+      <c r="ABX24" s="5"/>
+      <c r="ABY24" s="5"/>
+      <c r="ABZ24" s="5"/>
+      <c r="ACA24" s="5"/>
+      <c r="ACB24" s="5"/>
+      <c r="ACC24" s="5"/>
+      <c r="ACD24" s="5"/>
+      <c r="ACE24" s="5"/>
+      <c r="ACF24" s="5"/>
+      <c r="ACG24" s="5"/>
+      <c r="ACH24" s="5"/>
+      <c r="ACI24" s="5"/>
+      <c r="ACJ24" s="5"/>
+      <c r="ACK24" s="5"/>
+      <c r="ACL24" s="5"/>
+      <c r="ACM24" s="5"/>
+      <c r="ACN24" s="5"/>
+      <c r="ACO24" s="5"/>
+      <c r="ACP24" s="5"/>
+      <c r="ACQ24" s="5"/>
+      <c r="ACR24" s="5"/>
+      <c r="ACS24" s="5"/>
+      <c r="ACT24" s="5"/>
+      <c r="ACU24" s="5"/>
+      <c r="ACV24" s="5"/>
+      <c r="ACW24" s="5"/>
+      <c r="ACX24" s="5"/>
+      <c r="ACY24" s="5"/>
+      <c r="ACZ24" s="5"/>
+      <c r="ADA24" s="5"/>
+      <c r="ADB24" s="5"/>
+      <c r="ADC24" s="5"/>
+      <c r="ADD24" s="5"/>
+      <c r="ADE24" s="5"/>
+      <c r="ADF24" s="5"/>
+      <c r="ADG24" s="5"/>
+      <c r="ADH24" s="5"/>
+      <c r="ADI24" s="5"/>
+      <c r="ADJ24" s="5"/>
+      <c r="ADK24" s="5"/>
+      <c r="ADL24" s="5"/>
+      <c r="ADM24" s="5"/>
+      <c r="ADN24" s="5"/>
+      <c r="ADO24" s="5"/>
+      <c r="ADP24" s="5"/>
+      <c r="ADQ24" s="5"/>
+      <c r="ADR24" s="5"/>
+      <c r="ADS24" s="5"/>
+      <c r="ADT24" s="5"/>
+      <c r="ADU24" s="5"/>
+      <c r="ADV24" s="5"/>
+      <c r="ADW24" s="5"/>
+      <c r="ADX24" s="5"/>
+      <c r="ADY24" s="5"/>
+      <c r="ADZ24" s="5"/>
+      <c r="AEA24" s="5"/>
+      <c r="AEB24" s="5"/>
+      <c r="AEC24" s="5"/>
+      <c r="AED24" s="5"/>
+      <c r="AEE24" s="5"/>
+      <c r="AEF24" s="5"/>
+      <c r="AEG24" s="5"/>
+      <c r="AEH24" s="5"/>
+      <c r="AEI24" s="5"/>
+      <c r="AEJ24" s="5"/>
+      <c r="AEK24" s="5"/>
+      <c r="AEL24" s="5"/>
+      <c r="AEM24" s="5"/>
+      <c r="AEN24" s="5"/>
+      <c r="AEO24" s="5"/>
+      <c r="AEP24" s="5"/>
+      <c r="AEQ24" s="5"/>
+      <c r="AER24" s="5"/>
+      <c r="AES24" s="5"/>
+      <c r="AET24" s="5"/>
+      <c r="AEU24" s="5"/>
+      <c r="AEV24" s="5"/>
+      <c r="AEW24" s="5"/>
+      <c r="AEX24" s="5"/>
+      <c r="AEY24" s="5"/>
+      <c r="AEZ24" s="5"/>
+      <c r="AFA24" s="5"/>
+      <c r="AFB24" s="5"/>
+      <c r="AFC24" s="5"/>
+      <c r="AFD24" s="5"/>
+      <c r="AFE24" s="5"/>
+      <c r="AFF24" s="5"/>
+      <c r="AFG24" s="5"/>
+      <c r="AFH24" s="5"/>
+      <c r="AFI24" s="5"/>
+      <c r="AFJ24" s="5"/>
+      <c r="AFK24" s="5"/>
+      <c r="AFL24" s="5"/>
+      <c r="AFM24" s="5"/>
+      <c r="AFN24" s="5"/>
+      <c r="AFO24" s="5"/>
+      <c r="AFP24" s="5"/>
+      <c r="AFQ24" s="5"/>
+      <c r="AFR24" s="5"/>
+      <c r="AFS24" s="5"/>
+      <c r="AFT24" s="5"/>
+      <c r="AFU24" s="5"/>
+      <c r="AFV24" s="5"/>
+      <c r="AFW24" s="5"/>
+      <c r="AFX24" s="5"/>
+      <c r="AFY24" s="5"/>
+      <c r="AFZ24" s="5"/>
+      <c r="AGA24" s="5"/>
+      <c r="AGB24" s="5"/>
+      <c r="AGC24" s="5"/>
+      <c r="AGD24" s="5"/>
+      <c r="AGE24" s="5"/>
+      <c r="AGF24" s="5"/>
+      <c r="AGG24" s="5"/>
+      <c r="AGH24" s="5"/>
+      <c r="AGI24" s="5"/>
+      <c r="AGJ24" s="5"/>
+      <c r="AGK24" s="5"/>
+      <c r="AGL24" s="5"/>
+      <c r="AGM24" s="5"/>
+      <c r="AGN24" s="5"/>
+      <c r="AGO24" s="5"/>
+      <c r="AGP24" s="5"/>
+      <c r="AGQ24" s="5"/>
+      <c r="AGR24" s="5"/>
+      <c r="AGS24" s="5"/>
+      <c r="AGT24" s="5"/>
+      <c r="AGU24" s="5"/>
+      <c r="AGV24" s="5"/>
+      <c r="AGW24" s="5"/>
+      <c r="AGX24" s="5"/>
+      <c r="AGY24" s="5"/>
+      <c r="AGZ24" s="5"/>
+      <c r="AHA24" s="5"/>
+      <c r="AHB24" s="5"/>
+      <c r="AHC24" s="5"/>
+      <c r="AHD24" s="5"/>
+      <c r="AHE24" s="5"/>
+      <c r="AHF24" s="5"/>
+      <c r="AHG24" s="5"/>
+      <c r="AHH24" s="5"/>
+      <c r="AHI24" s="5"/>
+      <c r="AHJ24" s="5"/>
+      <c r="AHK24" s="5"/>
+      <c r="AHL24" s="5"/>
+      <c r="AHM24" s="5"/>
+      <c r="AHN24" s="5"/>
+      <c r="AHO24" s="5"/>
+      <c r="AHP24" s="5"/>
+      <c r="AHQ24" s="5"/>
+      <c r="AHR24" s="5"/>
+      <c r="AHS24" s="5"/>
+      <c r="AHT24" s="5"/>
+      <c r="AHU24" s="5"/>
+      <c r="AHV24" s="5"/>
+      <c r="AHW24" s="5"/>
+      <c r="AHX24" s="5"/>
+      <c r="AHY24" s="5"/>
+      <c r="AHZ24" s="5"/>
+      <c r="AIA24" s="5"/>
+      <c r="AIB24" s="5"/>
+      <c r="AIC24" s="5"/>
+      <c r="AID24" s="5"/>
+      <c r="AIE24" s="5"/>
+      <c r="AIF24" s="5"/>
+      <c r="AIG24" s="5"/>
+      <c r="AIH24" s="5"/>
+      <c r="AII24" s="5"/>
+      <c r="AIJ24" s="5"/>
+      <c r="AIK24" s="5"/>
+      <c r="AIL24" s="5"/>
+      <c r="AIM24" s="5"/>
+      <c r="AIN24" s="5"/>
+      <c r="AIO24" s="5"/>
+      <c r="AIP24" s="5"/>
+      <c r="AIQ24" s="5"/>
+      <c r="AIR24" s="5"/>
+      <c r="AIS24" s="5"/>
+      <c r="AIT24" s="5"/>
+      <c r="AIU24" s="5"/>
+      <c r="AIV24" s="5"/>
+      <c r="AIW24" s="5"/>
+      <c r="AIX24" s="5"/>
+      <c r="AIY24" s="5"/>
+      <c r="AIZ24" s="5"/>
+      <c r="AJA24" s="5"/>
+      <c r="AJB24" s="5"/>
+      <c r="AJC24" s="5"/>
+      <c r="AJD24" s="5"/>
+      <c r="AJE24" s="5"/>
+      <c r="AJF24" s="5"/>
+      <c r="AJG24" s="5"/>
+      <c r="AJH24" s="5"/>
+      <c r="AJI24" s="5"/>
+      <c r="AJJ24" s="5"/>
+      <c r="AJK24" s="5"/>
+      <c r="AJL24" s="5"/>
+      <c r="AJM24" s="5"/>
+      <c r="AJN24" s="5"/>
+      <c r="AJO24" s="5"/>
+      <c r="AJP24" s="5"/>
+      <c r="AJQ24" s="5"/>
+      <c r="AJR24" s="5"/>
+      <c r="AJS24" s="5"/>
+      <c r="AJT24" s="5"/>
+      <c r="AJU24" s="5"/>
+      <c r="AJV24" s="5"/>
+      <c r="AJW24" s="5"/>
+      <c r="AJX24" s="5"/>
+      <c r="AJY24" s="5"/>
+      <c r="AJZ24" s="5"/>
+      <c r="AKA24" s="5"/>
+      <c r="AKB24" s="5"/>
+      <c r="AKC24" s="5"/>
+      <c r="AKD24" s="5"/>
+      <c r="AKE24" s="5"/>
+      <c r="AKF24" s="5"/>
+      <c r="AKG24" s="5"/>
+      <c r="AKH24" s="5"/>
+      <c r="AKI24" s="5"/>
+      <c r="AKJ24" s="5"/>
+      <c r="AKK24" s="5"/>
+      <c r="AKL24" s="5"/>
+      <c r="AKM24" s="5"/>
+      <c r="AKN24" s="5"/>
+      <c r="AKO24" s="5"/>
+      <c r="AKP24" s="5"/>
+      <c r="AKQ24" s="5"/>
+      <c r="AKR24" s="5"/>
+      <c r="AKS24" s="5"/>
+      <c r="AKT24" s="5"/>
+      <c r="AKU24" s="5"/>
+      <c r="AKV24" s="5"/>
+      <c r="AKW24" s="5"/>
+      <c r="AKX24" s="5"/>
+      <c r="AKY24" s="5"/>
+      <c r="AKZ24" s="5"/>
+      <c r="ALA24" s="5"/>
+      <c r="ALB24" s="5"/>
+      <c r="ALC24" s="5"/>
+      <c r="ALD24" s="5"/>
+      <c r="ALE24" s="5"/>
+      <c r="ALF24" s="5"/>
+      <c r="ALG24" s="5"/>
+      <c r="ALH24" s="5"/>
+      <c r="ALI24" s="5"/>
+      <c r="ALJ24" s="5"/>
+      <c r="ALK24" s="5"/>
+      <c r="ALL24" s="5"/>
+      <c r="ALM24" s="5"/>
+      <c r="ALN24" s="5"/>
+      <c r="ALO24" s="5"/>
+      <c r="ALP24" s="5"/>
+      <c r="ALQ24" s="5"/>
+      <c r="ALR24" s="5"/>
+      <c r="ALS24" s="5"/>
+      <c r="ALT24" s="5"/>
+      <c r="ALU24" s="5"/>
+      <c r="ALV24" s="5"/>
+      <c r="ALW24" s="5"/>
+      <c r="ALX24" s="5"/>
+      <c r="ALY24" s="5"/>
+      <c r="ALZ24" s="5"/>
+      <c r="AMA24" s="5"/>
+      <c r="AMB24" s="5"/>
+      <c r="AMC24" s="5"/>
+      <c r="AMD24" s="5"/>
+      <c r="AME24" s="5"/>
+      <c r="AMF24" s="5"/>
+      <c r="AMG24" s="5"/>
+      <c r="AMH24" s="5"/>
+      <c r="AMI24" s="5"/>
+      <c r="AMJ24" s="5"/>
+      <c r="AMK24" s="5"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="pKFT46AcXRrznfWpmO12FPPtk8Stkq83/gBYtpLA8HQFC7aZLAdf2WJU+dOj9PZT/L7JPEe68/xM25EHPxktXQ==" saltValue="g+GUymTOlW49z+xbPyQ28w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="HJ0S9SXxH3hc2civzakeUynsclYwZAyDBSkWZhvUUJkGIlw412GwLUnabLTRCCh71tnxAaaHbW//DrRuZOEW6g==" saltValue="3Y6Hg9ERWiGKdmbGDL+Dng==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A19:B19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -9131,6 +9218,46 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="2" max="2" width="153.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection password="E50B" sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -9174,7 +9301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F286"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -9686,7 +9813,7 @@
       <c r="B55" t="s">
         <v>317</v>
       </c>
-      <c r="E55" s="80" t="s">
+      <c r="E55" t="s">
         <v>551</v>
       </c>
     </row>
@@ -10904,6 +11031,46 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03F88BF-42E1-4D49-809C-4FA79F23F636}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="120.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="138" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="72" t="s">
+        <v>559</v>
+      </c>
+      <c r="B1" s="72"/>
+    </row>
+    <row r="2" spans="1:2" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="70" t="s">
+        <v>558</v>
+      </c>
+      <c r="B2" s="70" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="66" x14ac:dyDescent="0.2">
+      <c r="A3" s="68" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" s="69" t="s">
+        <v>556</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11046,7 +11213,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N1048576"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11071,7 +11238,7 @@
       <c r="A1" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="75" t="s">
+      <c r="B1" s="81" t="s">
         <v>59</v>
       </c>
       <c r="C1" s="30" t="s">
@@ -11084,27 +11251,27 @@
     </row>
     <row r="2" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="20"/>
-      <c r="B2" s="75"/>
-      <c r="C2" s="76" t="s">
+      <c r="B2" s="81"/>
+      <c r="C2" s="82" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="82"/>
+      <c r="M2" s="82"/>
+      <c r="N2" s="82"/>
     </row>
     <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="75"/>
+      <c r="B3" s="81"/>
       <c r="C3" s="20" t="s">
         <v>36</v>
       </c>
@@ -11175,7 +11342,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11328,7 +11495,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11460,7 +11627,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11921,7 +12088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AT7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11950,15 +12117,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="83" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="75"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="81"/>
       <c r="D1" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="E1" s="75" t="s">
+      <c r="E1" s="81" t="s">
         <v>59</v>
       </c>
       <c r="F1" s="43" t="s">
@@ -12008,63 +12175,63 @@
     <row r="2" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A2" s="49"/>
       <c r="B2" s="50"/>
-      <c r="C2" s="75"/>
+      <c r="C2" s="81"/>
       <c r="D2" s="51"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="78" t="s">
+      <c r="E2" s="81"/>
+      <c r="F2" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
-      <c r="L2" s="77" t="s">
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="84"/>
+      <c r="L2" s="85" t="s">
         <v>112</v>
       </c>
-      <c r="M2" s="77"/>
-      <c r="N2" s="77"/>
-      <c r="O2" s="77" t="s">
+      <c r="M2" s="85"/>
+      <c r="N2" s="85"/>
+      <c r="O2" s="85" t="s">
         <v>118</v>
       </c>
-      <c r="P2" s="77"/>
-      <c r="Q2" s="77"/>
-      <c r="R2" s="78" t="s">
+      <c r="P2" s="85"/>
+      <c r="Q2" s="85"/>
+      <c r="R2" s="84" t="s">
         <v>125</v>
       </c>
-      <c r="S2" s="78"/>
-      <c r="T2" s="78"/>
-      <c r="U2" s="78"/>
-      <c r="V2" s="78"/>
-      <c r="W2" s="78" t="s">
+      <c r="S2" s="84"/>
+      <c r="T2" s="84"/>
+      <c r="U2" s="84"/>
+      <c r="V2" s="84"/>
+      <c r="W2" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="X2" s="78"/>
-      <c r="Y2" s="78"/>
-      <c r="Z2" s="78" t="s">
+      <c r="X2" s="84"/>
+      <c r="Y2" s="84"/>
+      <c r="Z2" s="84" t="s">
         <v>143</v>
       </c>
-      <c r="AA2" s="78"/>
-      <c r="AB2" s="78"/>
-      <c r="AC2" s="78"/>
-      <c r="AD2" s="78"/>
-      <c r="AE2" s="78"/>
-      <c r="AF2" s="78"/>
-      <c r="AG2" s="78"/>
-      <c r="AH2" s="78"/>
-      <c r="AI2" s="78"/>
-      <c r="AJ2" s="78" t="s">
+      <c r="AA2" s="84"/>
+      <c r="AB2" s="84"/>
+      <c r="AC2" s="84"/>
+      <c r="AD2" s="84"/>
+      <c r="AE2" s="84"/>
+      <c r="AF2" s="84"/>
+      <c r="AG2" s="84"/>
+      <c r="AH2" s="84"/>
+      <c r="AI2" s="84"/>
+      <c r="AJ2" s="84" t="s">
         <v>164</v>
       </c>
-      <c r="AK2" s="78"/>
-      <c r="AL2" s="78"/>
-      <c r="AM2" s="78"/>
-      <c r="AN2" s="78"/>
-      <c r="AO2" s="78"/>
-      <c r="AP2" s="78"/>
-      <c r="AQ2" s="78"/>
-      <c r="AR2" s="78"/>
-      <c r="AS2" s="78"/>
+      <c r="AK2" s="84"/>
+      <c r="AL2" s="84"/>
+      <c r="AM2" s="84"/>
+      <c r="AN2" s="84"/>
+      <c r="AO2" s="84"/>
+      <c r="AP2" s="84"/>
+      <c r="AQ2" s="84"/>
+      <c r="AR2" s="84"/>
+      <c r="AS2" s="84"/>
     </row>
     <row r="3" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A3" s="52" t="s">
@@ -12073,11 +12240,11 @@
       <c r="B3" s="53" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="75"/>
+      <c r="C3" s="81"/>
       <c r="D3" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="75"/>
+      <c r="E3" s="81"/>
       <c r="F3" s="54" t="s">
         <v>101</v>
       </c>
@@ -12220,16 +12387,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="R2:V2"/>
+    <mergeCell ref="W2:Y2"/>
+    <mergeCell ref="Z2:AI2"/>
+    <mergeCell ref="AJ2:AS2"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="E1:E3"/>
     <mergeCell ref="F2:K2"/>
     <mergeCell ref="L2:N2"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="R2:V2"/>
-    <mergeCell ref="W2:Y2"/>
-    <mergeCell ref="Z2:AI2"/>
-    <mergeCell ref="AJ2:AS2"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Metadata and VCF" prompt="These sample names must match those provided in the VCF file(s)" sqref="E1 B4:B1003" xr:uid="{00000000-0002-0000-0700-000000000000}">
@@ -12293,44 +12460,4 @@
     </ext>
   </extLst>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="2" max="2" width="153.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="B3" t="s">
-        <v>195</v>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection password="E50B" sheet="1" objects="1" scenarios="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
EVA-4241 Add checkbox for data acknowledgement statements (#181)
</commit_message>
<xml_diff>
--- a/eva_sub_cli/etc/EVA_Submission_template.xlsx
+++ b/eva_sub_cli/etc/EVA_Submission_template.xlsx
@@ -1,31 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcezard/PycharmProjects/eva-sub-cli/eva_sub_cli/etc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkumar2/PycharmProjects/eva-sub-cli/eva_sub_cli/etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A9AA12-83B5-5F4E-A99B-DAAE6E8CF182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148322AA-EF35-134D-81E1-68607A71F539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLEASE READ FIRST" sheetId="1" r:id="rId1"/>
     <sheet name="Submitter Details" sheetId="2" r:id="rId2"/>
-    <sheet name="Project HELP" sheetId="3" r:id="rId3"/>
-    <sheet name="Project" sheetId="4" r:id="rId4"/>
-    <sheet name="Analysis HELP" sheetId="5" r:id="rId5"/>
-    <sheet name="Analysis" sheetId="6" r:id="rId6"/>
-    <sheet name="Sample HELP" sheetId="7" r:id="rId7"/>
-    <sheet name="Sample" sheetId="8" r:id="rId8"/>
-    <sheet name="Files HELP" sheetId="9" r:id="rId9"/>
-    <sheet name="Files" sheetId="10" r:id="rId10"/>
-    <sheet name="CVs" sheetId="11" r:id="rId11"/>
+    <sheet name="Statements" sheetId="13" r:id="rId3"/>
+    <sheet name="Project HELP" sheetId="3" r:id="rId4"/>
+    <sheet name="Project" sheetId="4" r:id="rId5"/>
+    <sheet name="Analysis HELP" sheetId="5" r:id="rId6"/>
+    <sheet name="Analysis" sheetId="6" r:id="rId7"/>
+    <sheet name="Sample HELP" sheetId="7" r:id="rId8"/>
+    <sheet name="Sample" sheetId="8" r:id="rId9"/>
+    <sheet name="Files HELP" sheetId="9" r:id="rId10"/>
+    <sheet name="Files" sheetId="10" r:id="rId11"/>
+    <sheet name="CVs" sheetId="11" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="562">
   <si>
     <t>PLEASE READ FIRST</t>
   </si>
@@ -1911,7 +1912,25 @@
     <t>PacBio Vega</t>
   </si>
   <si>
-    <t>V3.0.1 Jun 2026</t>
+    <t>Submitters must confirm they have the right to openly share the submitted data and that the submission complies with applicable access and benefit-sharing obligations. See the "Data Access Acknowledgement" worksheet for the full statement.</t>
+  </si>
+  <si>
+    <t>To the best of my knowledge, the data being submitted are not subject to any restrictions that prohibit their open sharing and are submitted in compliance with applicable national and international access and benefit-sharing obligations, in accordance with the EMBL-EBI Terms of Use (https://www.ebi.ac.uk/about/terms-of-use/).</t>
+  </si>
+  <si>
+    <t>Statement</t>
+  </si>
+  <si>
+    <t>Acknowledgement</t>
+  </si>
+  <si>
+    <t>Data Acknowledgement</t>
+  </si>
+  <si>
+    <t>V3.1.0 Sep 2026</t>
+  </si>
+  <si>
+    <t>Statements</t>
   </si>
 </sst>
 </file>
@@ -1921,7 +1940,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -2132,6 +2151,27 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="36"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -2356,7 +2396,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2489,16 +2529,30 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2512,22 +2566,33 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2611,6 +2676,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2789,7 +2871,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMK23"/>
+  <dimension ref="A1:AMK24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="61.6640625" customWidth="1"/>
@@ -2798,8 +2880,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1025" s="5" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="68"/>
-      <c r="B1" s="68"/>
+      <c r="A1" s="72"/>
+      <c r="B1" s="72"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -2808,10 +2890,10 @@
       <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:1025" s="5" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="71"/>
+      <c r="B2" s="73"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -2820,10 +2902,10 @@
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A3" s="72" t="s">
-        <v>555</v>
-      </c>
-      <c r="B3" s="72"/>
+      <c r="A3" s="74" t="s">
+        <v>560</v>
+      </c>
+      <c r="B3" s="74"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -2832,10 +2914,10 @@
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="75" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="73"/>
+      <c r="B4" s="75"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2844,10 +2926,10 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:1025" s="5" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="74"/>
+      <c r="B5" s="76"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -3897,8 +3979,8 @@
       <c r="AMK7" s="5"/>
     </row>
     <row r="8" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="68"/>
-      <c r="B8" s="68"/>
+      <c r="A8" s="72"/>
+      <c r="B8" s="72"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -4924,10 +5006,10 @@
       <c r="AMK8" s="5"/>
     </row>
     <row r="9" spans="1:1025" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="69" t="s">
+      <c r="A9" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="69"/>
+      <c r="B9" s="78"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
@@ -5953,8 +6035,8 @@
       <c r="AMK9" s="5"/>
     </row>
     <row r="10" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="68"/>
-      <c r="B10" s="68"/>
+      <c r="A10" s="72"/>
+      <c r="B10" s="72"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -6980,10 +7062,10 @@
       <c r="AMK10" s="5"/>
     </row>
     <row r="11" spans="1:1025" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="70" t="s">
+      <c r="A11" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="70"/>
+      <c r="B11" s="79"/>
     </row>
     <row r="12" spans="1:1025" ht="20" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
@@ -7002,2128 +7084,2136 @@
       </c>
       <c r="C13" s="14"/>
     </row>
-    <row r="14" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:1025" ht="60" x14ac:dyDescent="0.2">
+      <c r="A14" s="16" t="s">
+        <v>561</v>
+      </c>
+      <c r="B14" s="67" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
+      <c r="A15" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B15" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
-      <c r="A15" s="16" t="s">
+    <row r="16" spans="1:1025" ht="80" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B16" s="13" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:1025" ht="100" x14ac:dyDescent="0.2">
-      <c r="A16" s="17" t="s">
+    <row r="17" spans="1:1025" ht="100" x14ac:dyDescent="0.2">
+      <c r="A17" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B17" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:1025" ht="60" x14ac:dyDescent="0.2">
-      <c r="A17" s="18" t="s">
+    <row r="18" spans="1:1025" ht="60" x14ac:dyDescent="0.2">
+      <c r="A18" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B18" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:1025" s="5" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="67" t="s">
+    <row r="20" spans="1:1025" s="5" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="67"/>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-      <c r="G19"/>
-      <c r="H19"/>
-      <c r="I19"/>
-      <c r="J19"/>
-      <c r="K19"/>
-      <c r="L19"/>
-      <c r="M19"/>
-      <c r="N19"/>
-      <c r="O19"/>
-      <c r="P19"/>
-      <c r="Q19"/>
-      <c r="R19"/>
-      <c r="S19"/>
-      <c r="T19"/>
-      <c r="U19"/>
-      <c r="V19"/>
-      <c r="W19"/>
-      <c r="X19"/>
-      <c r="Y19"/>
-      <c r="Z19"/>
-      <c r="AA19"/>
-      <c r="AB19"/>
-      <c r="AC19"/>
-      <c r="AD19"/>
-      <c r="AE19"/>
-      <c r="AF19"/>
-      <c r="AG19"/>
-      <c r="AH19"/>
-      <c r="AI19"/>
-      <c r="AJ19"/>
-      <c r="AK19"/>
-      <c r="AL19"/>
-      <c r="AM19"/>
-      <c r="AN19"/>
-      <c r="AO19"/>
-      <c r="AP19"/>
-      <c r="AQ19"/>
-      <c r="AR19"/>
-      <c r="AS19"/>
-      <c r="AT19"/>
-      <c r="AU19"/>
-      <c r="AV19"/>
-      <c r="AW19"/>
-      <c r="AX19"/>
-      <c r="AY19"/>
-      <c r="AZ19"/>
-      <c r="BA19"/>
-      <c r="BB19"/>
-      <c r="BC19"/>
-      <c r="BD19"/>
-      <c r="BE19"/>
-      <c r="BF19"/>
-      <c r="BG19"/>
-      <c r="BH19"/>
-      <c r="BI19"/>
-      <c r="BJ19"/>
-      <c r="BK19"/>
-      <c r="BL19"/>
-      <c r="BM19"/>
-      <c r="BN19"/>
-      <c r="BO19"/>
-      <c r="BP19"/>
-      <c r="BQ19"/>
-      <c r="BR19"/>
-      <c r="BS19"/>
-      <c r="BT19"/>
-      <c r="BU19"/>
-      <c r="BV19"/>
-      <c r="BW19"/>
-      <c r="BX19"/>
-      <c r="BY19"/>
-      <c r="BZ19"/>
-      <c r="CA19"/>
-      <c r="CB19"/>
-      <c r="CC19"/>
-      <c r="CD19"/>
-      <c r="CE19"/>
-      <c r="CF19"/>
-      <c r="CG19"/>
-      <c r="CH19"/>
-      <c r="CI19"/>
-      <c r="CJ19"/>
-      <c r="CK19"/>
-      <c r="CL19"/>
-      <c r="CM19"/>
-      <c r="CN19"/>
-      <c r="CO19"/>
-      <c r="CP19"/>
-      <c r="CQ19"/>
-      <c r="CR19"/>
-      <c r="CS19"/>
-      <c r="CT19"/>
-      <c r="CU19"/>
-      <c r="CV19"/>
-      <c r="CW19"/>
-      <c r="CX19"/>
-      <c r="CY19"/>
-      <c r="CZ19"/>
-      <c r="DA19"/>
-      <c r="DB19"/>
-      <c r="DC19"/>
-      <c r="DD19"/>
-      <c r="DE19"/>
-      <c r="DF19"/>
-      <c r="DG19"/>
-      <c r="DH19"/>
-      <c r="DI19"/>
-      <c r="DJ19"/>
-      <c r="DK19"/>
-      <c r="DL19"/>
-      <c r="DM19"/>
-      <c r="DN19"/>
-      <c r="DO19"/>
-      <c r="DP19"/>
-      <c r="DQ19"/>
-      <c r="DR19"/>
-      <c r="DS19"/>
-      <c r="DT19"/>
-      <c r="DU19"/>
-      <c r="DV19"/>
-      <c r="DW19"/>
-      <c r="DX19"/>
-      <c r="DY19"/>
-      <c r="DZ19"/>
-      <c r="EA19"/>
-      <c r="EB19"/>
-      <c r="EC19"/>
-      <c r="ED19"/>
-      <c r="EE19"/>
-      <c r="EF19"/>
-      <c r="EG19"/>
-      <c r="EH19"/>
-      <c r="EI19"/>
-      <c r="EJ19"/>
-      <c r="EK19"/>
-      <c r="EL19"/>
-      <c r="EM19"/>
-      <c r="EN19"/>
-      <c r="EO19"/>
-      <c r="EP19"/>
-      <c r="EQ19"/>
-      <c r="ER19"/>
-      <c r="ES19"/>
-      <c r="ET19"/>
-      <c r="EU19"/>
-      <c r="EV19"/>
-      <c r="EW19"/>
-      <c r="EX19"/>
-      <c r="EY19"/>
-      <c r="EZ19"/>
-      <c r="FA19"/>
-      <c r="FB19"/>
-      <c r="FC19"/>
-      <c r="FD19"/>
-      <c r="FE19"/>
-      <c r="FF19"/>
-      <c r="FG19"/>
-      <c r="FH19"/>
-      <c r="FI19"/>
-      <c r="FJ19"/>
-      <c r="FK19"/>
-      <c r="FL19"/>
-      <c r="FM19"/>
-      <c r="FN19"/>
-      <c r="FO19"/>
-      <c r="FP19"/>
-      <c r="FQ19"/>
-      <c r="FR19"/>
-      <c r="FS19"/>
-      <c r="FT19"/>
-      <c r="FU19"/>
-      <c r="FV19"/>
-      <c r="FW19"/>
-      <c r="FX19"/>
-      <c r="FY19"/>
-      <c r="FZ19"/>
-      <c r="GA19"/>
-      <c r="GB19"/>
-      <c r="GC19"/>
-      <c r="GD19"/>
-      <c r="GE19"/>
-      <c r="GF19"/>
-      <c r="GG19"/>
-      <c r="GH19"/>
-      <c r="GI19"/>
-      <c r="GJ19"/>
-      <c r="GK19"/>
-      <c r="GL19"/>
-      <c r="GM19"/>
-      <c r="GN19"/>
-      <c r="GO19"/>
-      <c r="GP19"/>
-      <c r="GQ19"/>
-      <c r="GR19"/>
-      <c r="GS19"/>
-      <c r="GT19"/>
-      <c r="GU19"/>
-      <c r="GV19"/>
-      <c r="GW19"/>
-      <c r="GX19"/>
-      <c r="GY19"/>
-      <c r="GZ19"/>
-      <c r="HA19"/>
-      <c r="HB19"/>
-      <c r="HC19"/>
-      <c r="HD19"/>
-      <c r="HE19"/>
-      <c r="HF19"/>
-      <c r="HG19"/>
-      <c r="HH19"/>
-      <c r="HI19"/>
-      <c r="HJ19"/>
-      <c r="HK19"/>
-      <c r="HL19"/>
-      <c r="HM19"/>
-      <c r="HN19"/>
-      <c r="HO19"/>
-      <c r="HP19"/>
-      <c r="HQ19"/>
-      <c r="HR19"/>
-      <c r="HS19"/>
-      <c r="HT19"/>
-      <c r="HU19"/>
-      <c r="HV19"/>
-      <c r="HW19"/>
-      <c r="HX19"/>
-      <c r="HY19"/>
-      <c r="HZ19"/>
-      <c r="IA19"/>
-      <c r="IB19"/>
-      <c r="IC19"/>
-      <c r="ID19"/>
-      <c r="IE19"/>
-      <c r="IF19"/>
-      <c r="IG19"/>
-      <c r="IH19"/>
-      <c r="II19"/>
-      <c r="IJ19"/>
-      <c r="IK19"/>
-      <c r="IL19"/>
-      <c r="IM19"/>
-      <c r="IN19"/>
-      <c r="IO19"/>
-      <c r="IP19"/>
-      <c r="IQ19"/>
-      <c r="IR19"/>
-      <c r="IS19"/>
-      <c r="IT19"/>
-      <c r="IU19"/>
-      <c r="IV19"/>
-      <c r="IW19"/>
-      <c r="IX19"/>
-      <c r="IY19"/>
-      <c r="IZ19"/>
-      <c r="JA19"/>
-      <c r="JB19"/>
-      <c r="JC19"/>
-      <c r="JD19"/>
-      <c r="JE19"/>
-      <c r="JF19"/>
-      <c r="JG19"/>
-      <c r="JH19"/>
-      <c r="JI19"/>
-      <c r="JJ19"/>
-      <c r="JK19"/>
-      <c r="JL19"/>
-      <c r="JM19"/>
-      <c r="JN19"/>
-      <c r="JO19"/>
-      <c r="JP19"/>
-      <c r="JQ19"/>
-      <c r="JR19"/>
-      <c r="JS19"/>
-      <c r="JT19"/>
-      <c r="JU19"/>
-      <c r="JV19"/>
-      <c r="JW19"/>
-      <c r="JX19"/>
-      <c r="JY19"/>
-      <c r="JZ19"/>
-      <c r="KA19"/>
-      <c r="KB19"/>
-      <c r="KC19"/>
-      <c r="KD19"/>
-      <c r="KE19"/>
-      <c r="KF19"/>
-      <c r="KG19"/>
-      <c r="KH19"/>
-      <c r="KI19"/>
-      <c r="KJ19"/>
-      <c r="KK19"/>
-      <c r="KL19"/>
-      <c r="KM19"/>
-      <c r="KN19"/>
-      <c r="KO19"/>
-      <c r="KP19"/>
-      <c r="KQ19"/>
-      <c r="KR19"/>
-      <c r="KS19"/>
-      <c r="KT19"/>
-      <c r="KU19"/>
-      <c r="KV19"/>
-      <c r="KW19"/>
-      <c r="KX19"/>
-      <c r="KY19"/>
-      <c r="KZ19"/>
-      <c r="LA19"/>
-      <c r="LB19"/>
-      <c r="LC19"/>
-      <c r="LD19"/>
-      <c r="LE19"/>
-      <c r="LF19"/>
-      <c r="LG19"/>
-      <c r="LH19"/>
-      <c r="LI19"/>
-      <c r="LJ19"/>
-      <c r="LK19"/>
-      <c r="LL19"/>
-      <c r="LM19"/>
-      <c r="LN19"/>
-      <c r="LO19"/>
-      <c r="LP19"/>
-      <c r="LQ19"/>
-      <c r="LR19"/>
-      <c r="LS19"/>
-      <c r="LT19"/>
-      <c r="LU19"/>
-      <c r="LV19"/>
-      <c r="LW19"/>
-      <c r="LX19"/>
-      <c r="LY19"/>
-      <c r="LZ19"/>
-      <c r="MA19"/>
-      <c r="MB19"/>
-      <c r="MC19"/>
-      <c r="MD19"/>
-      <c r="ME19"/>
-      <c r="MF19"/>
-      <c r="MG19"/>
-      <c r="MH19"/>
-      <c r="MI19"/>
-      <c r="MJ19"/>
-      <c r="MK19"/>
-      <c r="ML19"/>
-      <c r="MM19"/>
-      <c r="MN19"/>
-      <c r="MO19"/>
-      <c r="MP19"/>
-      <c r="MQ19"/>
-      <c r="MR19"/>
-      <c r="MS19"/>
-      <c r="MT19"/>
-      <c r="MU19"/>
-      <c r="MV19"/>
-      <c r="MW19"/>
-      <c r="MX19"/>
-      <c r="MY19"/>
-      <c r="MZ19"/>
-      <c r="NA19"/>
-      <c r="NB19"/>
-      <c r="NC19"/>
-      <c r="ND19"/>
-      <c r="NE19"/>
-      <c r="NF19"/>
-      <c r="NG19"/>
-      <c r="NH19"/>
-      <c r="NI19"/>
-      <c r="NJ19"/>
-      <c r="NK19"/>
-      <c r="NL19"/>
-      <c r="NM19"/>
-      <c r="NN19"/>
-      <c r="NO19"/>
-      <c r="NP19"/>
-      <c r="NQ19"/>
-      <c r="NR19"/>
-      <c r="NS19"/>
-      <c r="NT19"/>
-      <c r="NU19"/>
-      <c r="NV19"/>
-      <c r="NW19"/>
-      <c r="NX19"/>
-      <c r="NY19"/>
-      <c r="NZ19"/>
-      <c r="OA19"/>
-      <c r="OB19"/>
-      <c r="OC19"/>
-      <c r="OD19"/>
-      <c r="OE19"/>
-      <c r="OF19"/>
-      <c r="OG19"/>
-      <c r="OH19"/>
-      <c r="OI19"/>
-      <c r="OJ19"/>
-      <c r="OK19"/>
-      <c r="OL19"/>
-      <c r="OM19"/>
-      <c r="ON19"/>
-      <c r="OO19"/>
-      <c r="OP19"/>
-      <c r="OQ19"/>
-      <c r="OR19"/>
-      <c r="OS19"/>
-      <c r="OT19"/>
-      <c r="OU19"/>
-      <c r="OV19"/>
-      <c r="OW19"/>
-      <c r="OX19"/>
-      <c r="OY19"/>
-      <c r="OZ19"/>
-      <c r="PA19"/>
-      <c r="PB19"/>
-      <c r="PC19"/>
-      <c r="PD19"/>
-      <c r="PE19"/>
-      <c r="PF19"/>
-      <c r="PG19"/>
-      <c r="PH19"/>
-      <c r="PI19"/>
-      <c r="PJ19"/>
-      <c r="PK19"/>
-      <c r="PL19"/>
-      <c r="PM19"/>
-      <c r="PN19"/>
-      <c r="PO19"/>
-      <c r="PP19"/>
-      <c r="PQ19"/>
-      <c r="PR19"/>
-      <c r="PS19"/>
-      <c r="PT19"/>
-      <c r="PU19"/>
-      <c r="PV19"/>
-      <c r="PW19"/>
-      <c r="PX19"/>
-      <c r="PY19"/>
-      <c r="PZ19"/>
-      <c r="QA19"/>
-      <c r="QB19"/>
-      <c r="QC19"/>
-      <c r="QD19"/>
-      <c r="QE19"/>
-      <c r="QF19"/>
-      <c r="QG19"/>
-      <c r="QH19"/>
-      <c r="QI19"/>
-      <c r="QJ19"/>
-      <c r="QK19"/>
-      <c r="QL19"/>
-      <c r="QM19"/>
-      <c r="QN19"/>
-      <c r="QO19"/>
-      <c r="QP19"/>
-      <c r="QQ19"/>
-      <c r="QR19"/>
-      <c r="QS19"/>
-      <c r="QT19"/>
-      <c r="QU19"/>
-      <c r="QV19"/>
-      <c r="QW19"/>
-      <c r="QX19"/>
-      <c r="QY19"/>
-      <c r="QZ19"/>
-      <c r="RA19"/>
-      <c r="RB19"/>
-      <c r="RC19"/>
-      <c r="RD19"/>
-      <c r="RE19"/>
-      <c r="RF19"/>
-      <c r="RG19"/>
-      <c r="RH19"/>
-      <c r="RI19"/>
-      <c r="RJ19"/>
-      <c r="RK19"/>
-      <c r="RL19"/>
-      <c r="RM19"/>
-      <c r="RN19"/>
-      <c r="RO19"/>
-      <c r="RP19"/>
-      <c r="RQ19"/>
-      <c r="RR19"/>
-      <c r="RS19"/>
-      <c r="RT19"/>
-      <c r="RU19"/>
-      <c r="RV19"/>
-      <c r="RW19"/>
-      <c r="RX19"/>
-      <c r="RY19"/>
-      <c r="RZ19"/>
-      <c r="SA19"/>
-      <c r="SB19"/>
-      <c r="SC19"/>
-      <c r="SD19"/>
-      <c r="SE19"/>
-      <c r="SF19"/>
-      <c r="SG19"/>
-      <c r="SH19"/>
-      <c r="SI19"/>
-      <c r="SJ19"/>
-      <c r="SK19"/>
-      <c r="SL19"/>
-      <c r="SM19"/>
-      <c r="SN19"/>
-      <c r="SO19"/>
-      <c r="SP19"/>
-      <c r="SQ19"/>
-      <c r="SR19"/>
-      <c r="SS19"/>
-      <c r="ST19"/>
-      <c r="SU19"/>
-      <c r="SV19"/>
-      <c r="SW19"/>
-      <c r="SX19"/>
-      <c r="SY19"/>
-      <c r="SZ19"/>
-      <c r="TA19"/>
-      <c r="TB19"/>
-      <c r="TC19"/>
-      <c r="TD19"/>
-      <c r="TE19"/>
-      <c r="TF19"/>
-      <c r="TG19"/>
-      <c r="TH19"/>
-      <c r="TI19"/>
-      <c r="TJ19"/>
-      <c r="TK19"/>
-      <c r="TL19"/>
-      <c r="TM19"/>
-      <c r="TN19"/>
-      <c r="TO19"/>
-      <c r="TP19"/>
-      <c r="TQ19"/>
-      <c r="TR19"/>
-      <c r="TS19"/>
-      <c r="TT19"/>
-      <c r="TU19"/>
-      <c r="TV19"/>
-      <c r="TW19"/>
-      <c r="TX19"/>
-      <c r="TY19"/>
-      <c r="TZ19"/>
-      <c r="UA19"/>
-      <c r="UB19"/>
-      <c r="UC19"/>
-      <c r="UD19"/>
-      <c r="UE19"/>
-      <c r="UF19"/>
-      <c r="UG19"/>
-      <c r="UH19"/>
-      <c r="UI19"/>
-      <c r="UJ19"/>
-      <c r="UK19"/>
-      <c r="UL19"/>
-      <c r="UM19"/>
-      <c r="UN19"/>
-      <c r="UO19"/>
-      <c r="UP19"/>
-      <c r="UQ19"/>
-      <c r="UR19"/>
-      <c r="US19"/>
-      <c r="UT19"/>
-      <c r="UU19"/>
-      <c r="UV19"/>
-      <c r="UW19"/>
-      <c r="UX19"/>
-      <c r="UY19"/>
-      <c r="UZ19"/>
-      <c r="VA19"/>
-      <c r="VB19"/>
-      <c r="VC19"/>
-      <c r="VD19"/>
-      <c r="VE19"/>
-      <c r="VF19"/>
-      <c r="VG19"/>
-      <c r="VH19"/>
-      <c r="VI19"/>
-      <c r="VJ19"/>
-      <c r="VK19"/>
-      <c r="VL19"/>
-      <c r="VM19"/>
-      <c r="VN19"/>
-      <c r="VO19"/>
-      <c r="VP19"/>
-      <c r="VQ19"/>
-      <c r="VR19"/>
-      <c r="VS19"/>
-      <c r="VT19"/>
-      <c r="VU19"/>
-      <c r="VV19"/>
-      <c r="VW19"/>
-      <c r="VX19"/>
-      <c r="VY19"/>
-      <c r="VZ19"/>
-      <c r="WA19"/>
-      <c r="WB19"/>
-      <c r="WC19"/>
-      <c r="WD19"/>
-      <c r="WE19"/>
-      <c r="WF19"/>
-      <c r="WG19"/>
-      <c r="WH19"/>
-      <c r="WI19"/>
-      <c r="WJ19"/>
-      <c r="WK19"/>
-      <c r="WL19"/>
-      <c r="WM19"/>
-      <c r="WN19"/>
-      <c r="WO19"/>
-      <c r="WP19"/>
-      <c r="WQ19"/>
-      <c r="WR19"/>
-      <c r="WS19"/>
-      <c r="WT19"/>
-      <c r="WU19"/>
-      <c r="WV19"/>
-      <c r="WW19"/>
-      <c r="WX19"/>
-      <c r="WY19"/>
-      <c r="WZ19"/>
-      <c r="XA19"/>
-      <c r="XB19"/>
-      <c r="XC19"/>
-      <c r="XD19"/>
-      <c r="XE19"/>
-      <c r="XF19"/>
-      <c r="XG19"/>
-      <c r="XH19"/>
-      <c r="XI19"/>
-      <c r="XJ19"/>
-      <c r="XK19"/>
-      <c r="XL19"/>
-      <c r="XM19"/>
-      <c r="XN19"/>
-      <c r="XO19"/>
-      <c r="XP19"/>
-      <c r="XQ19"/>
-      <c r="XR19"/>
-      <c r="XS19"/>
-      <c r="XT19"/>
-      <c r="XU19"/>
-      <c r="XV19"/>
-      <c r="XW19"/>
-      <c r="XX19"/>
-      <c r="XY19"/>
-      <c r="XZ19"/>
-      <c r="YA19"/>
-      <c r="YB19"/>
-      <c r="YC19"/>
-      <c r="YD19"/>
-      <c r="YE19"/>
-      <c r="YF19"/>
-      <c r="YG19"/>
-      <c r="YH19"/>
-      <c r="YI19"/>
-      <c r="YJ19"/>
-      <c r="YK19"/>
-      <c r="YL19"/>
-      <c r="YM19"/>
-      <c r="YN19"/>
-      <c r="YO19"/>
-      <c r="YP19"/>
-      <c r="YQ19"/>
-      <c r="YR19"/>
-      <c r="YS19"/>
-      <c r="YT19"/>
-      <c r="YU19"/>
-      <c r="YV19"/>
-      <c r="YW19"/>
-      <c r="YX19"/>
-      <c r="YY19"/>
-      <c r="YZ19"/>
-      <c r="ZA19"/>
-      <c r="ZB19"/>
-      <c r="ZC19"/>
-      <c r="ZD19"/>
-      <c r="ZE19"/>
-      <c r="ZF19"/>
-      <c r="ZG19"/>
-      <c r="ZH19"/>
-      <c r="ZI19"/>
-      <c r="ZJ19"/>
-      <c r="ZK19"/>
-      <c r="ZL19"/>
-      <c r="ZM19"/>
-      <c r="ZN19"/>
-      <c r="ZO19"/>
-      <c r="ZP19"/>
-      <c r="ZQ19"/>
-      <c r="ZR19"/>
-      <c r="ZS19"/>
-      <c r="ZT19"/>
-      <c r="ZU19"/>
-      <c r="ZV19"/>
-      <c r="ZW19"/>
-      <c r="ZX19"/>
-      <c r="ZY19"/>
-      <c r="ZZ19"/>
-      <c r="AAA19"/>
-      <c r="AAB19"/>
-      <c r="AAC19"/>
-      <c r="AAD19"/>
-      <c r="AAE19"/>
-      <c r="AAF19"/>
-      <c r="AAG19"/>
-      <c r="AAH19"/>
-      <c r="AAI19"/>
-      <c r="AAJ19"/>
-      <c r="AAK19"/>
-      <c r="AAL19"/>
-      <c r="AAM19"/>
-      <c r="AAN19"/>
-      <c r="AAO19"/>
-      <c r="AAP19"/>
-      <c r="AAQ19"/>
-      <c r="AAR19"/>
-      <c r="AAS19"/>
-      <c r="AAT19"/>
-      <c r="AAU19"/>
-      <c r="AAV19"/>
-      <c r="AAW19"/>
-      <c r="AAX19"/>
-      <c r="AAY19"/>
-      <c r="AAZ19"/>
-      <c r="ABA19"/>
-      <c r="ABB19"/>
-      <c r="ABC19"/>
-      <c r="ABD19"/>
-      <c r="ABE19"/>
-      <c r="ABF19"/>
-      <c r="ABG19"/>
-      <c r="ABH19"/>
-      <c r="ABI19"/>
-      <c r="ABJ19"/>
-      <c r="ABK19"/>
-      <c r="ABL19"/>
-      <c r="ABM19"/>
-      <c r="ABN19"/>
-      <c r="ABO19"/>
-      <c r="ABP19"/>
-      <c r="ABQ19"/>
-      <c r="ABR19"/>
-      <c r="ABS19"/>
-      <c r="ABT19"/>
-      <c r="ABU19"/>
-      <c r="ABV19"/>
-      <c r="ABW19"/>
-      <c r="ABX19"/>
-      <c r="ABY19"/>
-      <c r="ABZ19"/>
-      <c r="ACA19"/>
-      <c r="ACB19"/>
-      <c r="ACC19"/>
-      <c r="ACD19"/>
-      <c r="ACE19"/>
-      <c r="ACF19"/>
-      <c r="ACG19"/>
-      <c r="ACH19"/>
-      <c r="ACI19"/>
-      <c r="ACJ19"/>
-      <c r="ACK19"/>
-      <c r="ACL19"/>
-      <c r="ACM19"/>
-      <c r="ACN19"/>
-      <c r="ACO19"/>
-      <c r="ACP19"/>
-      <c r="ACQ19"/>
-      <c r="ACR19"/>
-      <c r="ACS19"/>
-      <c r="ACT19"/>
-      <c r="ACU19"/>
-      <c r="ACV19"/>
-      <c r="ACW19"/>
-      <c r="ACX19"/>
-      <c r="ACY19"/>
-      <c r="ACZ19"/>
-      <c r="ADA19"/>
-      <c r="ADB19"/>
-      <c r="ADC19"/>
-      <c r="ADD19"/>
-      <c r="ADE19"/>
-      <c r="ADF19"/>
-      <c r="ADG19"/>
-      <c r="ADH19"/>
-      <c r="ADI19"/>
-      <c r="ADJ19"/>
-      <c r="ADK19"/>
-      <c r="ADL19"/>
-      <c r="ADM19"/>
-      <c r="ADN19"/>
-      <c r="ADO19"/>
-      <c r="ADP19"/>
-      <c r="ADQ19"/>
-      <c r="ADR19"/>
-      <c r="ADS19"/>
-      <c r="ADT19"/>
-      <c r="ADU19"/>
-      <c r="ADV19"/>
-      <c r="ADW19"/>
-      <c r="ADX19"/>
-      <c r="ADY19"/>
-      <c r="ADZ19"/>
-      <c r="AEA19"/>
-      <c r="AEB19"/>
-      <c r="AEC19"/>
-      <c r="AED19"/>
-      <c r="AEE19"/>
-      <c r="AEF19"/>
-      <c r="AEG19"/>
-      <c r="AEH19"/>
-      <c r="AEI19"/>
-      <c r="AEJ19"/>
-      <c r="AEK19"/>
-      <c r="AEL19"/>
-      <c r="AEM19"/>
-      <c r="AEN19"/>
-      <c r="AEO19"/>
-      <c r="AEP19"/>
-      <c r="AEQ19"/>
-      <c r="AER19"/>
-      <c r="AES19"/>
-      <c r="AET19"/>
-      <c r="AEU19"/>
-      <c r="AEV19"/>
-      <c r="AEW19"/>
-      <c r="AEX19"/>
-      <c r="AEY19"/>
-      <c r="AEZ19"/>
-      <c r="AFA19"/>
-      <c r="AFB19"/>
-      <c r="AFC19"/>
-      <c r="AFD19"/>
-      <c r="AFE19"/>
-      <c r="AFF19"/>
-      <c r="AFG19"/>
-      <c r="AFH19"/>
-      <c r="AFI19"/>
-      <c r="AFJ19"/>
-      <c r="AFK19"/>
-      <c r="AFL19"/>
-      <c r="AFM19"/>
-      <c r="AFN19"/>
-      <c r="AFO19"/>
-      <c r="AFP19"/>
-      <c r="AFQ19"/>
-      <c r="AFR19"/>
-      <c r="AFS19"/>
-      <c r="AFT19"/>
-      <c r="AFU19"/>
-      <c r="AFV19"/>
-      <c r="AFW19"/>
-      <c r="AFX19"/>
-      <c r="AFY19"/>
-      <c r="AFZ19"/>
-      <c r="AGA19"/>
-      <c r="AGB19"/>
-      <c r="AGC19"/>
-      <c r="AGD19"/>
-      <c r="AGE19"/>
-      <c r="AGF19"/>
-      <c r="AGG19"/>
-      <c r="AGH19"/>
-      <c r="AGI19"/>
-      <c r="AGJ19"/>
-      <c r="AGK19"/>
-      <c r="AGL19"/>
-      <c r="AGM19"/>
-      <c r="AGN19"/>
-      <c r="AGO19"/>
-      <c r="AGP19"/>
-      <c r="AGQ19"/>
-      <c r="AGR19"/>
-      <c r="AGS19"/>
-      <c r="AGT19"/>
-      <c r="AGU19"/>
-      <c r="AGV19"/>
-      <c r="AGW19"/>
-      <c r="AGX19"/>
-      <c r="AGY19"/>
-      <c r="AGZ19"/>
-      <c r="AHA19"/>
-      <c r="AHB19"/>
-      <c r="AHC19"/>
-      <c r="AHD19"/>
-      <c r="AHE19"/>
-      <c r="AHF19"/>
-      <c r="AHG19"/>
-      <c r="AHH19"/>
-      <c r="AHI19"/>
-      <c r="AHJ19"/>
-      <c r="AHK19"/>
-      <c r="AHL19"/>
-      <c r="AHM19"/>
-      <c r="AHN19"/>
-      <c r="AHO19"/>
-      <c r="AHP19"/>
-      <c r="AHQ19"/>
-      <c r="AHR19"/>
-      <c r="AHS19"/>
-      <c r="AHT19"/>
-      <c r="AHU19"/>
-      <c r="AHV19"/>
-      <c r="AHW19"/>
-      <c r="AHX19"/>
-      <c r="AHY19"/>
-      <c r="AHZ19"/>
-      <c r="AIA19"/>
-      <c r="AIB19"/>
-      <c r="AIC19"/>
-      <c r="AID19"/>
-      <c r="AIE19"/>
-      <c r="AIF19"/>
-      <c r="AIG19"/>
-      <c r="AIH19"/>
-      <c r="AII19"/>
-      <c r="AIJ19"/>
-      <c r="AIK19"/>
-      <c r="AIL19"/>
-      <c r="AIM19"/>
-      <c r="AIN19"/>
-      <c r="AIO19"/>
-      <c r="AIP19"/>
-      <c r="AIQ19"/>
-      <c r="AIR19"/>
-      <c r="AIS19"/>
-      <c r="AIT19"/>
-      <c r="AIU19"/>
-      <c r="AIV19"/>
-      <c r="AIW19"/>
-      <c r="AIX19"/>
-      <c r="AIY19"/>
-      <c r="AIZ19"/>
-      <c r="AJA19"/>
-      <c r="AJB19"/>
-      <c r="AJC19"/>
-      <c r="AJD19"/>
-      <c r="AJE19"/>
-      <c r="AJF19"/>
-      <c r="AJG19"/>
-      <c r="AJH19"/>
-      <c r="AJI19"/>
-      <c r="AJJ19"/>
-      <c r="AJK19"/>
-      <c r="AJL19"/>
-      <c r="AJM19"/>
-      <c r="AJN19"/>
-      <c r="AJO19"/>
-      <c r="AJP19"/>
-      <c r="AJQ19"/>
-      <c r="AJR19"/>
-      <c r="AJS19"/>
-      <c r="AJT19"/>
-      <c r="AJU19"/>
-      <c r="AJV19"/>
-      <c r="AJW19"/>
-      <c r="AJX19"/>
-      <c r="AJY19"/>
-      <c r="AJZ19"/>
-      <c r="AKA19"/>
-      <c r="AKB19"/>
-      <c r="AKC19"/>
-      <c r="AKD19"/>
-      <c r="AKE19"/>
-      <c r="AKF19"/>
-      <c r="AKG19"/>
-      <c r="AKH19"/>
-      <c r="AKI19"/>
-      <c r="AKJ19"/>
-      <c r="AKK19"/>
-      <c r="AKL19"/>
-      <c r="AKM19"/>
-      <c r="AKN19"/>
-      <c r="AKO19"/>
-      <c r="AKP19"/>
-      <c r="AKQ19"/>
-      <c r="AKR19"/>
-      <c r="AKS19"/>
-      <c r="AKT19"/>
-      <c r="AKU19"/>
-      <c r="AKV19"/>
-      <c r="AKW19"/>
-      <c r="AKX19"/>
-      <c r="AKY19"/>
-      <c r="AKZ19"/>
-      <c r="ALA19"/>
-      <c r="ALB19"/>
-      <c r="ALC19"/>
-      <c r="ALD19"/>
-      <c r="ALE19"/>
-      <c r="ALF19"/>
-      <c r="ALG19"/>
-      <c r="ALH19"/>
-      <c r="ALI19"/>
-      <c r="ALJ19"/>
-      <c r="ALK19"/>
-      <c r="ALL19"/>
-      <c r="ALM19"/>
-      <c r="ALN19"/>
-      <c r="ALO19"/>
-      <c r="ALP19"/>
-      <c r="ALQ19"/>
-      <c r="ALR19"/>
-      <c r="ALS19"/>
-      <c r="ALT19"/>
-      <c r="ALU19"/>
-      <c r="ALV19"/>
-      <c r="ALW19"/>
-      <c r="ALX19"/>
-      <c r="ALY19"/>
-      <c r="ALZ19"/>
-      <c r="AMA19"/>
-      <c r="AMB19"/>
-      <c r="AMC19"/>
-      <c r="AMD19"/>
-      <c r="AME19"/>
-      <c r="AMF19"/>
-      <c r="AMG19"/>
-      <c r="AMH19"/>
-      <c r="AMI19"/>
-      <c r="AMJ19"/>
-      <c r="AMK19"/>
-    </row>
-    <row r="20" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="67" t="s">
+      <c r="B20" s="77"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+      <c r="AR20"/>
+      <c r="AS20"/>
+      <c r="AT20"/>
+      <c r="AU20"/>
+      <c r="AV20"/>
+      <c r="AW20"/>
+      <c r="AX20"/>
+      <c r="AY20"/>
+      <c r="AZ20"/>
+      <c r="BA20"/>
+      <c r="BB20"/>
+      <c r="BC20"/>
+      <c r="BD20"/>
+      <c r="BE20"/>
+      <c r="BF20"/>
+      <c r="BG20"/>
+      <c r="BH20"/>
+      <c r="BI20"/>
+      <c r="BJ20"/>
+      <c r="BK20"/>
+      <c r="BL20"/>
+      <c r="BM20"/>
+      <c r="BN20"/>
+      <c r="BO20"/>
+      <c r="BP20"/>
+      <c r="BQ20"/>
+      <c r="BR20"/>
+      <c r="BS20"/>
+      <c r="BT20"/>
+      <c r="BU20"/>
+      <c r="BV20"/>
+      <c r="BW20"/>
+      <c r="BX20"/>
+      <c r="BY20"/>
+      <c r="BZ20"/>
+      <c r="CA20"/>
+      <c r="CB20"/>
+      <c r="CC20"/>
+      <c r="CD20"/>
+      <c r="CE20"/>
+      <c r="CF20"/>
+      <c r="CG20"/>
+      <c r="CH20"/>
+      <c r="CI20"/>
+      <c r="CJ20"/>
+      <c r="CK20"/>
+      <c r="CL20"/>
+      <c r="CM20"/>
+      <c r="CN20"/>
+      <c r="CO20"/>
+      <c r="CP20"/>
+      <c r="CQ20"/>
+      <c r="CR20"/>
+      <c r="CS20"/>
+      <c r="CT20"/>
+      <c r="CU20"/>
+      <c r="CV20"/>
+      <c r="CW20"/>
+      <c r="CX20"/>
+      <c r="CY20"/>
+      <c r="CZ20"/>
+      <c r="DA20"/>
+      <c r="DB20"/>
+      <c r="DC20"/>
+      <c r="DD20"/>
+      <c r="DE20"/>
+      <c r="DF20"/>
+      <c r="DG20"/>
+      <c r="DH20"/>
+      <c r="DI20"/>
+      <c r="DJ20"/>
+      <c r="DK20"/>
+      <c r="DL20"/>
+      <c r="DM20"/>
+      <c r="DN20"/>
+      <c r="DO20"/>
+      <c r="DP20"/>
+      <c r="DQ20"/>
+      <c r="DR20"/>
+      <c r="DS20"/>
+      <c r="DT20"/>
+      <c r="DU20"/>
+      <c r="DV20"/>
+      <c r="DW20"/>
+      <c r="DX20"/>
+      <c r="DY20"/>
+      <c r="DZ20"/>
+      <c r="EA20"/>
+      <c r="EB20"/>
+      <c r="EC20"/>
+      <c r="ED20"/>
+      <c r="EE20"/>
+      <c r="EF20"/>
+      <c r="EG20"/>
+      <c r="EH20"/>
+      <c r="EI20"/>
+      <c r="EJ20"/>
+      <c r="EK20"/>
+      <c r="EL20"/>
+      <c r="EM20"/>
+      <c r="EN20"/>
+      <c r="EO20"/>
+      <c r="EP20"/>
+      <c r="EQ20"/>
+      <c r="ER20"/>
+      <c r="ES20"/>
+      <c r="ET20"/>
+      <c r="EU20"/>
+      <c r="EV20"/>
+      <c r="EW20"/>
+      <c r="EX20"/>
+      <c r="EY20"/>
+      <c r="EZ20"/>
+      <c r="FA20"/>
+      <c r="FB20"/>
+      <c r="FC20"/>
+      <c r="FD20"/>
+      <c r="FE20"/>
+      <c r="FF20"/>
+      <c r="FG20"/>
+      <c r="FH20"/>
+      <c r="FI20"/>
+      <c r="FJ20"/>
+      <c r="FK20"/>
+      <c r="FL20"/>
+      <c r="FM20"/>
+      <c r="FN20"/>
+      <c r="FO20"/>
+      <c r="FP20"/>
+      <c r="FQ20"/>
+      <c r="FR20"/>
+      <c r="FS20"/>
+      <c r="FT20"/>
+      <c r="FU20"/>
+      <c r="FV20"/>
+      <c r="FW20"/>
+      <c r="FX20"/>
+      <c r="FY20"/>
+      <c r="FZ20"/>
+      <c r="GA20"/>
+      <c r="GB20"/>
+      <c r="GC20"/>
+      <c r="GD20"/>
+      <c r="GE20"/>
+      <c r="GF20"/>
+      <c r="GG20"/>
+      <c r="GH20"/>
+      <c r="GI20"/>
+      <c r="GJ20"/>
+      <c r="GK20"/>
+      <c r="GL20"/>
+      <c r="GM20"/>
+      <c r="GN20"/>
+      <c r="GO20"/>
+      <c r="GP20"/>
+      <c r="GQ20"/>
+      <c r="GR20"/>
+      <c r="GS20"/>
+      <c r="GT20"/>
+      <c r="GU20"/>
+      <c r="GV20"/>
+      <c r="GW20"/>
+      <c r="GX20"/>
+      <c r="GY20"/>
+      <c r="GZ20"/>
+      <c r="HA20"/>
+      <c r="HB20"/>
+      <c r="HC20"/>
+      <c r="HD20"/>
+      <c r="HE20"/>
+      <c r="HF20"/>
+      <c r="HG20"/>
+      <c r="HH20"/>
+      <c r="HI20"/>
+      <c r="HJ20"/>
+      <c r="HK20"/>
+      <c r="HL20"/>
+      <c r="HM20"/>
+      <c r="HN20"/>
+      <c r="HO20"/>
+      <c r="HP20"/>
+      <c r="HQ20"/>
+      <c r="HR20"/>
+      <c r="HS20"/>
+      <c r="HT20"/>
+      <c r="HU20"/>
+      <c r="HV20"/>
+      <c r="HW20"/>
+      <c r="HX20"/>
+      <c r="HY20"/>
+      <c r="HZ20"/>
+      <c r="IA20"/>
+      <c r="IB20"/>
+      <c r="IC20"/>
+      <c r="ID20"/>
+      <c r="IE20"/>
+      <c r="IF20"/>
+      <c r="IG20"/>
+      <c r="IH20"/>
+      <c r="II20"/>
+      <c r="IJ20"/>
+      <c r="IK20"/>
+      <c r="IL20"/>
+      <c r="IM20"/>
+      <c r="IN20"/>
+      <c r="IO20"/>
+      <c r="IP20"/>
+      <c r="IQ20"/>
+      <c r="IR20"/>
+      <c r="IS20"/>
+      <c r="IT20"/>
+      <c r="IU20"/>
+      <c r="IV20"/>
+      <c r="IW20"/>
+      <c r="IX20"/>
+      <c r="IY20"/>
+      <c r="IZ20"/>
+      <c r="JA20"/>
+      <c r="JB20"/>
+      <c r="JC20"/>
+      <c r="JD20"/>
+      <c r="JE20"/>
+      <c r="JF20"/>
+      <c r="JG20"/>
+      <c r="JH20"/>
+      <c r="JI20"/>
+      <c r="JJ20"/>
+      <c r="JK20"/>
+      <c r="JL20"/>
+      <c r="JM20"/>
+      <c r="JN20"/>
+      <c r="JO20"/>
+      <c r="JP20"/>
+      <c r="JQ20"/>
+      <c r="JR20"/>
+      <c r="JS20"/>
+      <c r="JT20"/>
+      <c r="JU20"/>
+      <c r="JV20"/>
+      <c r="JW20"/>
+      <c r="JX20"/>
+      <c r="JY20"/>
+      <c r="JZ20"/>
+      <c r="KA20"/>
+      <c r="KB20"/>
+      <c r="KC20"/>
+      <c r="KD20"/>
+      <c r="KE20"/>
+      <c r="KF20"/>
+      <c r="KG20"/>
+      <c r="KH20"/>
+      <c r="KI20"/>
+      <c r="KJ20"/>
+      <c r="KK20"/>
+      <c r="KL20"/>
+      <c r="KM20"/>
+      <c r="KN20"/>
+      <c r="KO20"/>
+      <c r="KP20"/>
+      <c r="KQ20"/>
+      <c r="KR20"/>
+      <c r="KS20"/>
+      <c r="KT20"/>
+      <c r="KU20"/>
+      <c r="KV20"/>
+      <c r="KW20"/>
+      <c r="KX20"/>
+      <c r="KY20"/>
+      <c r="KZ20"/>
+      <c r="LA20"/>
+      <c r="LB20"/>
+      <c r="LC20"/>
+      <c r="LD20"/>
+      <c r="LE20"/>
+      <c r="LF20"/>
+      <c r="LG20"/>
+      <c r="LH20"/>
+      <c r="LI20"/>
+      <c r="LJ20"/>
+      <c r="LK20"/>
+      <c r="LL20"/>
+      <c r="LM20"/>
+      <c r="LN20"/>
+      <c r="LO20"/>
+      <c r="LP20"/>
+      <c r="LQ20"/>
+      <c r="LR20"/>
+      <c r="LS20"/>
+      <c r="LT20"/>
+      <c r="LU20"/>
+      <c r="LV20"/>
+      <c r="LW20"/>
+      <c r="LX20"/>
+      <c r="LY20"/>
+      <c r="LZ20"/>
+      <c r="MA20"/>
+      <c r="MB20"/>
+      <c r="MC20"/>
+      <c r="MD20"/>
+      <c r="ME20"/>
+      <c r="MF20"/>
+      <c r="MG20"/>
+      <c r="MH20"/>
+      <c r="MI20"/>
+      <c r="MJ20"/>
+      <c r="MK20"/>
+      <c r="ML20"/>
+      <c r="MM20"/>
+      <c r="MN20"/>
+      <c r="MO20"/>
+      <c r="MP20"/>
+      <c r="MQ20"/>
+      <c r="MR20"/>
+      <c r="MS20"/>
+      <c r="MT20"/>
+      <c r="MU20"/>
+      <c r="MV20"/>
+      <c r="MW20"/>
+      <c r="MX20"/>
+      <c r="MY20"/>
+      <c r="MZ20"/>
+      <c r="NA20"/>
+      <c r="NB20"/>
+      <c r="NC20"/>
+      <c r="ND20"/>
+      <c r="NE20"/>
+      <c r="NF20"/>
+      <c r="NG20"/>
+      <c r="NH20"/>
+      <c r="NI20"/>
+      <c r="NJ20"/>
+      <c r="NK20"/>
+      <c r="NL20"/>
+      <c r="NM20"/>
+      <c r="NN20"/>
+      <c r="NO20"/>
+      <c r="NP20"/>
+      <c r="NQ20"/>
+      <c r="NR20"/>
+      <c r="NS20"/>
+      <c r="NT20"/>
+      <c r="NU20"/>
+      <c r="NV20"/>
+      <c r="NW20"/>
+      <c r="NX20"/>
+      <c r="NY20"/>
+      <c r="NZ20"/>
+      <c r="OA20"/>
+      <c r="OB20"/>
+      <c r="OC20"/>
+      <c r="OD20"/>
+      <c r="OE20"/>
+      <c r="OF20"/>
+      <c r="OG20"/>
+      <c r="OH20"/>
+      <c r="OI20"/>
+      <c r="OJ20"/>
+      <c r="OK20"/>
+      <c r="OL20"/>
+      <c r="OM20"/>
+      <c r="ON20"/>
+      <c r="OO20"/>
+      <c r="OP20"/>
+      <c r="OQ20"/>
+      <c r="OR20"/>
+      <c r="OS20"/>
+      <c r="OT20"/>
+      <c r="OU20"/>
+      <c r="OV20"/>
+      <c r="OW20"/>
+      <c r="OX20"/>
+      <c r="OY20"/>
+      <c r="OZ20"/>
+      <c r="PA20"/>
+      <c r="PB20"/>
+      <c r="PC20"/>
+      <c r="PD20"/>
+      <c r="PE20"/>
+      <c r="PF20"/>
+      <c r="PG20"/>
+      <c r="PH20"/>
+      <c r="PI20"/>
+      <c r="PJ20"/>
+      <c r="PK20"/>
+      <c r="PL20"/>
+      <c r="PM20"/>
+      <c r="PN20"/>
+      <c r="PO20"/>
+      <c r="PP20"/>
+      <c r="PQ20"/>
+      <c r="PR20"/>
+      <c r="PS20"/>
+      <c r="PT20"/>
+      <c r="PU20"/>
+      <c r="PV20"/>
+      <c r="PW20"/>
+      <c r="PX20"/>
+      <c r="PY20"/>
+      <c r="PZ20"/>
+      <c r="QA20"/>
+      <c r="QB20"/>
+      <c r="QC20"/>
+      <c r="QD20"/>
+      <c r="QE20"/>
+      <c r="QF20"/>
+      <c r="QG20"/>
+      <c r="QH20"/>
+      <c r="QI20"/>
+      <c r="QJ20"/>
+      <c r="QK20"/>
+      <c r="QL20"/>
+      <c r="QM20"/>
+      <c r="QN20"/>
+      <c r="QO20"/>
+      <c r="QP20"/>
+      <c r="QQ20"/>
+      <c r="QR20"/>
+      <c r="QS20"/>
+      <c r="QT20"/>
+      <c r="QU20"/>
+      <c r="QV20"/>
+      <c r="QW20"/>
+      <c r="QX20"/>
+      <c r="QY20"/>
+      <c r="QZ20"/>
+      <c r="RA20"/>
+      <c r="RB20"/>
+      <c r="RC20"/>
+      <c r="RD20"/>
+      <c r="RE20"/>
+      <c r="RF20"/>
+      <c r="RG20"/>
+      <c r="RH20"/>
+      <c r="RI20"/>
+      <c r="RJ20"/>
+      <c r="RK20"/>
+      <c r="RL20"/>
+      <c r="RM20"/>
+      <c r="RN20"/>
+      <c r="RO20"/>
+      <c r="RP20"/>
+      <c r="RQ20"/>
+      <c r="RR20"/>
+      <c r="RS20"/>
+      <c r="RT20"/>
+      <c r="RU20"/>
+      <c r="RV20"/>
+      <c r="RW20"/>
+      <c r="RX20"/>
+      <c r="RY20"/>
+      <c r="RZ20"/>
+      <c r="SA20"/>
+      <c r="SB20"/>
+      <c r="SC20"/>
+      <c r="SD20"/>
+      <c r="SE20"/>
+      <c r="SF20"/>
+      <c r="SG20"/>
+      <c r="SH20"/>
+      <c r="SI20"/>
+      <c r="SJ20"/>
+      <c r="SK20"/>
+      <c r="SL20"/>
+      <c r="SM20"/>
+      <c r="SN20"/>
+      <c r="SO20"/>
+      <c r="SP20"/>
+      <c r="SQ20"/>
+      <c r="SR20"/>
+      <c r="SS20"/>
+      <c r="ST20"/>
+      <c r="SU20"/>
+      <c r="SV20"/>
+      <c r="SW20"/>
+      <c r="SX20"/>
+      <c r="SY20"/>
+      <c r="SZ20"/>
+      <c r="TA20"/>
+      <c r="TB20"/>
+      <c r="TC20"/>
+      <c r="TD20"/>
+      <c r="TE20"/>
+      <c r="TF20"/>
+      <c r="TG20"/>
+      <c r="TH20"/>
+      <c r="TI20"/>
+      <c r="TJ20"/>
+      <c r="TK20"/>
+      <c r="TL20"/>
+      <c r="TM20"/>
+      <c r="TN20"/>
+      <c r="TO20"/>
+      <c r="TP20"/>
+      <c r="TQ20"/>
+      <c r="TR20"/>
+      <c r="TS20"/>
+      <c r="TT20"/>
+      <c r="TU20"/>
+      <c r="TV20"/>
+      <c r="TW20"/>
+      <c r="TX20"/>
+      <c r="TY20"/>
+      <c r="TZ20"/>
+      <c r="UA20"/>
+      <c r="UB20"/>
+      <c r="UC20"/>
+      <c r="UD20"/>
+      <c r="UE20"/>
+      <c r="UF20"/>
+      <c r="UG20"/>
+      <c r="UH20"/>
+      <c r="UI20"/>
+      <c r="UJ20"/>
+      <c r="UK20"/>
+      <c r="UL20"/>
+      <c r="UM20"/>
+      <c r="UN20"/>
+      <c r="UO20"/>
+      <c r="UP20"/>
+      <c r="UQ20"/>
+      <c r="UR20"/>
+      <c r="US20"/>
+      <c r="UT20"/>
+      <c r="UU20"/>
+      <c r="UV20"/>
+      <c r="UW20"/>
+      <c r="UX20"/>
+      <c r="UY20"/>
+      <c r="UZ20"/>
+      <c r="VA20"/>
+      <c r="VB20"/>
+      <c r="VC20"/>
+      <c r="VD20"/>
+      <c r="VE20"/>
+      <c r="VF20"/>
+      <c r="VG20"/>
+      <c r="VH20"/>
+      <c r="VI20"/>
+      <c r="VJ20"/>
+      <c r="VK20"/>
+      <c r="VL20"/>
+      <c r="VM20"/>
+      <c r="VN20"/>
+      <c r="VO20"/>
+      <c r="VP20"/>
+      <c r="VQ20"/>
+      <c r="VR20"/>
+      <c r="VS20"/>
+      <c r="VT20"/>
+      <c r="VU20"/>
+      <c r="VV20"/>
+      <c r="VW20"/>
+      <c r="VX20"/>
+      <c r="VY20"/>
+      <c r="VZ20"/>
+      <c r="WA20"/>
+      <c r="WB20"/>
+      <c r="WC20"/>
+      <c r="WD20"/>
+      <c r="WE20"/>
+      <c r="WF20"/>
+      <c r="WG20"/>
+      <c r="WH20"/>
+      <c r="WI20"/>
+      <c r="WJ20"/>
+      <c r="WK20"/>
+      <c r="WL20"/>
+      <c r="WM20"/>
+      <c r="WN20"/>
+      <c r="WO20"/>
+      <c r="WP20"/>
+      <c r="WQ20"/>
+      <c r="WR20"/>
+      <c r="WS20"/>
+      <c r="WT20"/>
+      <c r="WU20"/>
+      <c r="WV20"/>
+      <c r="WW20"/>
+      <c r="WX20"/>
+      <c r="WY20"/>
+      <c r="WZ20"/>
+      <c r="XA20"/>
+      <c r="XB20"/>
+      <c r="XC20"/>
+      <c r="XD20"/>
+      <c r="XE20"/>
+      <c r="XF20"/>
+      <c r="XG20"/>
+      <c r="XH20"/>
+      <c r="XI20"/>
+      <c r="XJ20"/>
+      <c r="XK20"/>
+      <c r="XL20"/>
+      <c r="XM20"/>
+      <c r="XN20"/>
+      <c r="XO20"/>
+      <c r="XP20"/>
+      <c r="XQ20"/>
+      <c r="XR20"/>
+      <c r="XS20"/>
+      <c r="XT20"/>
+      <c r="XU20"/>
+      <c r="XV20"/>
+      <c r="XW20"/>
+      <c r="XX20"/>
+      <c r="XY20"/>
+      <c r="XZ20"/>
+      <c r="YA20"/>
+      <c r="YB20"/>
+      <c r="YC20"/>
+      <c r="YD20"/>
+      <c r="YE20"/>
+      <c r="YF20"/>
+      <c r="YG20"/>
+      <c r="YH20"/>
+      <c r="YI20"/>
+      <c r="YJ20"/>
+      <c r="YK20"/>
+      <c r="YL20"/>
+      <c r="YM20"/>
+      <c r="YN20"/>
+      <c r="YO20"/>
+      <c r="YP20"/>
+      <c r="YQ20"/>
+      <c r="YR20"/>
+      <c r="YS20"/>
+      <c r="YT20"/>
+      <c r="YU20"/>
+      <c r="YV20"/>
+      <c r="YW20"/>
+      <c r="YX20"/>
+      <c r="YY20"/>
+      <c r="YZ20"/>
+      <c r="ZA20"/>
+      <c r="ZB20"/>
+      <c r="ZC20"/>
+      <c r="ZD20"/>
+      <c r="ZE20"/>
+      <c r="ZF20"/>
+      <c r="ZG20"/>
+      <c r="ZH20"/>
+      <c r="ZI20"/>
+      <c r="ZJ20"/>
+      <c r="ZK20"/>
+      <c r="ZL20"/>
+      <c r="ZM20"/>
+      <c r="ZN20"/>
+      <c r="ZO20"/>
+      <c r="ZP20"/>
+      <c r="ZQ20"/>
+      <c r="ZR20"/>
+      <c r="ZS20"/>
+      <c r="ZT20"/>
+      <c r="ZU20"/>
+      <c r="ZV20"/>
+      <c r="ZW20"/>
+      <c r="ZX20"/>
+      <c r="ZY20"/>
+      <c r="ZZ20"/>
+      <c r="AAA20"/>
+      <c r="AAB20"/>
+      <c r="AAC20"/>
+      <c r="AAD20"/>
+      <c r="AAE20"/>
+      <c r="AAF20"/>
+      <c r="AAG20"/>
+      <c r="AAH20"/>
+      <c r="AAI20"/>
+      <c r="AAJ20"/>
+      <c r="AAK20"/>
+      <c r="AAL20"/>
+      <c r="AAM20"/>
+      <c r="AAN20"/>
+      <c r="AAO20"/>
+      <c r="AAP20"/>
+      <c r="AAQ20"/>
+      <c r="AAR20"/>
+      <c r="AAS20"/>
+      <c r="AAT20"/>
+      <c r="AAU20"/>
+      <c r="AAV20"/>
+      <c r="AAW20"/>
+      <c r="AAX20"/>
+      <c r="AAY20"/>
+      <c r="AAZ20"/>
+      <c r="ABA20"/>
+      <c r="ABB20"/>
+      <c r="ABC20"/>
+      <c r="ABD20"/>
+      <c r="ABE20"/>
+      <c r="ABF20"/>
+      <c r="ABG20"/>
+      <c r="ABH20"/>
+      <c r="ABI20"/>
+      <c r="ABJ20"/>
+      <c r="ABK20"/>
+      <c r="ABL20"/>
+      <c r="ABM20"/>
+      <c r="ABN20"/>
+      <c r="ABO20"/>
+      <c r="ABP20"/>
+      <c r="ABQ20"/>
+      <c r="ABR20"/>
+      <c r="ABS20"/>
+      <c r="ABT20"/>
+      <c r="ABU20"/>
+      <c r="ABV20"/>
+      <c r="ABW20"/>
+      <c r="ABX20"/>
+      <c r="ABY20"/>
+      <c r="ABZ20"/>
+      <c r="ACA20"/>
+      <c r="ACB20"/>
+      <c r="ACC20"/>
+      <c r="ACD20"/>
+      <c r="ACE20"/>
+      <c r="ACF20"/>
+      <c r="ACG20"/>
+      <c r="ACH20"/>
+      <c r="ACI20"/>
+      <c r="ACJ20"/>
+      <c r="ACK20"/>
+      <c r="ACL20"/>
+      <c r="ACM20"/>
+      <c r="ACN20"/>
+      <c r="ACO20"/>
+      <c r="ACP20"/>
+      <c r="ACQ20"/>
+      <c r="ACR20"/>
+      <c r="ACS20"/>
+      <c r="ACT20"/>
+      <c r="ACU20"/>
+      <c r="ACV20"/>
+      <c r="ACW20"/>
+      <c r="ACX20"/>
+      <c r="ACY20"/>
+      <c r="ACZ20"/>
+      <c r="ADA20"/>
+      <c r="ADB20"/>
+      <c r="ADC20"/>
+      <c r="ADD20"/>
+      <c r="ADE20"/>
+      <c r="ADF20"/>
+      <c r="ADG20"/>
+      <c r="ADH20"/>
+      <c r="ADI20"/>
+      <c r="ADJ20"/>
+      <c r="ADK20"/>
+      <c r="ADL20"/>
+      <c r="ADM20"/>
+      <c r="ADN20"/>
+      <c r="ADO20"/>
+      <c r="ADP20"/>
+      <c r="ADQ20"/>
+      <c r="ADR20"/>
+      <c r="ADS20"/>
+      <c r="ADT20"/>
+      <c r="ADU20"/>
+      <c r="ADV20"/>
+      <c r="ADW20"/>
+      <c r="ADX20"/>
+      <c r="ADY20"/>
+      <c r="ADZ20"/>
+      <c r="AEA20"/>
+      <c r="AEB20"/>
+      <c r="AEC20"/>
+      <c r="AED20"/>
+      <c r="AEE20"/>
+      <c r="AEF20"/>
+      <c r="AEG20"/>
+      <c r="AEH20"/>
+      <c r="AEI20"/>
+      <c r="AEJ20"/>
+      <c r="AEK20"/>
+      <c r="AEL20"/>
+      <c r="AEM20"/>
+      <c r="AEN20"/>
+      <c r="AEO20"/>
+      <c r="AEP20"/>
+      <c r="AEQ20"/>
+      <c r="AER20"/>
+      <c r="AES20"/>
+      <c r="AET20"/>
+      <c r="AEU20"/>
+      <c r="AEV20"/>
+      <c r="AEW20"/>
+      <c r="AEX20"/>
+      <c r="AEY20"/>
+      <c r="AEZ20"/>
+      <c r="AFA20"/>
+      <c r="AFB20"/>
+      <c r="AFC20"/>
+      <c r="AFD20"/>
+      <c r="AFE20"/>
+      <c r="AFF20"/>
+      <c r="AFG20"/>
+      <c r="AFH20"/>
+      <c r="AFI20"/>
+      <c r="AFJ20"/>
+      <c r="AFK20"/>
+      <c r="AFL20"/>
+      <c r="AFM20"/>
+      <c r="AFN20"/>
+      <c r="AFO20"/>
+      <c r="AFP20"/>
+      <c r="AFQ20"/>
+      <c r="AFR20"/>
+      <c r="AFS20"/>
+      <c r="AFT20"/>
+      <c r="AFU20"/>
+      <c r="AFV20"/>
+      <c r="AFW20"/>
+      <c r="AFX20"/>
+      <c r="AFY20"/>
+      <c r="AFZ20"/>
+      <c r="AGA20"/>
+      <c r="AGB20"/>
+      <c r="AGC20"/>
+      <c r="AGD20"/>
+      <c r="AGE20"/>
+      <c r="AGF20"/>
+      <c r="AGG20"/>
+      <c r="AGH20"/>
+      <c r="AGI20"/>
+      <c r="AGJ20"/>
+      <c r="AGK20"/>
+      <c r="AGL20"/>
+      <c r="AGM20"/>
+      <c r="AGN20"/>
+      <c r="AGO20"/>
+      <c r="AGP20"/>
+      <c r="AGQ20"/>
+      <c r="AGR20"/>
+      <c r="AGS20"/>
+      <c r="AGT20"/>
+      <c r="AGU20"/>
+      <c r="AGV20"/>
+      <c r="AGW20"/>
+      <c r="AGX20"/>
+      <c r="AGY20"/>
+      <c r="AGZ20"/>
+      <c r="AHA20"/>
+      <c r="AHB20"/>
+      <c r="AHC20"/>
+      <c r="AHD20"/>
+      <c r="AHE20"/>
+      <c r="AHF20"/>
+      <c r="AHG20"/>
+      <c r="AHH20"/>
+      <c r="AHI20"/>
+      <c r="AHJ20"/>
+      <c r="AHK20"/>
+      <c r="AHL20"/>
+      <c r="AHM20"/>
+      <c r="AHN20"/>
+      <c r="AHO20"/>
+      <c r="AHP20"/>
+      <c r="AHQ20"/>
+      <c r="AHR20"/>
+      <c r="AHS20"/>
+      <c r="AHT20"/>
+      <c r="AHU20"/>
+      <c r="AHV20"/>
+      <c r="AHW20"/>
+      <c r="AHX20"/>
+      <c r="AHY20"/>
+      <c r="AHZ20"/>
+      <c r="AIA20"/>
+      <c r="AIB20"/>
+      <c r="AIC20"/>
+      <c r="AID20"/>
+      <c r="AIE20"/>
+      <c r="AIF20"/>
+      <c r="AIG20"/>
+      <c r="AIH20"/>
+      <c r="AII20"/>
+      <c r="AIJ20"/>
+      <c r="AIK20"/>
+      <c r="AIL20"/>
+      <c r="AIM20"/>
+      <c r="AIN20"/>
+      <c r="AIO20"/>
+      <c r="AIP20"/>
+      <c r="AIQ20"/>
+      <c r="AIR20"/>
+      <c r="AIS20"/>
+      <c r="AIT20"/>
+      <c r="AIU20"/>
+      <c r="AIV20"/>
+      <c r="AIW20"/>
+      <c r="AIX20"/>
+      <c r="AIY20"/>
+      <c r="AIZ20"/>
+      <c r="AJA20"/>
+      <c r="AJB20"/>
+      <c r="AJC20"/>
+      <c r="AJD20"/>
+      <c r="AJE20"/>
+      <c r="AJF20"/>
+      <c r="AJG20"/>
+      <c r="AJH20"/>
+      <c r="AJI20"/>
+      <c r="AJJ20"/>
+      <c r="AJK20"/>
+      <c r="AJL20"/>
+      <c r="AJM20"/>
+      <c r="AJN20"/>
+      <c r="AJO20"/>
+      <c r="AJP20"/>
+      <c r="AJQ20"/>
+      <c r="AJR20"/>
+      <c r="AJS20"/>
+      <c r="AJT20"/>
+      <c r="AJU20"/>
+      <c r="AJV20"/>
+      <c r="AJW20"/>
+      <c r="AJX20"/>
+      <c r="AJY20"/>
+      <c r="AJZ20"/>
+      <c r="AKA20"/>
+      <c r="AKB20"/>
+      <c r="AKC20"/>
+      <c r="AKD20"/>
+      <c r="AKE20"/>
+      <c r="AKF20"/>
+      <c r="AKG20"/>
+      <c r="AKH20"/>
+      <c r="AKI20"/>
+      <c r="AKJ20"/>
+      <c r="AKK20"/>
+      <c r="AKL20"/>
+      <c r="AKM20"/>
+      <c r="AKN20"/>
+      <c r="AKO20"/>
+      <c r="AKP20"/>
+      <c r="AKQ20"/>
+      <c r="AKR20"/>
+      <c r="AKS20"/>
+      <c r="AKT20"/>
+      <c r="AKU20"/>
+      <c r="AKV20"/>
+      <c r="AKW20"/>
+      <c r="AKX20"/>
+      <c r="AKY20"/>
+      <c r="AKZ20"/>
+      <c r="ALA20"/>
+      <c r="ALB20"/>
+      <c r="ALC20"/>
+      <c r="ALD20"/>
+      <c r="ALE20"/>
+      <c r="ALF20"/>
+      <c r="ALG20"/>
+      <c r="ALH20"/>
+      <c r="ALI20"/>
+      <c r="ALJ20"/>
+      <c r="ALK20"/>
+      <c r="ALL20"/>
+      <c r="ALM20"/>
+      <c r="ALN20"/>
+      <c r="ALO20"/>
+      <c r="ALP20"/>
+      <c r="ALQ20"/>
+      <c r="ALR20"/>
+      <c r="ALS20"/>
+      <c r="ALT20"/>
+      <c r="ALU20"/>
+      <c r="ALV20"/>
+      <c r="ALW20"/>
+      <c r="ALX20"/>
+      <c r="ALY20"/>
+      <c r="ALZ20"/>
+      <c r="AMA20"/>
+      <c r="AMB20"/>
+      <c r="AMC20"/>
+      <c r="AMD20"/>
+      <c r="AME20"/>
+      <c r="AMF20"/>
+      <c r="AMG20"/>
+      <c r="AMH20"/>
+      <c r="AMI20"/>
+      <c r="AMJ20"/>
+      <c r="AMK20"/>
+    </row>
+    <row r="21" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="67"/>
-    </row>
-    <row r="21" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="67" t="s">
+      <c r="B21" s="77"/>
+    </row>
+    <row r="22" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="67"/>
-    </row>
-    <row r="22" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="67" t="s">
+      <c r="B22" s="77"/>
+    </row>
+    <row r="23" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="67"/>
-    </row>
-    <row r="23" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="19"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="5"/>
-      <c r="W23" s="5"/>
-      <c r="X23" s="5"/>
-      <c r="Y23" s="5"/>
-      <c r="Z23" s="5"/>
-      <c r="AA23" s="5"/>
-      <c r="AB23" s="5"/>
-      <c r="AC23" s="5"/>
-      <c r="AD23" s="5"/>
-      <c r="AE23" s="5"/>
-      <c r="AF23" s="5"/>
-      <c r="AG23" s="5"/>
-      <c r="AH23" s="5"/>
-      <c r="AI23" s="5"/>
-      <c r="AJ23" s="5"/>
-      <c r="AK23" s="5"/>
-      <c r="AL23" s="5"/>
-      <c r="AM23" s="5"/>
-      <c r="AN23" s="5"/>
-      <c r="AO23" s="5"/>
-      <c r="AP23" s="5"/>
-      <c r="AQ23" s="5"/>
-      <c r="AR23" s="5"/>
-      <c r="AS23" s="5"/>
-      <c r="AT23" s="5"/>
-      <c r="AU23" s="5"/>
-      <c r="AV23" s="5"/>
-      <c r="AW23" s="5"/>
-      <c r="AX23" s="5"/>
-      <c r="AY23" s="5"/>
-      <c r="AZ23" s="5"/>
-      <c r="BA23" s="5"/>
-      <c r="BB23" s="5"/>
-      <c r="BC23" s="5"/>
-      <c r="BD23" s="5"/>
-      <c r="BE23" s="5"/>
-      <c r="BF23" s="5"/>
-      <c r="BG23" s="5"/>
-      <c r="BH23" s="5"/>
-      <c r="BI23" s="5"/>
-      <c r="BJ23" s="5"/>
-      <c r="BK23" s="5"/>
-      <c r="BL23" s="5"/>
-      <c r="BM23" s="5"/>
-      <c r="BN23" s="5"/>
-      <c r="BO23" s="5"/>
-      <c r="BP23" s="5"/>
-      <c r="BQ23" s="5"/>
-      <c r="BR23" s="5"/>
-      <c r="BS23" s="5"/>
-      <c r="BT23" s="5"/>
-      <c r="BU23" s="5"/>
-      <c r="BV23" s="5"/>
-      <c r="BW23" s="5"/>
-      <c r="BX23" s="5"/>
-      <c r="BY23" s="5"/>
-      <c r="BZ23" s="5"/>
-      <c r="CA23" s="5"/>
-      <c r="CB23" s="5"/>
-      <c r="CC23" s="5"/>
-      <c r="CD23" s="5"/>
-      <c r="CE23" s="5"/>
-      <c r="CF23" s="5"/>
-      <c r="CG23" s="5"/>
-      <c r="CH23" s="5"/>
-      <c r="CI23" s="5"/>
-      <c r="CJ23" s="5"/>
-      <c r="CK23" s="5"/>
-      <c r="CL23" s="5"/>
-      <c r="CM23" s="5"/>
-      <c r="CN23" s="5"/>
-      <c r="CO23" s="5"/>
-      <c r="CP23" s="5"/>
-      <c r="CQ23" s="5"/>
-      <c r="CR23" s="5"/>
-      <c r="CS23" s="5"/>
-      <c r="CT23" s="5"/>
-      <c r="CU23" s="5"/>
-      <c r="CV23" s="5"/>
-      <c r="CW23" s="5"/>
-      <c r="CX23" s="5"/>
-      <c r="CY23" s="5"/>
-      <c r="CZ23" s="5"/>
-      <c r="DA23" s="5"/>
-      <c r="DB23" s="5"/>
-      <c r="DC23" s="5"/>
-      <c r="DD23" s="5"/>
-      <c r="DE23" s="5"/>
-      <c r="DF23" s="5"/>
-      <c r="DG23" s="5"/>
-      <c r="DH23" s="5"/>
-      <c r="DI23" s="5"/>
-      <c r="DJ23" s="5"/>
-      <c r="DK23" s="5"/>
-      <c r="DL23" s="5"/>
-      <c r="DM23" s="5"/>
-      <c r="DN23" s="5"/>
-      <c r="DO23" s="5"/>
-      <c r="DP23" s="5"/>
-      <c r="DQ23" s="5"/>
-      <c r="DR23" s="5"/>
-      <c r="DS23" s="5"/>
-      <c r="DT23" s="5"/>
-      <c r="DU23" s="5"/>
-      <c r="DV23" s="5"/>
-      <c r="DW23" s="5"/>
-      <c r="DX23" s="5"/>
-      <c r="DY23" s="5"/>
-      <c r="DZ23" s="5"/>
-      <c r="EA23" s="5"/>
-      <c r="EB23" s="5"/>
-      <c r="EC23" s="5"/>
-      <c r="ED23" s="5"/>
-      <c r="EE23" s="5"/>
-      <c r="EF23" s="5"/>
-      <c r="EG23" s="5"/>
-      <c r="EH23" s="5"/>
-      <c r="EI23" s="5"/>
-      <c r="EJ23" s="5"/>
-      <c r="EK23" s="5"/>
-      <c r="EL23" s="5"/>
-      <c r="EM23" s="5"/>
-      <c r="EN23" s="5"/>
-      <c r="EO23" s="5"/>
-      <c r="EP23" s="5"/>
-      <c r="EQ23" s="5"/>
-      <c r="ER23" s="5"/>
-      <c r="ES23" s="5"/>
-      <c r="ET23" s="5"/>
-      <c r="EU23" s="5"/>
-      <c r="EV23" s="5"/>
-      <c r="EW23" s="5"/>
-      <c r="EX23" s="5"/>
-      <c r="EY23" s="5"/>
-      <c r="EZ23" s="5"/>
-      <c r="FA23" s="5"/>
-      <c r="FB23" s="5"/>
-      <c r="FC23" s="5"/>
-      <c r="FD23" s="5"/>
-      <c r="FE23" s="5"/>
-      <c r="FF23" s="5"/>
-      <c r="FG23" s="5"/>
-      <c r="FH23" s="5"/>
-      <c r="FI23" s="5"/>
-      <c r="FJ23" s="5"/>
-      <c r="FK23" s="5"/>
-      <c r="FL23" s="5"/>
-      <c r="FM23" s="5"/>
-      <c r="FN23" s="5"/>
-      <c r="FO23" s="5"/>
-      <c r="FP23" s="5"/>
-      <c r="FQ23" s="5"/>
-      <c r="FR23" s="5"/>
-      <c r="FS23" s="5"/>
-      <c r="FT23" s="5"/>
-      <c r="FU23" s="5"/>
-      <c r="FV23" s="5"/>
-      <c r="FW23" s="5"/>
-      <c r="FX23" s="5"/>
-      <c r="FY23" s="5"/>
-      <c r="FZ23" s="5"/>
-      <c r="GA23" s="5"/>
-      <c r="GB23" s="5"/>
-      <c r="GC23" s="5"/>
-      <c r="GD23" s="5"/>
-      <c r="GE23" s="5"/>
-      <c r="GF23" s="5"/>
-      <c r="GG23" s="5"/>
-      <c r="GH23" s="5"/>
-      <c r="GI23" s="5"/>
-      <c r="GJ23" s="5"/>
-      <c r="GK23" s="5"/>
-      <c r="GL23" s="5"/>
-      <c r="GM23" s="5"/>
-      <c r="GN23" s="5"/>
-      <c r="GO23" s="5"/>
-      <c r="GP23" s="5"/>
-      <c r="GQ23" s="5"/>
-      <c r="GR23" s="5"/>
-      <c r="GS23" s="5"/>
-      <c r="GT23" s="5"/>
-      <c r="GU23" s="5"/>
-      <c r="GV23" s="5"/>
-      <c r="GW23" s="5"/>
-      <c r="GX23" s="5"/>
-      <c r="GY23" s="5"/>
-      <c r="GZ23" s="5"/>
-      <c r="HA23" s="5"/>
-      <c r="HB23" s="5"/>
-      <c r="HC23" s="5"/>
-      <c r="HD23" s="5"/>
-      <c r="HE23" s="5"/>
-      <c r="HF23" s="5"/>
-      <c r="HG23" s="5"/>
-      <c r="HH23" s="5"/>
-      <c r="HI23" s="5"/>
-      <c r="HJ23" s="5"/>
-      <c r="HK23" s="5"/>
-      <c r="HL23" s="5"/>
-      <c r="HM23" s="5"/>
-      <c r="HN23" s="5"/>
-      <c r="HO23" s="5"/>
-      <c r="HP23" s="5"/>
-      <c r="HQ23" s="5"/>
-      <c r="HR23" s="5"/>
-      <c r="HS23" s="5"/>
-      <c r="HT23" s="5"/>
-      <c r="HU23" s="5"/>
-      <c r="HV23" s="5"/>
-      <c r="HW23" s="5"/>
-      <c r="HX23" s="5"/>
-      <c r="HY23" s="5"/>
-      <c r="HZ23" s="5"/>
-      <c r="IA23" s="5"/>
-      <c r="IB23" s="5"/>
-      <c r="IC23" s="5"/>
-      <c r="ID23" s="5"/>
-      <c r="IE23" s="5"/>
-      <c r="IF23" s="5"/>
-      <c r="IG23" s="5"/>
-      <c r="IH23" s="5"/>
-      <c r="II23" s="5"/>
-      <c r="IJ23" s="5"/>
-      <c r="IK23" s="5"/>
-      <c r="IL23" s="5"/>
-      <c r="IM23" s="5"/>
-      <c r="IN23" s="5"/>
-      <c r="IO23" s="5"/>
-      <c r="IP23" s="5"/>
-      <c r="IQ23" s="5"/>
-      <c r="IR23" s="5"/>
-      <c r="IS23" s="5"/>
-      <c r="IT23" s="5"/>
-      <c r="IU23" s="5"/>
-      <c r="IV23" s="5"/>
-      <c r="IW23" s="5"/>
-      <c r="IX23" s="5"/>
-      <c r="IY23" s="5"/>
-      <c r="IZ23" s="5"/>
-      <c r="JA23" s="5"/>
-      <c r="JB23" s="5"/>
-      <c r="JC23" s="5"/>
-      <c r="JD23" s="5"/>
-      <c r="JE23" s="5"/>
-      <c r="JF23" s="5"/>
-      <c r="JG23" s="5"/>
-      <c r="JH23" s="5"/>
-      <c r="JI23" s="5"/>
-      <c r="JJ23" s="5"/>
-      <c r="JK23" s="5"/>
-      <c r="JL23" s="5"/>
-      <c r="JM23" s="5"/>
-      <c r="JN23" s="5"/>
-      <c r="JO23" s="5"/>
-      <c r="JP23" s="5"/>
-      <c r="JQ23" s="5"/>
-      <c r="JR23" s="5"/>
-      <c r="JS23" s="5"/>
-      <c r="JT23" s="5"/>
-      <c r="JU23" s="5"/>
-      <c r="JV23" s="5"/>
-      <c r="JW23" s="5"/>
-      <c r="JX23" s="5"/>
-      <c r="JY23" s="5"/>
-      <c r="JZ23" s="5"/>
-      <c r="KA23" s="5"/>
-      <c r="KB23" s="5"/>
-      <c r="KC23" s="5"/>
-      <c r="KD23" s="5"/>
-      <c r="KE23" s="5"/>
-      <c r="KF23" s="5"/>
-      <c r="KG23" s="5"/>
-      <c r="KH23" s="5"/>
-      <c r="KI23" s="5"/>
-      <c r="KJ23" s="5"/>
-      <c r="KK23" s="5"/>
-      <c r="KL23" s="5"/>
-      <c r="KM23" s="5"/>
-      <c r="KN23" s="5"/>
-      <c r="KO23" s="5"/>
-      <c r="KP23" s="5"/>
-      <c r="KQ23" s="5"/>
-      <c r="KR23" s="5"/>
-      <c r="KS23" s="5"/>
-      <c r="KT23" s="5"/>
-      <c r="KU23" s="5"/>
-      <c r="KV23" s="5"/>
-      <c r="KW23" s="5"/>
-      <c r="KX23" s="5"/>
-      <c r="KY23" s="5"/>
-      <c r="KZ23" s="5"/>
-      <c r="LA23" s="5"/>
-      <c r="LB23" s="5"/>
-      <c r="LC23" s="5"/>
-      <c r="LD23" s="5"/>
-      <c r="LE23" s="5"/>
-      <c r="LF23" s="5"/>
-      <c r="LG23" s="5"/>
-      <c r="LH23" s="5"/>
-      <c r="LI23" s="5"/>
-      <c r="LJ23" s="5"/>
-      <c r="LK23" s="5"/>
-      <c r="LL23" s="5"/>
-      <c r="LM23" s="5"/>
-      <c r="LN23" s="5"/>
-      <c r="LO23" s="5"/>
-      <c r="LP23" s="5"/>
-      <c r="LQ23" s="5"/>
-      <c r="LR23" s="5"/>
-      <c r="LS23" s="5"/>
-      <c r="LT23" s="5"/>
-      <c r="LU23" s="5"/>
-      <c r="LV23" s="5"/>
-      <c r="LW23" s="5"/>
-      <c r="LX23" s="5"/>
-      <c r="LY23" s="5"/>
-      <c r="LZ23" s="5"/>
-      <c r="MA23" s="5"/>
-      <c r="MB23" s="5"/>
-      <c r="MC23" s="5"/>
-      <c r="MD23" s="5"/>
-      <c r="ME23" s="5"/>
-      <c r="MF23" s="5"/>
-      <c r="MG23" s="5"/>
-      <c r="MH23" s="5"/>
-      <c r="MI23" s="5"/>
-      <c r="MJ23" s="5"/>
-      <c r="MK23" s="5"/>
-      <c r="ML23" s="5"/>
-      <c r="MM23" s="5"/>
-      <c r="MN23" s="5"/>
-      <c r="MO23" s="5"/>
-      <c r="MP23" s="5"/>
-      <c r="MQ23" s="5"/>
-      <c r="MR23" s="5"/>
-      <c r="MS23" s="5"/>
-      <c r="MT23" s="5"/>
-      <c r="MU23" s="5"/>
-      <c r="MV23" s="5"/>
-      <c r="MW23" s="5"/>
-      <c r="MX23" s="5"/>
-      <c r="MY23" s="5"/>
-      <c r="MZ23" s="5"/>
-      <c r="NA23" s="5"/>
-      <c r="NB23" s="5"/>
-      <c r="NC23" s="5"/>
-      <c r="ND23" s="5"/>
-      <c r="NE23" s="5"/>
-      <c r="NF23" s="5"/>
-      <c r="NG23" s="5"/>
-      <c r="NH23" s="5"/>
-      <c r="NI23" s="5"/>
-      <c r="NJ23" s="5"/>
-      <c r="NK23" s="5"/>
-      <c r="NL23" s="5"/>
-      <c r="NM23" s="5"/>
-      <c r="NN23" s="5"/>
-      <c r="NO23" s="5"/>
-      <c r="NP23" s="5"/>
-      <c r="NQ23" s="5"/>
-      <c r="NR23" s="5"/>
-      <c r="NS23" s="5"/>
-      <c r="NT23" s="5"/>
-      <c r="NU23" s="5"/>
-      <c r="NV23" s="5"/>
-      <c r="NW23" s="5"/>
-      <c r="NX23" s="5"/>
-      <c r="NY23" s="5"/>
-      <c r="NZ23" s="5"/>
-      <c r="OA23" s="5"/>
-      <c r="OB23" s="5"/>
-      <c r="OC23" s="5"/>
-      <c r="OD23" s="5"/>
-      <c r="OE23" s="5"/>
-      <c r="OF23" s="5"/>
-      <c r="OG23" s="5"/>
-      <c r="OH23" s="5"/>
-      <c r="OI23" s="5"/>
-      <c r="OJ23" s="5"/>
-      <c r="OK23" s="5"/>
-      <c r="OL23" s="5"/>
-      <c r="OM23" s="5"/>
-      <c r="ON23" s="5"/>
-      <c r="OO23" s="5"/>
-      <c r="OP23" s="5"/>
-      <c r="OQ23" s="5"/>
-      <c r="OR23" s="5"/>
-      <c r="OS23" s="5"/>
-      <c r="OT23" s="5"/>
-      <c r="OU23" s="5"/>
-      <c r="OV23" s="5"/>
-      <c r="OW23" s="5"/>
-      <c r="OX23" s="5"/>
-      <c r="OY23" s="5"/>
-      <c r="OZ23" s="5"/>
-      <c r="PA23" s="5"/>
-      <c r="PB23" s="5"/>
-      <c r="PC23" s="5"/>
-      <c r="PD23" s="5"/>
-      <c r="PE23" s="5"/>
-      <c r="PF23" s="5"/>
-      <c r="PG23" s="5"/>
-      <c r="PH23" s="5"/>
-      <c r="PI23" s="5"/>
-      <c r="PJ23" s="5"/>
-      <c r="PK23" s="5"/>
-      <c r="PL23" s="5"/>
-      <c r="PM23" s="5"/>
-      <c r="PN23" s="5"/>
-      <c r="PO23" s="5"/>
-      <c r="PP23" s="5"/>
-      <c r="PQ23" s="5"/>
-      <c r="PR23" s="5"/>
-      <c r="PS23" s="5"/>
-      <c r="PT23" s="5"/>
-      <c r="PU23" s="5"/>
-      <c r="PV23" s="5"/>
-      <c r="PW23" s="5"/>
-      <c r="PX23" s="5"/>
-      <c r="PY23" s="5"/>
-      <c r="PZ23" s="5"/>
-      <c r="QA23" s="5"/>
-      <c r="QB23" s="5"/>
-      <c r="QC23" s="5"/>
-      <c r="QD23" s="5"/>
-      <c r="QE23" s="5"/>
-      <c r="QF23" s="5"/>
-      <c r="QG23" s="5"/>
-      <c r="QH23" s="5"/>
-      <c r="QI23" s="5"/>
-      <c r="QJ23" s="5"/>
-      <c r="QK23" s="5"/>
-      <c r="QL23" s="5"/>
-      <c r="QM23" s="5"/>
-      <c r="QN23" s="5"/>
-      <c r="QO23" s="5"/>
-      <c r="QP23" s="5"/>
-      <c r="QQ23" s="5"/>
-      <c r="QR23" s="5"/>
-      <c r="QS23" s="5"/>
-      <c r="QT23" s="5"/>
-      <c r="QU23" s="5"/>
-      <c r="QV23" s="5"/>
-      <c r="QW23" s="5"/>
-      <c r="QX23" s="5"/>
-      <c r="QY23" s="5"/>
-      <c r="QZ23" s="5"/>
-      <c r="RA23" s="5"/>
-      <c r="RB23" s="5"/>
-      <c r="RC23" s="5"/>
-      <c r="RD23" s="5"/>
-      <c r="RE23" s="5"/>
-      <c r="RF23" s="5"/>
-      <c r="RG23" s="5"/>
-      <c r="RH23" s="5"/>
-      <c r="RI23" s="5"/>
-      <c r="RJ23" s="5"/>
-      <c r="RK23" s="5"/>
-      <c r="RL23" s="5"/>
-      <c r="RM23" s="5"/>
-      <c r="RN23" s="5"/>
-      <c r="RO23" s="5"/>
-      <c r="RP23" s="5"/>
-      <c r="RQ23" s="5"/>
-      <c r="RR23" s="5"/>
-      <c r="RS23" s="5"/>
-      <c r="RT23" s="5"/>
-      <c r="RU23" s="5"/>
-      <c r="RV23" s="5"/>
-      <c r="RW23" s="5"/>
-      <c r="RX23" s="5"/>
-      <c r="RY23" s="5"/>
-      <c r="RZ23" s="5"/>
-      <c r="SA23" s="5"/>
-      <c r="SB23" s="5"/>
-      <c r="SC23" s="5"/>
-      <c r="SD23" s="5"/>
-      <c r="SE23" s="5"/>
-      <c r="SF23" s="5"/>
-      <c r="SG23" s="5"/>
-      <c r="SH23" s="5"/>
-      <c r="SI23" s="5"/>
-      <c r="SJ23" s="5"/>
-      <c r="SK23" s="5"/>
-      <c r="SL23" s="5"/>
-      <c r="SM23" s="5"/>
-      <c r="SN23" s="5"/>
-      <c r="SO23" s="5"/>
-      <c r="SP23" s="5"/>
-      <c r="SQ23" s="5"/>
-      <c r="SR23" s="5"/>
-      <c r="SS23" s="5"/>
-      <c r="ST23" s="5"/>
-      <c r="SU23" s="5"/>
-      <c r="SV23" s="5"/>
-      <c r="SW23" s="5"/>
-      <c r="SX23" s="5"/>
-      <c r="SY23" s="5"/>
-      <c r="SZ23" s="5"/>
-      <c r="TA23" s="5"/>
-      <c r="TB23" s="5"/>
-      <c r="TC23" s="5"/>
-      <c r="TD23" s="5"/>
-      <c r="TE23" s="5"/>
-      <c r="TF23" s="5"/>
-      <c r="TG23" s="5"/>
-      <c r="TH23" s="5"/>
-      <c r="TI23" s="5"/>
-      <c r="TJ23" s="5"/>
-      <c r="TK23" s="5"/>
-      <c r="TL23" s="5"/>
-      <c r="TM23" s="5"/>
-      <c r="TN23" s="5"/>
-      <c r="TO23" s="5"/>
-      <c r="TP23" s="5"/>
-      <c r="TQ23" s="5"/>
-      <c r="TR23" s="5"/>
-      <c r="TS23" s="5"/>
-      <c r="TT23" s="5"/>
-      <c r="TU23" s="5"/>
-      <c r="TV23" s="5"/>
-      <c r="TW23" s="5"/>
-      <c r="TX23" s="5"/>
-      <c r="TY23" s="5"/>
-      <c r="TZ23" s="5"/>
-      <c r="UA23" s="5"/>
-      <c r="UB23" s="5"/>
-      <c r="UC23" s="5"/>
-      <c r="UD23" s="5"/>
-      <c r="UE23" s="5"/>
-      <c r="UF23" s="5"/>
-      <c r="UG23" s="5"/>
-      <c r="UH23" s="5"/>
-      <c r="UI23" s="5"/>
-      <c r="UJ23" s="5"/>
-      <c r="UK23" s="5"/>
-      <c r="UL23" s="5"/>
-      <c r="UM23" s="5"/>
-      <c r="UN23" s="5"/>
-      <c r="UO23" s="5"/>
-      <c r="UP23" s="5"/>
-      <c r="UQ23" s="5"/>
-      <c r="UR23" s="5"/>
-      <c r="US23" s="5"/>
-      <c r="UT23" s="5"/>
-      <c r="UU23" s="5"/>
-      <c r="UV23" s="5"/>
-      <c r="UW23" s="5"/>
-      <c r="UX23" s="5"/>
-      <c r="UY23" s="5"/>
-      <c r="UZ23" s="5"/>
-      <c r="VA23" s="5"/>
-      <c r="VB23" s="5"/>
-      <c r="VC23" s="5"/>
-      <c r="VD23" s="5"/>
-      <c r="VE23" s="5"/>
-      <c r="VF23" s="5"/>
-      <c r="VG23" s="5"/>
-      <c r="VH23" s="5"/>
-      <c r="VI23" s="5"/>
-      <c r="VJ23" s="5"/>
-      <c r="VK23" s="5"/>
-      <c r="VL23" s="5"/>
-      <c r="VM23" s="5"/>
-      <c r="VN23" s="5"/>
-      <c r="VO23" s="5"/>
-      <c r="VP23" s="5"/>
-      <c r="VQ23" s="5"/>
-      <c r="VR23" s="5"/>
-      <c r="VS23" s="5"/>
-      <c r="VT23" s="5"/>
-      <c r="VU23" s="5"/>
-      <c r="VV23" s="5"/>
-      <c r="VW23" s="5"/>
-      <c r="VX23" s="5"/>
-      <c r="VY23" s="5"/>
-      <c r="VZ23" s="5"/>
-      <c r="WA23" s="5"/>
-      <c r="WB23" s="5"/>
-      <c r="WC23" s="5"/>
-      <c r="WD23" s="5"/>
-      <c r="WE23" s="5"/>
-      <c r="WF23" s="5"/>
-      <c r="WG23" s="5"/>
-      <c r="WH23" s="5"/>
-      <c r="WI23" s="5"/>
-      <c r="WJ23" s="5"/>
-      <c r="WK23" s="5"/>
-      <c r="WL23" s="5"/>
-      <c r="WM23" s="5"/>
-      <c r="WN23" s="5"/>
-      <c r="WO23" s="5"/>
-      <c r="WP23" s="5"/>
-      <c r="WQ23" s="5"/>
-      <c r="WR23" s="5"/>
-      <c r="WS23" s="5"/>
-      <c r="WT23" s="5"/>
-      <c r="WU23" s="5"/>
-      <c r="WV23" s="5"/>
-      <c r="WW23" s="5"/>
-      <c r="WX23" s="5"/>
-      <c r="WY23" s="5"/>
-      <c r="WZ23" s="5"/>
-      <c r="XA23" s="5"/>
-      <c r="XB23" s="5"/>
-      <c r="XC23" s="5"/>
-      <c r="XD23" s="5"/>
-      <c r="XE23" s="5"/>
-      <c r="XF23" s="5"/>
-      <c r="XG23" s="5"/>
-      <c r="XH23" s="5"/>
-      <c r="XI23" s="5"/>
-      <c r="XJ23" s="5"/>
-      <c r="XK23" s="5"/>
-      <c r="XL23" s="5"/>
-      <c r="XM23" s="5"/>
-      <c r="XN23" s="5"/>
-      <c r="XO23" s="5"/>
-      <c r="XP23" s="5"/>
-      <c r="XQ23" s="5"/>
-      <c r="XR23" s="5"/>
-      <c r="XS23" s="5"/>
-      <c r="XT23" s="5"/>
-      <c r="XU23" s="5"/>
-      <c r="XV23" s="5"/>
-      <c r="XW23" s="5"/>
-      <c r="XX23" s="5"/>
-      <c r="XY23" s="5"/>
-      <c r="XZ23" s="5"/>
-      <c r="YA23" s="5"/>
-      <c r="YB23" s="5"/>
-      <c r="YC23" s="5"/>
-      <c r="YD23" s="5"/>
-      <c r="YE23" s="5"/>
-      <c r="YF23" s="5"/>
-      <c r="YG23" s="5"/>
-      <c r="YH23" s="5"/>
-      <c r="YI23" s="5"/>
-      <c r="YJ23" s="5"/>
-      <c r="YK23" s="5"/>
-      <c r="YL23" s="5"/>
-      <c r="YM23" s="5"/>
-      <c r="YN23" s="5"/>
-      <c r="YO23" s="5"/>
-      <c r="YP23" s="5"/>
-      <c r="YQ23" s="5"/>
-      <c r="YR23" s="5"/>
-      <c r="YS23" s="5"/>
-      <c r="YT23" s="5"/>
-      <c r="YU23" s="5"/>
-      <c r="YV23" s="5"/>
-      <c r="YW23" s="5"/>
-      <c r="YX23" s="5"/>
-      <c r="YY23" s="5"/>
-      <c r="YZ23" s="5"/>
-      <c r="ZA23" s="5"/>
-      <c r="ZB23" s="5"/>
-      <c r="ZC23" s="5"/>
-      <c r="ZD23" s="5"/>
-      <c r="ZE23" s="5"/>
-      <c r="ZF23" s="5"/>
-      <c r="ZG23" s="5"/>
-      <c r="ZH23" s="5"/>
-      <c r="ZI23" s="5"/>
-      <c r="ZJ23" s="5"/>
-      <c r="ZK23" s="5"/>
-      <c r="ZL23" s="5"/>
-      <c r="ZM23" s="5"/>
-      <c r="ZN23" s="5"/>
-      <c r="ZO23" s="5"/>
-      <c r="ZP23" s="5"/>
-      <c r="ZQ23" s="5"/>
-      <c r="ZR23" s="5"/>
-      <c r="ZS23" s="5"/>
-      <c r="ZT23" s="5"/>
-      <c r="ZU23" s="5"/>
-      <c r="ZV23" s="5"/>
-      <c r="ZW23" s="5"/>
-      <c r="ZX23" s="5"/>
-      <c r="ZY23" s="5"/>
-      <c r="ZZ23" s="5"/>
-      <c r="AAA23" s="5"/>
-      <c r="AAB23" s="5"/>
-      <c r="AAC23" s="5"/>
-      <c r="AAD23" s="5"/>
-      <c r="AAE23" s="5"/>
-      <c r="AAF23" s="5"/>
-      <c r="AAG23" s="5"/>
-      <c r="AAH23" s="5"/>
-      <c r="AAI23" s="5"/>
-      <c r="AAJ23" s="5"/>
-      <c r="AAK23" s="5"/>
-      <c r="AAL23" s="5"/>
-      <c r="AAM23" s="5"/>
-      <c r="AAN23" s="5"/>
-      <c r="AAO23" s="5"/>
-      <c r="AAP23" s="5"/>
-      <c r="AAQ23" s="5"/>
-      <c r="AAR23" s="5"/>
-      <c r="AAS23" s="5"/>
-      <c r="AAT23" s="5"/>
-      <c r="AAU23" s="5"/>
-      <c r="AAV23" s="5"/>
-      <c r="AAW23" s="5"/>
-      <c r="AAX23" s="5"/>
-      <c r="AAY23" s="5"/>
-      <c r="AAZ23" s="5"/>
-      <c r="ABA23" s="5"/>
-      <c r="ABB23" s="5"/>
-      <c r="ABC23" s="5"/>
-      <c r="ABD23" s="5"/>
-      <c r="ABE23" s="5"/>
-      <c r="ABF23" s="5"/>
-      <c r="ABG23" s="5"/>
-      <c r="ABH23" s="5"/>
-      <c r="ABI23" s="5"/>
-      <c r="ABJ23" s="5"/>
-      <c r="ABK23" s="5"/>
-      <c r="ABL23" s="5"/>
-      <c r="ABM23" s="5"/>
-      <c r="ABN23" s="5"/>
-      <c r="ABO23" s="5"/>
-      <c r="ABP23" s="5"/>
-      <c r="ABQ23" s="5"/>
-      <c r="ABR23" s="5"/>
-      <c r="ABS23" s="5"/>
-      <c r="ABT23" s="5"/>
-      <c r="ABU23" s="5"/>
-      <c r="ABV23" s="5"/>
-      <c r="ABW23" s="5"/>
-      <c r="ABX23" s="5"/>
-      <c r="ABY23" s="5"/>
-      <c r="ABZ23" s="5"/>
-      <c r="ACA23" s="5"/>
-      <c r="ACB23" s="5"/>
-      <c r="ACC23" s="5"/>
-      <c r="ACD23" s="5"/>
-      <c r="ACE23" s="5"/>
-      <c r="ACF23" s="5"/>
-      <c r="ACG23" s="5"/>
-      <c r="ACH23" s="5"/>
-      <c r="ACI23" s="5"/>
-      <c r="ACJ23" s="5"/>
-      <c r="ACK23" s="5"/>
-      <c r="ACL23" s="5"/>
-      <c r="ACM23" s="5"/>
-      <c r="ACN23" s="5"/>
-      <c r="ACO23" s="5"/>
-      <c r="ACP23" s="5"/>
-      <c r="ACQ23" s="5"/>
-      <c r="ACR23" s="5"/>
-      <c r="ACS23" s="5"/>
-      <c r="ACT23" s="5"/>
-      <c r="ACU23" s="5"/>
-      <c r="ACV23" s="5"/>
-      <c r="ACW23" s="5"/>
-      <c r="ACX23" s="5"/>
-      <c r="ACY23" s="5"/>
-      <c r="ACZ23" s="5"/>
-      <c r="ADA23" s="5"/>
-      <c r="ADB23" s="5"/>
-      <c r="ADC23" s="5"/>
-      <c r="ADD23" s="5"/>
-      <c r="ADE23" s="5"/>
-      <c r="ADF23" s="5"/>
-      <c r="ADG23" s="5"/>
-      <c r="ADH23" s="5"/>
-      <c r="ADI23" s="5"/>
-      <c r="ADJ23" s="5"/>
-      <c r="ADK23" s="5"/>
-      <c r="ADL23" s="5"/>
-      <c r="ADM23" s="5"/>
-      <c r="ADN23" s="5"/>
-      <c r="ADO23" s="5"/>
-      <c r="ADP23" s="5"/>
-      <c r="ADQ23" s="5"/>
-      <c r="ADR23" s="5"/>
-      <c r="ADS23" s="5"/>
-      <c r="ADT23" s="5"/>
-      <c r="ADU23" s="5"/>
-      <c r="ADV23" s="5"/>
-      <c r="ADW23" s="5"/>
-      <c r="ADX23" s="5"/>
-      <c r="ADY23" s="5"/>
-      <c r="ADZ23" s="5"/>
-      <c r="AEA23" s="5"/>
-      <c r="AEB23" s="5"/>
-      <c r="AEC23" s="5"/>
-      <c r="AED23" s="5"/>
-      <c r="AEE23" s="5"/>
-      <c r="AEF23" s="5"/>
-      <c r="AEG23" s="5"/>
-      <c r="AEH23" s="5"/>
-      <c r="AEI23" s="5"/>
-      <c r="AEJ23" s="5"/>
-      <c r="AEK23" s="5"/>
-      <c r="AEL23" s="5"/>
-      <c r="AEM23" s="5"/>
-      <c r="AEN23" s="5"/>
-      <c r="AEO23" s="5"/>
-      <c r="AEP23" s="5"/>
-      <c r="AEQ23" s="5"/>
-      <c r="AER23" s="5"/>
-      <c r="AES23" s="5"/>
-      <c r="AET23" s="5"/>
-      <c r="AEU23" s="5"/>
-      <c r="AEV23" s="5"/>
-      <c r="AEW23" s="5"/>
-      <c r="AEX23" s="5"/>
-      <c r="AEY23" s="5"/>
-      <c r="AEZ23" s="5"/>
-      <c r="AFA23" s="5"/>
-      <c r="AFB23" s="5"/>
-      <c r="AFC23" s="5"/>
-      <c r="AFD23" s="5"/>
-      <c r="AFE23" s="5"/>
-      <c r="AFF23" s="5"/>
-      <c r="AFG23" s="5"/>
-      <c r="AFH23" s="5"/>
-      <c r="AFI23" s="5"/>
-      <c r="AFJ23" s="5"/>
-      <c r="AFK23" s="5"/>
-      <c r="AFL23" s="5"/>
-      <c r="AFM23" s="5"/>
-      <c r="AFN23" s="5"/>
-      <c r="AFO23" s="5"/>
-      <c r="AFP23" s="5"/>
-      <c r="AFQ23" s="5"/>
-      <c r="AFR23" s="5"/>
-      <c r="AFS23" s="5"/>
-      <c r="AFT23" s="5"/>
-      <c r="AFU23" s="5"/>
-      <c r="AFV23" s="5"/>
-      <c r="AFW23" s="5"/>
-      <c r="AFX23" s="5"/>
-      <c r="AFY23" s="5"/>
-      <c r="AFZ23" s="5"/>
-      <c r="AGA23" s="5"/>
-      <c r="AGB23" s="5"/>
-      <c r="AGC23" s="5"/>
-      <c r="AGD23" s="5"/>
-      <c r="AGE23" s="5"/>
-      <c r="AGF23" s="5"/>
-      <c r="AGG23" s="5"/>
-      <c r="AGH23" s="5"/>
-      <c r="AGI23" s="5"/>
-      <c r="AGJ23" s="5"/>
-      <c r="AGK23" s="5"/>
-      <c r="AGL23" s="5"/>
-      <c r="AGM23" s="5"/>
-      <c r="AGN23" s="5"/>
-      <c r="AGO23" s="5"/>
-      <c r="AGP23" s="5"/>
-      <c r="AGQ23" s="5"/>
-      <c r="AGR23" s="5"/>
-      <c r="AGS23" s="5"/>
-      <c r="AGT23" s="5"/>
-      <c r="AGU23" s="5"/>
-      <c r="AGV23" s="5"/>
-      <c r="AGW23" s="5"/>
-      <c r="AGX23" s="5"/>
-      <c r="AGY23" s="5"/>
-      <c r="AGZ23" s="5"/>
-      <c r="AHA23" s="5"/>
-      <c r="AHB23" s="5"/>
-      <c r="AHC23" s="5"/>
-      <c r="AHD23" s="5"/>
-      <c r="AHE23" s="5"/>
-      <c r="AHF23" s="5"/>
-      <c r="AHG23" s="5"/>
-      <c r="AHH23" s="5"/>
-      <c r="AHI23" s="5"/>
-      <c r="AHJ23" s="5"/>
-      <c r="AHK23" s="5"/>
-      <c r="AHL23" s="5"/>
-      <c r="AHM23" s="5"/>
-      <c r="AHN23" s="5"/>
-      <c r="AHO23" s="5"/>
-      <c r="AHP23" s="5"/>
-      <c r="AHQ23" s="5"/>
-      <c r="AHR23" s="5"/>
-      <c r="AHS23" s="5"/>
-      <c r="AHT23" s="5"/>
-      <c r="AHU23" s="5"/>
-      <c r="AHV23" s="5"/>
-      <c r="AHW23" s="5"/>
-      <c r="AHX23" s="5"/>
-      <c r="AHY23" s="5"/>
-      <c r="AHZ23" s="5"/>
-      <c r="AIA23" s="5"/>
-      <c r="AIB23" s="5"/>
-      <c r="AIC23" s="5"/>
-      <c r="AID23" s="5"/>
-      <c r="AIE23" s="5"/>
-      <c r="AIF23" s="5"/>
-      <c r="AIG23" s="5"/>
-      <c r="AIH23" s="5"/>
-      <c r="AII23" s="5"/>
-      <c r="AIJ23" s="5"/>
-      <c r="AIK23" s="5"/>
-      <c r="AIL23" s="5"/>
-      <c r="AIM23" s="5"/>
-      <c r="AIN23" s="5"/>
-      <c r="AIO23" s="5"/>
-      <c r="AIP23" s="5"/>
-      <c r="AIQ23" s="5"/>
-      <c r="AIR23" s="5"/>
-      <c r="AIS23" s="5"/>
-      <c r="AIT23" s="5"/>
-      <c r="AIU23" s="5"/>
-      <c r="AIV23" s="5"/>
-      <c r="AIW23" s="5"/>
-      <c r="AIX23" s="5"/>
-      <c r="AIY23" s="5"/>
-      <c r="AIZ23" s="5"/>
-      <c r="AJA23" s="5"/>
-      <c r="AJB23" s="5"/>
-      <c r="AJC23" s="5"/>
-      <c r="AJD23" s="5"/>
-      <c r="AJE23" s="5"/>
-      <c r="AJF23" s="5"/>
-      <c r="AJG23" s="5"/>
-      <c r="AJH23" s="5"/>
-      <c r="AJI23" s="5"/>
-      <c r="AJJ23" s="5"/>
-      <c r="AJK23" s="5"/>
-      <c r="AJL23" s="5"/>
-      <c r="AJM23" s="5"/>
-      <c r="AJN23" s="5"/>
-      <c r="AJO23" s="5"/>
-      <c r="AJP23" s="5"/>
-      <c r="AJQ23" s="5"/>
-      <c r="AJR23" s="5"/>
-      <c r="AJS23" s="5"/>
-      <c r="AJT23" s="5"/>
-      <c r="AJU23" s="5"/>
-      <c r="AJV23" s="5"/>
-      <c r="AJW23" s="5"/>
-      <c r="AJX23" s="5"/>
-      <c r="AJY23" s="5"/>
-      <c r="AJZ23" s="5"/>
-      <c r="AKA23" s="5"/>
-      <c r="AKB23" s="5"/>
-      <c r="AKC23" s="5"/>
-      <c r="AKD23" s="5"/>
-      <c r="AKE23" s="5"/>
-      <c r="AKF23" s="5"/>
-      <c r="AKG23" s="5"/>
-      <c r="AKH23" s="5"/>
-      <c r="AKI23" s="5"/>
-      <c r="AKJ23" s="5"/>
-      <c r="AKK23" s="5"/>
-      <c r="AKL23" s="5"/>
-      <c r="AKM23" s="5"/>
-      <c r="AKN23" s="5"/>
-      <c r="AKO23" s="5"/>
-      <c r="AKP23" s="5"/>
-      <c r="AKQ23" s="5"/>
-      <c r="AKR23" s="5"/>
-      <c r="AKS23" s="5"/>
-      <c r="AKT23" s="5"/>
-      <c r="AKU23" s="5"/>
-      <c r="AKV23" s="5"/>
-      <c r="AKW23" s="5"/>
-      <c r="AKX23" s="5"/>
-      <c r="AKY23" s="5"/>
-      <c r="AKZ23" s="5"/>
-      <c r="ALA23" s="5"/>
-      <c r="ALB23" s="5"/>
-      <c r="ALC23" s="5"/>
-      <c r="ALD23" s="5"/>
-      <c r="ALE23" s="5"/>
-      <c r="ALF23" s="5"/>
-      <c r="ALG23" s="5"/>
-      <c r="ALH23" s="5"/>
-      <c r="ALI23" s="5"/>
-      <c r="ALJ23" s="5"/>
-      <c r="ALK23" s="5"/>
-      <c r="ALL23" s="5"/>
-      <c r="ALM23" s="5"/>
-      <c r="ALN23" s="5"/>
-      <c r="ALO23" s="5"/>
-      <c r="ALP23" s="5"/>
-      <c r="ALQ23" s="5"/>
-      <c r="ALR23" s="5"/>
-      <c r="ALS23" s="5"/>
-      <c r="ALT23" s="5"/>
-      <c r="ALU23" s="5"/>
-      <c r="ALV23" s="5"/>
-      <c r="ALW23" s="5"/>
-      <c r="ALX23" s="5"/>
-      <c r="ALY23" s="5"/>
-      <c r="ALZ23" s="5"/>
-      <c r="AMA23" s="5"/>
-      <c r="AMB23" s="5"/>
-      <c r="AMC23" s="5"/>
-      <c r="AMD23" s="5"/>
-      <c r="AME23" s="5"/>
-      <c r="AMF23" s="5"/>
-      <c r="AMG23" s="5"/>
-      <c r="AMH23" s="5"/>
-      <c r="AMI23" s="5"/>
-      <c r="AMJ23" s="5"/>
-      <c r="AMK23" s="5"/>
+      <c r="B23" s="77"/>
+    </row>
+    <row r="24" spans="1:1025" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+      <c r="S24" s="5"/>
+      <c r="T24" s="5"/>
+      <c r="U24" s="5"/>
+      <c r="V24" s="5"/>
+      <c r="W24" s="5"/>
+      <c r="X24" s="5"/>
+      <c r="Y24" s="5"/>
+      <c r="Z24" s="5"/>
+      <c r="AA24" s="5"/>
+      <c r="AB24" s="5"/>
+      <c r="AC24" s="5"/>
+      <c r="AD24" s="5"/>
+      <c r="AE24" s="5"/>
+      <c r="AF24" s="5"/>
+      <c r="AG24" s="5"/>
+      <c r="AH24" s="5"/>
+      <c r="AI24" s="5"/>
+      <c r="AJ24" s="5"/>
+      <c r="AK24" s="5"/>
+      <c r="AL24" s="5"/>
+      <c r="AM24" s="5"/>
+      <c r="AN24" s="5"/>
+      <c r="AO24" s="5"/>
+      <c r="AP24" s="5"/>
+      <c r="AQ24" s="5"/>
+      <c r="AR24" s="5"/>
+      <c r="AS24" s="5"/>
+      <c r="AT24" s="5"/>
+      <c r="AU24" s="5"/>
+      <c r="AV24" s="5"/>
+      <c r="AW24" s="5"/>
+      <c r="AX24" s="5"/>
+      <c r="AY24" s="5"/>
+      <c r="AZ24" s="5"/>
+      <c r="BA24" s="5"/>
+      <c r="BB24" s="5"/>
+      <c r="BC24" s="5"/>
+      <c r="BD24" s="5"/>
+      <c r="BE24" s="5"/>
+      <c r="BF24" s="5"/>
+      <c r="BG24" s="5"/>
+      <c r="BH24" s="5"/>
+      <c r="BI24" s="5"/>
+      <c r="BJ24" s="5"/>
+      <c r="BK24" s="5"/>
+      <c r="BL24" s="5"/>
+      <c r="BM24" s="5"/>
+      <c r="BN24" s="5"/>
+      <c r="BO24" s="5"/>
+      <c r="BP24" s="5"/>
+      <c r="BQ24" s="5"/>
+      <c r="BR24" s="5"/>
+      <c r="BS24" s="5"/>
+      <c r="BT24" s="5"/>
+      <c r="BU24" s="5"/>
+      <c r="BV24" s="5"/>
+      <c r="BW24" s="5"/>
+      <c r="BX24" s="5"/>
+      <c r="BY24" s="5"/>
+      <c r="BZ24" s="5"/>
+      <c r="CA24" s="5"/>
+      <c r="CB24" s="5"/>
+      <c r="CC24" s="5"/>
+      <c r="CD24" s="5"/>
+      <c r="CE24" s="5"/>
+      <c r="CF24" s="5"/>
+      <c r="CG24" s="5"/>
+      <c r="CH24" s="5"/>
+      <c r="CI24" s="5"/>
+      <c r="CJ24" s="5"/>
+      <c r="CK24" s="5"/>
+      <c r="CL24" s="5"/>
+      <c r="CM24" s="5"/>
+      <c r="CN24" s="5"/>
+      <c r="CO24" s="5"/>
+      <c r="CP24" s="5"/>
+      <c r="CQ24" s="5"/>
+      <c r="CR24" s="5"/>
+      <c r="CS24" s="5"/>
+      <c r="CT24" s="5"/>
+      <c r="CU24" s="5"/>
+      <c r="CV24" s="5"/>
+      <c r="CW24" s="5"/>
+      <c r="CX24" s="5"/>
+      <c r="CY24" s="5"/>
+      <c r="CZ24" s="5"/>
+      <c r="DA24" s="5"/>
+      <c r="DB24" s="5"/>
+      <c r="DC24" s="5"/>
+      <c r="DD24" s="5"/>
+      <c r="DE24" s="5"/>
+      <c r="DF24" s="5"/>
+      <c r="DG24" s="5"/>
+      <c r="DH24" s="5"/>
+      <c r="DI24" s="5"/>
+      <c r="DJ24" s="5"/>
+      <c r="DK24" s="5"/>
+      <c r="DL24" s="5"/>
+      <c r="DM24" s="5"/>
+      <c r="DN24" s="5"/>
+      <c r="DO24" s="5"/>
+      <c r="DP24" s="5"/>
+      <c r="DQ24" s="5"/>
+      <c r="DR24" s="5"/>
+      <c r="DS24" s="5"/>
+      <c r="DT24" s="5"/>
+      <c r="DU24" s="5"/>
+      <c r="DV24" s="5"/>
+      <c r="DW24" s="5"/>
+      <c r="DX24" s="5"/>
+      <c r="DY24" s="5"/>
+      <c r="DZ24" s="5"/>
+      <c r="EA24" s="5"/>
+      <c r="EB24" s="5"/>
+      <c r="EC24" s="5"/>
+      <c r="ED24" s="5"/>
+      <c r="EE24" s="5"/>
+      <c r="EF24" s="5"/>
+      <c r="EG24" s="5"/>
+      <c r="EH24" s="5"/>
+      <c r="EI24" s="5"/>
+      <c r="EJ24" s="5"/>
+      <c r="EK24" s="5"/>
+      <c r="EL24" s="5"/>
+      <c r="EM24" s="5"/>
+      <c r="EN24" s="5"/>
+      <c r="EO24" s="5"/>
+      <c r="EP24" s="5"/>
+      <c r="EQ24" s="5"/>
+      <c r="ER24" s="5"/>
+      <c r="ES24" s="5"/>
+      <c r="ET24" s="5"/>
+      <c r="EU24" s="5"/>
+      <c r="EV24" s="5"/>
+      <c r="EW24" s="5"/>
+      <c r="EX24" s="5"/>
+      <c r="EY24" s="5"/>
+      <c r="EZ24" s="5"/>
+      <c r="FA24" s="5"/>
+      <c r="FB24" s="5"/>
+      <c r="FC24" s="5"/>
+      <c r="FD24" s="5"/>
+      <c r="FE24" s="5"/>
+      <c r="FF24" s="5"/>
+      <c r="FG24" s="5"/>
+      <c r="FH24" s="5"/>
+      <c r="FI24" s="5"/>
+      <c r="FJ24" s="5"/>
+      <c r="FK24" s="5"/>
+      <c r="FL24" s="5"/>
+      <c r="FM24" s="5"/>
+      <c r="FN24" s="5"/>
+      <c r="FO24" s="5"/>
+      <c r="FP24" s="5"/>
+      <c r="FQ24" s="5"/>
+      <c r="FR24" s="5"/>
+      <c r="FS24" s="5"/>
+      <c r="FT24" s="5"/>
+      <c r="FU24" s="5"/>
+      <c r="FV24" s="5"/>
+      <c r="FW24" s="5"/>
+      <c r="FX24" s="5"/>
+      <c r="FY24" s="5"/>
+      <c r="FZ24" s="5"/>
+      <c r="GA24" s="5"/>
+      <c r="GB24" s="5"/>
+      <c r="GC24" s="5"/>
+      <c r="GD24" s="5"/>
+      <c r="GE24" s="5"/>
+      <c r="GF24" s="5"/>
+      <c r="GG24" s="5"/>
+      <c r="GH24" s="5"/>
+      <c r="GI24" s="5"/>
+      <c r="GJ24" s="5"/>
+      <c r="GK24" s="5"/>
+      <c r="GL24" s="5"/>
+      <c r="GM24" s="5"/>
+      <c r="GN24" s="5"/>
+      <c r="GO24" s="5"/>
+      <c r="GP24" s="5"/>
+      <c r="GQ24" s="5"/>
+      <c r="GR24" s="5"/>
+      <c r="GS24" s="5"/>
+      <c r="GT24" s="5"/>
+      <c r="GU24" s="5"/>
+      <c r="GV24" s="5"/>
+      <c r="GW24" s="5"/>
+      <c r="GX24" s="5"/>
+      <c r="GY24" s="5"/>
+      <c r="GZ24" s="5"/>
+      <c r="HA24" s="5"/>
+      <c r="HB24" s="5"/>
+      <c r="HC24" s="5"/>
+      <c r="HD24" s="5"/>
+      <c r="HE24" s="5"/>
+      <c r="HF24" s="5"/>
+      <c r="HG24" s="5"/>
+      <c r="HH24" s="5"/>
+      <c r="HI24" s="5"/>
+      <c r="HJ24" s="5"/>
+      <c r="HK24" s="5"/>
+      <c r="HL24" s="5"/>
+      <c r="HM24" s="5"/>
+      <c r="HN24" s="5"/>
+      <c r="HO24" s="5"/>
+      <c r="HP24" s="5"/>
+      <c r="HQ24" s="5"/>
+      <c r="HR24" s="5"/>
+      <c r="HS24" s="5"/>
+      <c r="HT24" s="5"/>
+      <c r="HU24" s="5"/>
+      <c r="HV24" s="5"/>
+      <c r="HW24" s="5"/>
+      <c r="HX24" s="5"/>
+      <c r="HY24" s="5"/>
+      <c r="HZ24" s="5"/>
+      <c r="IA24" s="5"/>
+      <c r="IB24" s="5"/>
+      <c r="IC24" s="5"/>
+      <c r="ID24" s="5"/>
+      <c r="IE24" s="5"/>
+      <c r="IF24" s="5"/>
+      <c r="IG24" s="5"/>
+      <c r="IH24" s="5"/>
+      <c r="II24" s="5"/>
+      <c r="IJ24" s="5"/>
+      <c r="IK24" s="5"/>
+      <c r="IL24" s="5"/>
+      <c r="IM24" s="5"/>
+      <c r="IN24" s="5"/>
+      <c r="IO24" s="5"/>
+      <c r="IP24" s="5"/>
+      <c r="IQ24" s="5"/>
+      <c r="IR24" s="5"/>
+      <c r="IS24" s="5"/>
+      <c r="IT24" s="5"/>
+      <c r="IU24" s="5"/>
+      <c r="IV24" s="5"/>
+      <c r="IW24" s="5"/>
+      <c r="IX24" s="5"/>
+      <c r="IY24" s="5"/>
+      <c r="IZ24" s="5"/>
+      <c r="JA24" s="5"/>
+      <c r="JB24" s="5"/>
+      <c r="JC24" s="5"/>
+      <c r="JD24" s="5"/>
+      <c r="JE24" s="5"/>
+      <c r="JF24" s="5"/>
+      <c r="JG24" s="5"/>
+      <c r="JH24" s="5"/>
+      <c r="JI24" s="5"/>
+      <c r="JJ24" s="5"/>
+      <c r="JK24" s="5"/>
+      <c r="JL24" s="5"/>
+      <c r="JM24" s="5"/>
+      <c r="JN24" s="5"/>
+      <c r="JO24" s="5"/>
+      <c r="JP24" s="5"/>
+      <c r="JQ24" s="5"/>
+      <c r="JR24" s="5"/>
+      <c r="JS24" s="5"/>
+      <c r="JT24" s="5"/>
+      <c r="JU24" s="5"/>
+      <c r="JV24" s="5"/>
+      <c r="JW24" s="5"/>
+      <c r="JX24" s="5"/>
+      <c r="JY24" s="5"/>
+      <c r="JZ24" s="5"/>
+      <c r="KA24" s="5"/>
+      <c r="KB24" s="5"/>
+      <c r="KC24" s="5"/>
+      <c r="KD24" s="5"/>
+      <c r="KE24" s="5"/>
+      <c r="KF24" s="5"/>
+      <c r="KG24" s="5"/>
+      <c r="KH24" s="5"/>
+      <c r="KI24" s="5"/>
+      <c r="KJ24" s="5"/>
+      <c r="KK24" s="5"/>
+      <c r="KL24" s="5"/>
+      <c r="KM24" s="5"/>
+      <c r="KN24" s="5"/>
+      <c r="KO24" s="5"/>
+      <c r="KP24" s="5"/>
+      <c r="KQ24" s="5"/>
+      <c r="KR24" s="5"/>
+      <c r="KS24" s="5"/>
+      <c r="KT24" s="5"/>
+      <c r="KU24" s="5"/>
+      <c r="KV24" s="5"/>
+      <c r="KW24" s="5"/>
+      <c r="KX24" s="5"/>
+      <c r="KY24" s="5"/>
+      <c r="KZ24" s="5"/>
+      <c r="LA24" s="5"/>
+      <c r="LB24" s="5"/>
+      <c r="LC24" s="5"/>
+      <c r="LD24" s="5"/>
+      <c r="LE24" s="5"/>
+      <c r="LF24" s="5"/>
+      <c r="LG24" s="5"/>
+      <c r="LH24" s="5"/>
+      <c r="LI24" s="5"/>
+      <c r="LJ24" s="5"/>
+      <c r="LK24" s="5"/>
+      <c r="LL24" s="5"/>
+      <c r="LM24" s="5"/>
+      <c r="LN24" s="5"/>
+      <c r="LO24" s="5"/>
+      <c r="LP24" s="5"/>
+      <c r="LQ24" s="5"/>
+      <c r="LR24" s="5"/>
+      <c r="LS24" s="5"/>
+      <c r="LT24" s="5"/>
+      <c r="LU24" s="5"/>
+      <c r="LV24" s="5"/>
+      <c r="LW24" s="5"/>
+      <c r="LX24" s="5"/>
+      <c r="LY24" s="5"/>
+      <c r="LZ24" s="5"/>
+      <c r="MA24" s="5"/>
+      <c r="MB24" s="5"/>
+      <c r="MC24" s="5"/>
+      <c r="MD24" s="5"/>
+      <c r="ME24" s="5"/>
+      <c r="MF24" s="5"/>
+      <c r="MG24" s="5"/>
+      <c r="MH24" s="5"/>
+      <c r="MI24" s="5"/>
+      <c r="MJ24" s="5"/>
+      <c r="MK24" s="5"/>
+      <c r="ML24" s="5"/>
+      <c r="MM24" s="5"/>
+      <c r="MN24" s="5"/>
+      <c r="MO24" s="5"/>
+      <c r="MP24" s="5"/>
+      <c r="MQ24" s="5"/>
+      <c r="MR24" s="5"/>
+      <c r="MS24" s="5"/>
+      <c r="MT24" s="5"/>
+      <c r="MU24" s="5"/>
+      <c r="MV24" s="5"/>
+      <c r="MW24" s="5"/>
+      <c r="MX24" s="5"/>
+      <c r="MY24" s="5"/>
+      <c r="MZ24" s="5"/>
+      <c r="NA24" s="5"/>
+      <c r="NB24" s="5"/>
+      <c r="NC24" s="5"/>
+      <c r="ND24" s="5"/>
+      <c r="NE24" s="5"/>
+      <c r="NF24" s="5"/>
+      <c r="NG24" s="5"/>
+      <c r="NH24" s="5"/>
+      <c r="NI24" s="5"/>
+      <c r="NJ24" s="5"/>
+      <c r="NK24" s="5"/>
+      <c r="NL24" s="5"/>
+      <c r="NM24" s="5"/>
+      <c r="NN24" s="5"/>
+      <c r="NO24" s="5"/>
+      <c r="NP24" s="5"/>
+      <c r="NQ24" s="5"/>
+      <c r="NR24" s="5"/>
+      <c r="NS24" s="5"/>
+      <c r="NT24" s="5"/>
+      <c r="NU24" s="5"/>
+      <c r="NV24" s="5"/>
+      <c r="NW24" s="5"/>
+      <c r="NX24" s="5"/>
+      <c r="NY24" s="5"/>
+      <c r="NZ24" s="5"/>
+      <c r="OA24" s="5"/>
+      <c r="OB24" s="5"/>
+      <c r="OC24" s="5"/>
+      <c r="OD24" s="5"/>
+      <c r="OE24" s="5"/>
+      <c r="OF24" s="5"/>
+      <c r="OG24" s="5"/>
+      <c r="OH24" s="5"/>
+      <c r="OI24" s="5"/>
+      <c r="OJ24" s="5"/>
+      <c r="OK24" s="5"/>
+      <c r="OL24" s="5"/>
+      <c r="OM24" s="5"/>
+      <c r="ON24" s="5"/>
+      <c r="OO24" s="5"/>
+      <c r="OP24" s="5"/>
+      <c r="OQ24" s="5"/>
+      <c r="OR24" s="5"/>
+      <c r="OS24" s="5"/>
+      <c r="OT24" s="5"/>
+      <c r="OU24" s="5"/>
+      <c r="OV24" s="5"/>
+      <c r="OW24" s="5"/>
+      <c r="OX24" s="5"/>
+      <c r="OY24" s="5"/>
+      <c r="OZ24" s="5"/>
+      <c r="PA24" s="5"/>
+      <c r="PB24" s="5"/>
+      <c r="PC24" s="5"/>
+      <c r="PD24" s="5"/>
+      <c r="PE24" s="5"/>
+      <c r="PF24" s="5"/>
+      <c r="PG24" s="5"/>
+      <c r="PH24" s="5"/>
+      <c r="PI24" s="5"/>
+      <c r="PJ24" s="5"/>
+      <c r="PK24" s="5"/>
+      <c r="PL24" s="5"/>
+      <c r="PM24" s="5"/>
+      <c r="PN24" s="5"/>
+      <c r="PO24" s="5"/>
+      <c r="PP24" s="5"/>
+      <c r="PQ24" s="5"/>
+      <c r="PR24" s="5"/>
+      <c r="PS24" s="5"/>
+      <c r="PT24" s="5"/>
+      <c r="PU24" s="5"/>
+      <c r="PV24" s="5"/>
+      <c r="PW24" s="5"/>
+      <c r="PX24" s="5"/>
+      <c r="PY24" s="5"/>
+      <c r="PZ24" s="5"/>
+      <c r="QA24" s="5"/>
+      <c r="QB24" s="5"/>
+      <c r="QC24" s="5"/>
+      <c r="QD24" s="5"/>
+      <c r="QE24" s="5"/>
+      <c r="QF24" s="5"/>
+      <c r="QG24" s="5"/>
+      <c r="QH24" s="5"/>
+      <c r="QI24" s="5"/>
+      <c r="QJ24" s="5"/>
+      <c r="QK24" s="5"/>
+      <c r="QL24" s="5"/>
+      <c r="QM24" s="5"/>
+      <c r="QN24" s="5"/>
+      <c r="QO24" s="5"/>
+      <c r="QP24" s="5"/>
+      <c r="QQ24" s="5"/>
+      <c r="QR24" s="5"/>
+      <c r="QS24" s="5"/>
+      <c r="QT24" s="5"/>
+      <c r="QU24" s="5"/>
+      <c r="QV24" s="5"/>
+      <c r="QW24" s="5"/>
+      <c r="QX24" s="5"/>
+      <c r="QY24" s="5"/>
+      <c r="QZ24" s="5"/>
+      <c r="RA24" s="5"/>
+      <c r="RB24" s="5"/>
+      <c r="RC24" s="5"/>
+      <c r="RD24" s="5"/>
+      <c r="RE24" s="5"/>
+      <c r="RF24" s="5"/>
+      <c r="RG24" s="5"/>
+      <c r="RH24" s="5"/>
+      <c r="RI24" s="5"/>
+      <c r="RJ24" s="5"/>
+      <c r="RK24" s="5"/>
+      <c r="RL24" s="5"/>
+      <c r="RM24" s="5"/>
+      <c r="RN24" s="5"/>
+      <c r="RO24" s="5"/>
+      <c r="RP24" s="5"/>
+      <c r="RQ24" s="5"/>
+      <c r="RR24" s="5"/>
+      <c r="RS24" s="5"/>
+      <c r="RT24" s="5"/>
+      <c r="RU24" s="5"/>
+      <c r="RV24" s="5"/>
+      <c r="RW24" s="5"/>
+      <c r="RX24" s="5"/>
+      <c r="RY24" s="5"/>
+      <c r="RZ24" s="5"/>
+      <c r="SA24" s="5"/>
+      <c r="SB24" s="5"/>
+      <c r="SC24" s="5"/>
+      <c r="SD24" s="5"/>
+      <c r="SE24" s="5"/>
+      <c r="SF24" s="5"/>
+      <c r="SG24" s="5"/>
+      <c r="SH24" s="5"/>
+      <c r="SI24" s="5"/>
+      <c r="SJ24" s="5"/>
+      <c r="SK24" s="5"/>
+      <c r="SL24" s="5"/>
+      <c r="SM24" s="5"/>
+      <c r="SN24" s="5"/>
+      <c r="SO24" s="5"/>
+      <c r="SP24" s="5"/>
+      <c r="SQ24" s="5"/>
+      <c r="SR24" s="5"/>
+      <c r="SS24" s="5"/>
+      <c r="ST24" s="5"/>
+      <c r="SU24" s="5"/>
+      <c r="SV24" s="5"/>
+      <c r="SW24" s="5"/>
+      <c r="SX24" s="5"/>
+      <c r="SY24" s="5"/>
+      <c r="SZ24" s="5"/>
+      <c r="TA24" s="5"/>
+      <c r="TB24" s="5"/>
+      <c r="TC24" s="5"/>
+      <c r="TD24" s="5"/>
+      <c r="TE24" s="5"/>
+      <c r="TF24" s="5"/>
+      <c r="TG24" s="5"/>
+      <c r="TH24" s="5"/>
+      <c r="TI24" s="5"/>
+      <c r="TJ24" s="5"/>
+      <c r="TK24" s="5"/>
+      <c r="TL24" s="5"/>
+      <c r="TM24" s="5"/>
+      <c r="TN24" s="5"/>
+      <c r="TO24" s="5"/>
+      <c r="TP24" s="5"/>
+      <c r="TQ24" s="5"/>
+      <c r="TR24" s="5"/>
+      <c r="TS24" s="5"/>
+      <c r="TT24" s="5"/>
+      <c r="TU24" s="5"/>
+      <c r="TV24" s="5"/>
+      <c r="TW24" s="5"/>
+      <c r="TX24" s="5"/>
+      <c r="TY24" s="5"/>
+      <c r="TZ24" s="5"/>
+      <c r="UA24" s="5"/>
+      <c r="UB24" s="5"/>
+      <c r="UC24" s="5"/>
+      <c r="UD24" s="5"/>
+      <c r="UE24" s="5"/>
+      <c r="UF24" s="5"/>
+      <c r="UG24" s="5"/>
+      <c r="UH24" s="5"/>
+      <c r="UI24" s="5"/>
+      <c r="UJ24" s="5"/>
+      <c r="UK24" s="5"/>
+      <c r="UL24" s="5"/>
+      <c r="UM24" s="5"/>
+      <c r="UN24" s="5"/>
+      <c r="UO24" s="5"/>
+      <c r="UP24" s="5"/>
+      <c r="UQ24" s="5"/>
+      <c r="UR24" s="5"/>
+      <c r="US24" s="5"/>
+      <c r="UT24" s="5"/>
+      <c r="UU24" s="5"/>
+      <c r="UV24" s="5"/>
+      <c r="UW24" s="5"/>
+      <c r="UX24" s="5"/>
+      <c r="UY24" s="5"/>
+      <c r="UZ24" s="5"/>
+      <c r="VA24" s="5"/>
+      <c r="VB24" s="5"/>
+      <c r="VC24" s="5"/>
+      <c r="VD24" s="5"/>
+      <c r="VE24" s="5"/>
+      <c r="VF24" s="5"/>
+      <c r="VG24" s="5"/>
+      <c r="VH24" s="5"/>
+      <c r="VI24" s="5"/>
+      <c r="VJ24" s="5"/>
+      <c r="VK24" s="5"/>
+      <c r="VL24" s="5"/>
+      <c r="VM24" s="5"/>
+      <c r="VN24" s="5"/>
+      <c r="VO24" s="5"/>
+      <c r="VP24" s="5"/>
+      <c r="VQ24" s="5"/>
+      <c r="VR24" s="5"/>
+      <c r="VS24" s="5"/>
+      <c r="VT24" s="5"/>
+      <c r="VU24" s="5"/>
+      <c r="VV24" s="5"/>
+      <c r="VW24" s="5"/>
+      <c r="VX24" s="5"/>
+      <c r="VY24" s="5"/>
+      <c r="VZ24" s="5"/>
+      <c r="WA24" s="5"/>
+      <c r="WB24" s="5"/>
+      <c r="WC24" s="5"/>
+      <c r="WD24" s="5"/>
+      <c r="WE24" s="5"/>
+      <c r="WF24" s="5"/>
+      <c r="WG24" s="5"/>
+      <c r="WH24" s="5"/>
+      <c r="WI24" s="5"/>
+      <c r="WJ24" s="5"/>
+      <c r="WK24" s="5"/>
+      <c r="WL24" s="5"/>
+      <c r="WM24" s="5"/>
+      <c r="WN24" s="5"/>
+      <c r="WO24" s="5"/>
+      <c r="WP24" s="5"/>
+      <c r="WQ24" s="5"/>
+      <c r="WR24" s="5"/>
+      <c r="WS24" s="5"/>
+      <c r="WT24" s="5"/>
+      <c r="WU24" s="5"/>
+      <c r="WV24" s="5"/>
+      <c r="WW24" s="5"/>
+      <c r="WX24" s="5"/>
+      <c r="WY24" s="5"/>
+      <c r="WZ24" s="5"/>
+      <c r="XA24" s="5"/>
+      <c r="XB24" s="5"/>
+      <c r="XC24" s="5"/>
+      <c r="XD24" s="5"/>
+      <c r="XE24" s="5"/>
+      <c r="XF24" s="5"/>
+      <c r="XG24" s="5"/>
+      <c r="XH24" s="5"/>
+      <c r="XI24" s="5"/>
+      <c r="XJ24" s="5"/>
+      <c r="XK24" s="5"/>
+      <c r="XL24" s="5"/>
+      <c r="XM24" s="5"/>
+      <c r="XN24" s="5"/>
+      <c r="XO24" s="5"/>
+      <c r="XP24" s="5"/>
+      <c r="XQ24" s="5"/>
+      <c r="XR24" s="5"/>
+      <c r="XS24" s="5"/>
+      <c r="XT24" s="5"/>
+      <c r="XU24" s="5"/>
+      <c r="XV24" s="5"/>
+      <c r="XW24" s="5"/>
+      <c r="XX24" s="5"/>
+      <c r="XY24" s="5"/>
+      <c r="XZ24" s="5"/>
+      <c r="YA24" s="5"/>
+      <c r="YB24" s="5"/>
+      <c r="YC24" s="5"/>
+      <c r="YD24" s="5"/>
+      <c r="YE24" s="5"/>
+      <c r="YF24" s="5"/>
+      <c r="YG24" s="5"/>
+      <c r="YH24" s="5"/>
+      <c r="YI24" s="5"/>
+      <c r="YJ24" s="5"/>
+      <c r="YK24" s="5"/>
+      <c r="YL24" s="5"/>
+      <c r="YM24" s="5"/>
+      <c r="YN24" s="5"/>
+      <c r="YO24" s="5"/>
+      <c r="YP24" s="5"/>
+      <c r="YQ24" s="5"/>
+      <c r="YR24" s="5"/>
+      <c r="YS24" s="5"/>
+      <c r="YT24" s="5"/>
+      <c r="YU24" s="5"/>
+      <c r="YV24" s="5"/>
+      <c r="YW24" s="5"/>
+      <c r="YX24" s="5"/>
+      <c r="YY24" s="5"/>
+      <c r="YZ24" s="5"/>
+      <c r="ZA24" s="5"/>
+      <c r="ZB24" s="5"/>
+      <c r="ZC24" s="5"/>
+      <c r="ZD24" s="5"/>
+      <c r="ZE24" s="5"/>
+      <c r="ZF24" s="5"/>
+      <c r="ZG24" s="5"/>
+      <c r="ZH24" s="5"/>
+      <c r="ZI24" s="5"/>
+      <c r="ZJ24" s="5"/>
+      <c r="ZK24" s="5"/>
+      <c r="ZL24" s="5"/>
+      <c r="ZM24" s="5"/>
+      <c r="ZN24" s="5"/>
+      <c r="ZO24" s="5"/>
+      <c r="ZP24" s="5"/>
+      <c r="ZQ24" s="5"/>
+      <c r="ZR24" s="5"/>
+      <c r="ZS24" s="5"/>
+      <c r="ZT24" s="5"/>
+      <c r="ZU24" s="5"/>
+      <c r="ZV24" s="5"/>
+      <c r="ZW24" s="5"/>
+      <c r="ZX24" s="5"/>
+      <c r="ZY24" s="5"/>
+      <c r="ZZ24" s="5"/>
+      <c r="AAA24" s="5"/>
+      <c r="AAB24" s="5"/>
+      <c r="AAC24" s="5"/>
+      <c r="AAD24" s="5"/>
+      <c r="AAE24" s="5"/>
+      <c r="AAF24" s="5"/>
+      <c r="AAG24" s="5"/>
+      <c r="AAH24" s="5"/>
+      <c r="AAI24" s="5"/>
+      <c r="AAJ24" s="5"/>
+      <c r="AAK24" s="5"/>
+      <c r="AAL24" s="5"/>
+      <c r="AAM24" s="5"/>
+      <c r="AAN24" s="5"/>
+      <c r="AAO24" s="5"/>
+      <c r="AAP24" s="5"/>
+      <c r="AAQ24" s="5"/>
+      <c r="AAR24" s="5"/>
+      <c r="AAS24" s="5"/>
+      <c r="AAT24" s="5"/>
+      <c r="AAU24" s="5"/>
+      <c r="AAV24" s="5"/>
+      <c r="AAW24" s="5"/>
+      <c r="AAX24" s="5"/>
+      <c r="AAY24" s="5"/>
+      <c r="AAZ24" s="5"/>
+      <c r="ABA24" s="5"/>
+      <c r="ABB24" s="5"/>
+      <c r="ABC24" s="5"/>
+      <c r="ABD24" s="5"/>
+      <c r="ABE24" s="5"/>
+      <c r="ABF24" s="5"/>
+      <c r="ABG24" s="5"/>
+      <c r="ABH24" s="5"/>
+      <c r="ABI24" s="5"/>
+      <c r="ABJ24" s="5"/>
+      <c r="ABK24" s="5"/>
+      <c r="ABL24" s="5"/>
+      <c r="ABM24" s="5"/>
+      <c r="ABN24" s="5"/>
+      <c r="ABO24" s="5"/>
+      <c r="ABP24" s="5"/>
+      <c r="ABQ24" s="5"/>
+      <c r="ABR24" s="5"/>
+      <c r="ABS24" s="5"/>
+      <c r="ABT24" s="5"/>
+      <c r="ABU24" s="5"/>
+      <c r="ABV24" s="5"/>
+      <c r="ABW24" s="5"/>
+      <c r="ABX24" s="5"/>
+      <c r="ABY24" s="5"/>
+      <c r="ABZ24" s="5"/>
+      <c r="ACA24" s="5"/>
+      <c r="ACB24" s="5"/>
+      <c r="ACC24" s="5"/>
+      <c r="ACD24" s="5"/>
+      <c r="ACE24" s="5"/>
+      <c r="ACF24" s="5"/>
+      <c r="ACG24" s="5"/>
+      <c r="ACH24" s="5"/>
+      <c r="ACI24" s="5"/>
+      <c r="ACJ24" s="5"/>
+      <c r="ACK24" s="5"/>
+      <c r="ACL24" s="5"/>
+      <c r="ACM24" s="5"/>
+      <c r="ACN24" s="5"/>
+      <c r="ACO24" s="5"/>
+      <c r="ACP24" s="5"/>
+      <c r="ACQ24" s="5"/>
+      <c r="ACR24" s="5"/>
+      <c r="ACS24" s="5"/>
+      <c r="ACT24" s="5"/>
+      <c r="ACU24" s="5"/>
+      <c r="ACV24" s="5"/>
+      <c r="ACW24" s="5"/>
+      <c r="ACX24" s="5"/>
+      <c r="ACY24" s="5"/>
+      <c r="ACZ24" s="5"/>
+      <c r="ADA24" s="5"/>
+      <c r="ADB24" s="5"/>
+      <c r="ADC24" s="5"/>
+      <c r="ADD24" s="5"/>
+      <c r="ADE24" s="5"/>
+      <c r="ADF24" s="5"/>
+      <c r="ADG24" s="5"/>
+      <c r="ADH24" s="5"/>
+      <c r="ADI24" s="5"/>
+      <c r="ADJ24" s="5"/>
+      <c r="ADK24" s="5"/>
+      <c r="ADL24" s="5"/>
+      <c r="ADM24" s="5"/>
+      <c r="ADN24" s="5"/>
+      <c r="ADO24" s="5"/>
+      <c r="ADP24" s="5"/>
+      <c r="ADQ24" s="5"/>
+      <c r="ADR24" s="5"/>
+      <c r="ADS24" s="5"/>
+      <c r="ADT24" s="5"/>
+      <c r="ADU24" s="5"/>
+      <c r="ADV24" s="5"/>
+      <c r="ADW24" s="5"/>
+      <c r="ADX24" s="5"/>
+      <c r="ADY24" s="5"/>
+      <c r="ADZ24" s="5"/>
+      <c r="AEA24" s="5"/>
+      <c r="AEB24" s="5"/>
+      <c r="AEC24" s="5"/>
+      <c r="AED24" s="5"/>
+      <c r="AEE24" s="5"/>
+      <c r="AEF24" s="5"/>
+      <c r="AEG24" s="5"/>
+      <c r="AEH24" s="5"/>
+      <c r="AEI24" s="5"/>
+      <c r="AEJ24" s="5"/>
+      <c r="AEK24" s="5"/>
+      <c r="AEL24" s="5"/>
+      <c r="AEM24" s="5"/>
+      <c r="AEN24" s="5"/>
+      <c r="AEO24" s="5"/>
+      <c r="AEP24" s="5"/>
+      <c r="AEQ24" s="5"/>
+      <c r="AER24" s="5"/>
+      <c r="AES24" s="5"/>
+      <c r="AET24" s="5"/>
+      <c r="AEU24" s="5"/>
+      <c r="AEV24" s="5"/>
+      <c r="AEW24" s="5"/>
+      <c r="AEX24" s="5"/>
+      <c r="AEY24" s="5"/>
+      <c r="AEZ24" s="5"/>
+      <c r="AFA24" s="5"/>
+      <c r="AFB24" s="5"/>
+      <c r="AFC24" s="5"/>
+      <c r="AFD24" s="5"/>
+      <c r="AFE24" s="5"/>
+      <c r="AFF24" s="5"/>
+      <c r="AFG24" s="5"/>
+      <c r="AFH24" s="5"/>
+      <c r="AFI24" s="5"/>
+      <c r="AFJ24" s="5"/>
+      <c r="AFK24" s="5"/>
+      <c r="AFL24" s="5"/>
+      <c r="AFM24" s="5"/>
+      <c r="AFN24" s="5"/>
+      <c r="AFO24" s="5"/>
+      <c r="AFP24" s="5"/>
+      <c r="AFQ24" s="5"/>
+      <c r="AFR24" s="5"/>
+      <c r="AFS24" s="5"/>
+      <c r="AFT24" s="5"/>
+      <c r="AFU24" s="5"/>
+      <c r="AFV24" s="5"/>
+      <c r="AFW24" s="5"/>
+      <c r="AFX24" s="5"/>
+      <c r="AFY24" s="5"/>
+      <c r="AFZ24" s="5"/>
+      <c r="AGA24" s="5"/>
+      <c r="AGB24" s="5"/>
+      <c r="AGC24" s="5"/>
+      <c r="AGD24" s="5"/>
+      <c r="AGE24" s="5"/>
+      <c r="AGF24" s="5"/>
+      <c r="AGG24" s="5"/>
+      <c r="AGH24" s="5"/>
+      <c r="AGI24" s="5"/>
+      <c r="AGJ24" s="5"/>
+      <c r="AGK24" s="5"/>
+      <c r="AGL24" s="5"/>
+      <c r="AGM24" s="5"/>
+      <c r="AGN24" s="5"/>
+      <c r="AGO24" s="5"/>
+      <c r="AGP24" s="5"/>
+      <c r="AGQ24" s="5"/>
+      <c r="AGR24" s="5"/>
+      <c r="AGS24" s="5"/>
+      <c r="AGT24" s="5"/>
+      <c r="AGU24" s="5"/>
+      <c r="AGV24" s="5"/>
+      <c r="AGW24" s="5"/>
+      <c r="AGX24" s="5"/>
+      <c r="AGY24" s="5"/>
+      <c r="AGZ24" s="5"/>
+      <c r="AHA24" s="5"/>
+      <c r="AHB24" s="5"/>
+      <c r="AHC24" s="5"/>
+      <c r="AHD24" s="5"/>
+      <c r="AHE24" s="5"/>
+      <c r="AHF24" s="5"/>
+      <c r="AHG24" s="5"/>
+      <c r="AHH24" s="5"/>
+      <c r="AHI24" s="5"/>
+      <c r="AHJ24" s="5"/>
+      <c r="AHK24" s="5"/>
+      <c r="AHL24" s="5"/>
+      <c r="AHM24" s="5"/>
+      <c r="AHN24" s="5"/>
+      <c r="AHO24" s="5"/>
+      <c r="AHP24" s="5"/>
+      <c r="AHQ24" s="5"/>
+      <c r="AHR24" s="5"/>
+      <c r="AHS24" s="5"/>
+      <c r="AHT24" s="5"/>
+      <c r="AHU24" s="5"/>
+      <c r="AHV24" s="5"/>
+      <c r="AHW24" s="5"/>
+      <c r="AHX24" s="5"/>
+      <c r="AHY24" s="5"/>
+      <c r="AHZ24" s="5"/>
+      <c r="AIA24" s="5"/>
+      <c r="AIB24" s="5"/>
+      <c r="AIC24" s="5"/>
+      <c r="AID24" s="5"/>
+      <c r="AIE24" s="5"/>
+      <c r="AIF24" s="5"/>
+      <c r="AIG24" s="5"/>
+      <c r="AIH24" s="5"/>
+      <c r="AII24" s="5"/>
+      <c r="AIJ24" s="5"/>
+      <c r="AIK24" s="5"/>
+      <c r="AIL24" s="5"/>
+      <c r="AIM24" s="5"/>
+      <c r="AIN24" s="5"/>
+      <c r="AIO24" s="5"/>
+      <c r="AIP24" s="5"/>
+      <c r="AIQ24" s="5"/>
+      <c r="AIR24" s="5"/>
+      <c r="AIS24" s="5"/>
+      <c r="AIT24" s="5"/>
+      <c r="AIU24" s="5"/>
+      <c r="AIV24" s="5"/>
+      <c r="AIW24" s="5"/>
+      <c r="AIX24" s="5"/>
+      <c r="AIY24" s="5"/>
+      <c r="AIZ24" s="5"/>
+      <c r="AJA24" s="5"/>
+      <c r="AJB24" s="5"/>
+      <c r="AJC24" s="5"/>
+      <c r="AJD24" s="5"/>
+      <c r="AJE24" s="5"/>
+      <c r="AJF24" s="5"/>
+      <c r="AJG24" s="5"/>
+      <c r="AJH24" s="5"/>
+      <c r="AJI24" s="5"/>
+      <c r="AJJ24" s="5"/>
+      <c r="AJK24" s="5"/>
+      <c r="AJL24" s="5"/>
+      <c r="AJM24" s="5"/>
+      <c r="AJN24" s="5"/>
+      <c r="AJO24" s="5"/>
+      <c r="AJP24" s="5"/>
+      <c r="AJQ24" s="5"/>
+      <c r="AJR24" s="5"/>
+      <c r="AJS24" s="5"/>
+      <c r="AJT24" s="5"/>
+      <c r="AJU24" s="5"/>
+      <c r="AJV24" s="5"/>
+      <c r="AJW24" s="5"/>
+      <c r="AJX24" s="5"/>
+      <c r="AJY24" s="5"/>
+      <c r="AJZ24" s="5"/>
+      <c r="AKA24" s="5"/>
+      <c r="AKB24" s="5"/>
+      <c r="AKC24" s="5"/>
+      <c r="AKD24" s="5"/>
+      <c r="AKE24" s="5"/>
+      <c r="AKF24" s="5"/>
+      <c r="AKG24" s="5"/>
+      <c r="AKH24" s="5"/>
+      <c r="AKI24" s="5"/>
+      <c r="AKJ24" s="5"/>
+      <c r="AKK24" s="5"/>
+      <c r="AKL24" s="5"/>
+      <c r="AKM24" s="5"/>
+      <c r="AKN24" s="5"/>
+      <c r="AKO24" s="5"/>
+      <c r="AKP24" s="5"/>
+      <c r="AKQ24" s="5"/>
+      <c r="AKR24" s="5"/>
+      <c r="AKS24" s="5"/>
+      <c r="AKT24" s="5"/>
+      <c r="AKU24" s="5"/>
+      <c r="AKV24" s="5"/>
+      <c r="AKW24" s="5"/>
+      <c r="AKX24" s="5"/>
+      <c r="AKY24" s="5"/>
+      <c r="AKZ24" s="5"/>
+      <c r="ALA24" s="5"/>
+      <c r="ALB24" s="5"/>
+      <c r="ALC24" s="5"/>
+      <c r="ALD24" s="5"/>
+      <c r="ALE24" s="5"/>
+      <c r="ALF24" s="5"/>
+      <c r="ALG24" s="5"/>
+      <c r="ALH24" s="5"/>
+      <c r="ALI24" s="5"/>
+      <c r="ALJ24" s="5"/>
+      <c r="ALK24" s="5"/>
+      <c r="ALL24" s="5"/>
+      <c r="ALM24" s="5"/>
+      <c r="ALN24" s="5"/>
+      <c r="ALO24" s="5"/>
+      <c r="ALP24" s="5"/>
+      <c r="ALQ24" s="5"/>
+      <c r="ALR24" s="5"/>
+      <c r="ALS24" s="5"/>
+      <c r="ALT24" s="5"/>
+      <c r="ALU24" s="5"/>
+      <c r="ALV24" s="5"/>
+      <c r="ALW24" s="5"/>
+      <c r="ALX24" s="5"/>
+      <c r="ALY24" s="5"/>
+      <c r="ALZ24" s="5"/>
+      <c r="AMA24" s="5"/>
+      <c r="AMB24" s="5"/>
+      <c r="AMC24" s="5"/>
+      <c r="AMD24" s="5"/>
+      <c r="AME24" s="5"/>
+      <c r="AMF24" s="5"/>
+      <c r="AMG24" s="5"/>
+      <c r="AMH24" s="5"/>
+      <c r="AMI24" s="5"/>
+      <c r="AMJ24" s="5"/>
+      <c r="AMK24" s="5"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="pKFT46AcXRrznfWpmO12FPPtk8Stkq83/gBYtpLA8HQFC7aZLAdf2WJU+dOj9PZT/L7JPEe68/xM25EHPxktXQ==" saltValue="g+GUymTOlW49z+xbPyQ28w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="aHGd4BS6zp6S67g/QM/z7UWhn6ji0L8rg78+mq771augM8qM/W/5s5Gfgc39DnZsZjWbPtfjR9iijYWx52MjAw==" saltValue="bAIP5qmIB5mva24+ui5YEw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A19:B19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -9131,6 +9221,46 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="2" max="2" width="153.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection password="E50B" sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -9174,7 +9304,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F286"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -9686,7 +9816,7 @@
       <c r="B55" t="s">
         <v>317</v>
       </c>
-      <c r="E55" s="80" t="s">
+      <c r="E55" t="s">
         <v>551</v>
       </c>
     </row>
@@ -10904,6 +11034,46 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03F88BF-42E1-4D49-809C-4FA79F23F636}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="120.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="138" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="80" t="s">
+        <v>559</v>
+      </c>
+      <c r="B1" s="80"/>
+    </row>
+    <row r="2" spans="1:2" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="70" t="s">
+        <v>558</v>
+      </c>
+      <c r="B2" s="70" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="66" x14ac:dyDescent="0.2">
+      <c r="A3" s="68" t="b">
+        <v>0</v>
+      </c>
+      <c r="B3" s="69" t="s">
+        <v>556</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11046,7 +11216,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N1048576"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11071,7 +11241,7 @@
       <c r="A1" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="75" t="s">
+      <c r="B1" s="81" t="s">
         <v>59</v>
       </c>
       <c r="C1" s="30" t="s">
@@ -11084,27 +11254,27 @@
     </row>
     <row r="2" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="20"/>
-      <c r="B2" s="75"/>
-      <c r="C2" s="76" t="s">
+      <c r="B2" s="81"/>
+      <c r="C2" s="82" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="82"/>
+      <c r="M2" s="82"/>
+      <c r="N2" s="82"/>
     </row>
     <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="75"/>
+      <c r="B3" s="81"/>
       <c r="C3" s="20" t="s">
         <v>36</v>
       </c>
@@ -11175,7 +11345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11328,7 +11498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11460,7 +11630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11921,7 +12091,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AT7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -11950,15 +12120,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="83" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="75"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="81"/>
       <c r="D1" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="E1" s="75" t="s">
+      <c r="E1" s="81" t="s">
         <v>59</v>
       </c>
       <c r="F1" s="43" t="s">
@@ -12008,63 +12178,63 @@
     <row r="2" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A2" s="49"/>
       <c r="B2" s="50"/>
-      <c r="C2" s="75"/>
+      <c r="C2" s="81"/>
       <c r="D2" s="51"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="78" t="s">
+      <c r="E2" s="81"/>
+      <c r="F2" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
-      <c r="L2" s="77" t="s">
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="84"/>
+      <c r="L2" s="85" t="s">
         <v>112</v>
       </c>
-      <c r="M2" s="77"/>
-      <c r="N2" s="77"/>
-      <c r="O2" s="77" t="s">
+      <c r="M2" s="85"/>
+      <c r="N2" s="85"/>
+      <c r="O2" s="85" t="s">
         <v>118</v>
       </c>
-      <c r="P2" s="77"/>
-      <c r="Q2" s="77"/>
-      <c r="R2" s="78" t="s">
+      <c r="P2" s="85"/>
+      <c r="Q2" s="85"/>
+      <c r="R2" s="84" t="s">
         <v>125</v>
       </c>
-      <c r="S2" s="78"/>
-      <c r="T2" s="78"/>
-      <c r="U2" s="78"/>
-      <c r="V2" s="78"/>
-      <c r="W2" s="78" t="s">
+      <c r="S2" s="84"/>
+      <c r="T2" s="84"/>
+      <c r="U2" s="84"/>
+      <c r="V2" s="84"/>
+      <c r="W2" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="X2" s="78"/>
-      <c r="Y2" s="78"/>
-      <c r="Z2" s="78" t="s">
+      <c r="X2" s="84"/>
+      <c r="Y2" s="84"/>
+      <c r="Z2" s="84" t="s">
         <v>143</v>
       </c>
-      <c r="AA2" s="78"/>
-      <c r="AB2" s="78"/>
-      <c r="AC2" s="78"/>
-      <c r="AD2" s="78"/>
-      <c r="AE2" s="78"/>
-      <c r="AF2" s="78"/>
-      <c r="AG2" s="78"/>
-      <c r="AH2" s="78"/>
-      <c r="AI2" s="78"/>
-      <c r="AJ2" s="78" t="s">
+      <c r="AA2" s="84"/>
+      <c r="AB2" s="84"/>
+      <c r="AC2" s="84"/>
+      <c r="AD2" s="84"/>
+      <c r="AE2" s="84"/>
+      <c r="AF2" s="84"/>
+      <c r="AG2" s="84"/>
+      <c r="AH2" s="84"/>
+      <c r="AI2" s="84"/>
+      <c r="AJ2" s="84" t="s">
         <v>164</v>
       </c>
-      <c r="AK2" s="78"/>
-      <c r="AL2" s="78"/>
-      <c r="AM2" s="78"/>
-      <c r="AN2" s="78"/>
-      <c r="AO2" s="78"/>
-      <c r="AP2" s="78"/>
-      <c r="AQ2" s="78"/>
-      <c r="AR2" s="78"/>
-      <c r="AS2" s="78"/>
+      <c r="AK2" s="84"/>
+      <c r="AL2" s="84"/>
+      <c r="AM2" s="84"/>
+      <c r="AN2" s="84"/>
+      <c r="AO2" s="84"/>
+      <c r="AP2" s="84"/>
+      <c r="AQ2" s="84"/>
+      <c r="AR2" s="84"/>
+      <c r="AS2" s="84"/>
     </row>
     <row r="3" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A3" s="52" t="s">
@@ -12073,11 +12243,11 @@
       <c r="B3" s="53" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="75"/>
+      <c r="C3" s="81"/>
       <c r="D3" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="75"/>
+      <c r="E3" s="81"/>
       <c r="F3" s="54" t="s">
         <v>101</v>
       </c>
@@ -12220,16 +12390,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="R2:V2"/>
+    <mergeCell ref="W2:Y2"/>
+    <mergeCell ref="Z2:AI2"/>
+    <mergeCell ref="AJ2:AS2"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="E1:E3"/>
     <mergeCell ref="F2:K2"/>
     <mergeCell ref="L2:N2"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="R2:V2"/>
-    <mergeCell ref="W2:Y2"/>
-    <mergeCell ref="Z2:AI2"/>
-    <mergeCell ref="AJ2:AS2"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Metadata and VCF" prompt="These sample names must match those provided in the VCF file(s)" sqref="E1 B4:B1003" xr:uid="{00000000-0002-0000-0700-000000000000}">
@@ -12293,44 +12463,4 @@
     </ext>
   </extLst>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="2" max="2" width="153.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="B3" t="s">
-        <v>195</v>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection password="E50B" sheet="1" objects="1" scenarios="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>